<commit_message>
update excel_template.xlsx,ignore database data files
</commit_message>
<xml_diff>
--- a/web-console/server/assets/excel_template.xlsx
+++ b/web-console/server/assets/excel_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ORA\Downloads\UBA_web\or_dev\web-console\server\assets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\DEV\UBA6\web-console\server\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A397D30-26BD-4DAE-BDA6-F8EB98C37555}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A0BE590-A765-4F8F-ACFA-417049B22B4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="1" xr2:uid="{3E3B58E4-0181-4207-8002-E1D914CEBC2E}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3E3B58E4-0181-4207-8002-E1D914CEBC2E}"/>
   </bookViews>
   <sheets>
     <sheet name="Report" sheetId="1" r:id="rId1"/>
@@ -454,6 +454,923 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="2.4483389978238169E-2"/>
+          <c:y val="4.7792374087071994E-2"/>
+          <c:w val="0.94714843493388978"/>
+          <c:h val="0.89839320293349512"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:v>Temprture </c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:srgbClr val="0070C0"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>[0]!Time</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>[0]!Temp</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-D4ED-46DC-869B-EE0C9C2EF0E9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="538752176"/>
+        <c:axId val="538753616"/>
+        <c:extLst>
+          <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+            <c15:filteredScatterSeries>
+              <c15:ser>
+                <c:idx val="0"/>
+                <c:order val="0"/>
+                <c:tx>
+                  <c:v>Voltage</c:v>
+                </c:tx>
+                <c:spPr>
+                  <a:ln w="38100" cap="rnd">
+                    <a:solidFill>
+                      <a:schemeClr val="accent1"/>
+                    </a:solidFill>
+                    <a:round/>
+                  </a:ln>
+                  <a:effectLst/>
+                </c:spPr>
+                <c:marker>
+                  <c:symbol val="none"/>
+                </c:marker>
+                <c:xVal>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Time</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:xVal>
+                <c:yVal>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Voltage</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:yVal>
+                <c:smooth val="0"/>
+                <c:extLst>
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000001-D4ED-46DC-869B-EE0C9C2EF0E9}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredScatterSeries>
+          </c:ext>
+        </c:extLst>
+      </c:scatterChart>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="548909984"/>
+        <c:axId val="572448592"/>
+        <c:extLst>
+          <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+            <c15:filteredScatterSeries>
+              <c15:ser>
+                <c:idx val="1"/>
+                <c:order val="1"/>
+                <c:tx>
+                  <c:v>Current</c:v>
+                </c:tx>
+                <c:spPr>
+                  <a:ln w="38100" cap="rnd">
+                    <a:solidFill>
+                      <a:schemeClr val="accent2"/>
+                    </a:solidFill>
+                    <a:round/>
+                  </a:ln>
+                  <a:effectLst/>
+                </c:spPr>
+                <c:marker>
+                  <c:symbol val="none"/>
+                </c:marker>
+                <c:xVal>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Time</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:xVal>
+                <c:yVal>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Cur</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:yVal>
+                <c:smooth val="0"/>
+                <c:extLst>
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000002-D4ED-46DC-869B-EE0C9C2EF0E9}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredScatterSeries>
+          </c:ext>
+        </c:extLst>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="538752176"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:minorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="5000"/>
+                  <a:lumOff val="95000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:minorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="538753616"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="538753616"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="40"/>
+          <c:min val="10"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="low"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="accent5">
+                    <a:lumMod val="75000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-IL"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="538752176"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+        <c:majorUnit val="3"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="572448592"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="1"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="r"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="high"/>
+        <c:crossAx val="548909984"/>
+        <c:crosses val="max"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="548909984"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="1"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="572448592"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="t"/>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.7998643672420106"/>
+          <c:y val="0.78767517625973249"/>
+          <c:w val="0.10907123241506654"/>
+          <c:h val="5.2467796107256472E-2"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-IL"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:noFill/>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-IL"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="1.8390346032920592E-2"/>
+          <c:y val="3.498752828110973E-2"/>
+          <c:w val="0.92124839634892319"/>
+          <c:h val="0.90635983893333416"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="538752176"/>
+        <c:axId val="538753616"/>
+        <c:extLst>
+          <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+            <c15:filteredScatterSeries>
+              <c15:ser>
+                <c:idx val="0"/>
+                <c:order val="0"/>
+                <c:tx>
+                  <c:v>Voltage</c:v>
+                </c:tx>
+                <c:spPr>
+                  <a:ln w="28575" cap="rnd">
+                    <a:solidFill>
+                      <a:schemeClr val="accent1"/>
+                    </a:solidFill>
+                    <a:round/>
+                  </a:ln>
+                  <a:effectLst/>
+                </c:spPr>
+                <c:marker>
+                  <c:symbol val="none"/>
+                </c:marker>
+                <c:xVal>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Time</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:xVal>
+                <c:yVal>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Voltage</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:yVal>
+                <c:smooth val="0"/>
+                <c:extLst>
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000000-3E5E-4D86-A6D8-00C02409DB60}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredScatterSeries>
+            <c15:filteredScatterSeries>
+              <c15:ser>
+                <c:idx val="2"/>
+                <c:order val="2"/>
+                <c:tx>
+                  <c:v>Temprture </c:v>
+                </c:tx>
+                <c:spPr>
+                  <a:ln w="28575" cap="rnd">
+                    <a:solidFill>
+                      <a:schemeClr val="accent3"/>
+                    </a:solidFill>
+                    <a:round/>
+                  </a:ln>
+                  <a:effectLst/>
+                </c:spPr>
+                <c:marker>
+                  <c:symbol val="none"/>
+                </c:marker>
+                <c:xVal>
+                  <c:numRef>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Time</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:xVal>
+                <c:yVal>
+                  <c:numRef>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Temp</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:yVal>
+                <c:smooth val="0"/>
+                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000001-3E5E-4D86-A6D8-00C02409DB60}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredScatterSeries>
+          </c:ext>
+        </c:extLst>
+      </c:scatterChart>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Current</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>[0]!Time</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>[0]!Cur</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-3E5E-4D86-A6D8-00C02409DB60}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="548909984"/>
+        <c:axId val="572448592"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="538752176"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="1"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="538753616"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="538753616"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:min val="0"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="high"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="bg1"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-IL"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="538752176"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="572448592"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="r"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:srgbClr val="FF0000"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-IL"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="548909984"/>
+        <c:crosses val="max"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="548909984"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="bg1"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-IL"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="572448592"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+        <c:majorUnit val="0.1"/>
+        <c:minorUnit val="1.0000000000000002E-2"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.80566647533210101"/>
+          <c:y val="0.81655369968699099"/>
+          <c:w val="8.0866861773946044E-2"/>
+          <c:h val="5.3625314899907628E-2"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-IL"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:noFill/>
+    <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1"/>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-IL"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
       <c:layout/>
@@ -869,6 +1786,447 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="1.3042762160857644E-2"/>
+          <c:y val="3.9135691333752574E-2"/>
+          <c:w val="0.93216865552763761"/>
+          <c:h val="0.90009773498387535"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Voltage</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:srgbClr val="00B050"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>[0]!Time</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>[0]!Voltage</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-9AAC-4A56-A8F3-EE39410B3FD8}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="538752176"/>
+        <c:axId val="538753616"/>
+        <c:extLst>
+          <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+            <c15:filteredScatterSeries>
+              <c15:ser>
+                <c:idx val="2"/>
+                <c:order val="2"/>
+                <c:tx>
+                  <c:v>Temprture </c:v>
+                </c:tx>
+                <c:spPr>
+                  <a:ln w="28575" cap="rnd">
+                    <a:solidFill>
+                      <a:schemeClr val="accent3"/>
+                    </a:solidFill>
+                    <a:round/>
+                  </a:ln>
+                  <a:effectLst/>
+                </c:spPr>
+                <c:marker>
+                  <c:symbol val="none"/>
+                </c:marker>
+                <c:xVal>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Time</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:xVal>
+                <c:yVal>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Temp</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:yVal>
+                <c:smooth val="0"/>
+                <c:extLst>
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000000-9AAC-4A56-A8F3-EE39410B3FD8}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredScatterSeries>
+          </c:ext>
+        </c:extLst>
+      </c:scatterChart>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="548909984"/>
+        <c:axId val="572448592"/>
+        <c:extLst>
+          <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+            <c15:filteredScatterSeries>
+              <c15:ser>
+                <c:idx val="1"/>
+                <c:order val="1"/>
+                <c:tx>
+                  <c:v>Current</c:v>
+                </c:tx>
+                <c:spPr>
+                  <a:ln w="9525" cap="rnd">
+                    <a:solidFill>
+                      <a:schemeClr val="accent2"/>
+                    </a:solidFill>
+                    <a:round/>
+                  </a:ln>
+                  <a:effectLst/>
+                </c:spPr>
+                <c:marker>
+                  <c:symbol val="none"/>
+                </c:marker>
+                <c:xVal>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Time</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:xVal>
+                <c:yVal>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Cur</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:yVal>
+                <c:smooth val="0"/>
+                <c:extLst>
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000002-9AAC-4A56-A8F3-EE39410B3FD8}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredScatterSeries>
+          </c:ext>
+        </c:extLst>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="538752176"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-IL"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="538753616"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="538753616"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="high"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:solidFill>
+              <a:schemeClr val="tx1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:srgbClr val="00B050"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-IL"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="538752176"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="572448592"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="1"/>
+          <c:min val="0"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="r"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="548909984"/>
+        <c:crosses val="max"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="548909984"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="1"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="572448592"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="19050">
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.82691141849951322"/>
+          <c:y val="0.85637522606985139"/>
+          <c:w val="8.436597058502586E-2"/>
+          <c:h val="5.2249736939881872E-2"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-IL"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:noFill/>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:noFill/>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-IL"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -909,8 +2267,128 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="225">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
@@ -921,7 +2399,7 @@
         <a:lumOff val="35000"/>
       </a:schemeClr>
     </cs:fontRef>
-    <cs:defRPr sz="1000" kern="1200"/>
+    <cs:defRPr sz="900" kern="1200" cap="all"/>
   </cs:axisTitle>
   <cs:categoryAxis>
     <cs:lnRef idx="0"/>
@@ -937,21 +2415,21 @@
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
           <a:schemeClr val="tx1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
       </a:ln>
     </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
+    <cs:defRPr sz="900" b="0" kern="1200" cap="none" spc="0" normalizeH="0" baseline="0"/>
   </cs:categoryAxis>
   <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="dk1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:solidFill>
@@ -967,7 +2445,7 @@
         <a:round/>
       </a:ln>
     </cs:spPr>
-    <cs:defRPr sz="1000" kern="1200"/>
+    <cs:defRPr sz="900" kern="1200"/>
   </cs:chartArea>
   <cs:dataLabel>
     <cs:lnRef idx="0"/>
@@ -987,22 +2465,17 @@
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
       <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:spPr>
       <a:solidFill>
-        <a:schemeClr val="lt1"/>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
       </a:solidFill>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
     </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
     <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
@@ -1011,6 +2484,511 @@
   </cs:dataLabelCallout>
   <cs:dataPoint>
     <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="38100" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="8"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="major">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="2000" b="0" kern="1200" cap="none" spc="0" normalizeH="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="322">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
     <cs:fillRef idx="1">
       <cs:styleClr val="auto"/>
     </cs:fillRef>
@@ -1039,7 +3017,7 @@
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="19050" cap="rnd">
+      <a:ln w="28575" cap="rnd">
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
@@ -1071,10 +3049,10 @@
     <cs:lnRef idx="0">
       <cs:styleClr val="auto"/>
     </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="9525" cap="rnd">
@@ -1235,8 +3213,8 @@
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
           <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -1300,6 +3278,17 @@
         <a:lumOff val="35000"/>
       </a:schemeClr>
     </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
   </cs:seriesAxis>
   <cs:seriesLine>
@@ -1395,6 +3384,49 @@
         <a:lumOff val="35000"/>
       </a:schemeClr>
     </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
     <cs:spPr>
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
@@ -1406,6 +3438,984 @@
         <a:round/>
       </a:ln>
     </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="322">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
     <cs:defRPr sz="900" kern="1200"/>
   </cs:valueAxis>
   <cs:wall>
@@ -1430,15 +4440,91 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>136072</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>27214</xdr:rowOff>
+      <xdr:colOff>105131</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>179053</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>178224</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>151825</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="7" name="Chart 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{80F85B0E-700A-4724-8B40-68BD122674AB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>78038</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>7327</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>169546</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>20956</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="8" name="Chart 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3F2436C3-92FD-47C1-AC85-E4ADC3EC8563}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>8563</xdr:colOff>
+      <xdr:row>78</xdr:row>
+      <xdr:rowOff>12937</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>612320</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>27214</xdr:rowOff>
+      <xdr:colOff>633254</xdr:colOff>
+      <xdr:row>100</xdr:row>
+      <xdr:rowOff>18651</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1457,7 +4543,45 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>79813</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>26372</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>556126</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>10886</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="6" name="Chart 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A342E69C-40E3-4049-92C5-8B4CFE72E6B5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1483,9 +4607,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1523,7 +4647,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1629,7 +4753,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1771,7 +4895,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1783,23 +4907,23 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B1:O78"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="2"/>
-    <col min="2" max="2" width="2.140625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="2.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="9" width="19.7109375" style="2" customWidth="1"/>
-    <col min="10" max="10" width="9.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="2.140625" style="2" customWidth="1"/>
-    <col min="12" max="12" width="9.140625" style="18"/>
-    <col min="13" max="13" width="82.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="123.28515625" style="2" customWidth="1"/>
-    <col min="15" max="15" width="78.85546875" style="2" customWidth="1"/>
-    <col min="16" max="16384" width="9.140625" style="2"/>
+    <col min="1" max="1" width="7.44140625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="2.109375" style="2" customWidth="1"/>
+    <col min="3" max="3" width="2.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="9" width="19.6640625" style="2" customWidth="1"/>
+    <col min="10" max="10" width="9.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="4.109375" style="2" customWidth="1"/>
+    <col min="12" max="12" width="9.109375" style="18"/>
+    <col min="13" max="13" width="82.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="123.33203125" style="2" customWidth="1"/>
+    <col min="15" max="15" width="78.88671875" style="2" customWidth="1"/>
+    <col min="16" max="16384" width="9.109375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:14" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="2:14" ht="8.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="3"/>
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
@@ -1811,7 +4935,7 @@
       <c r="J2" s="4"/>
       <c r="K2" s="5"/>
     </row>
-    <row r="3" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B3" s="6"/>
       <c r="D3" s="7" t="s">
         <v>19</v>
@@ -1829,7 +4953,7 @@
       <c r="K3" s="9"/>
       <c r="N3" s="10"/>
     </row>
-    <row r="4" spans="2:14" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:14" ht="5.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="6"/>
       <c r="C4" s="11"/>
       <c r="D4" s="11"/>
@@ -1842,7 +4966,7 @@
       <c r="K4" s="9"/>
       <c r="N4" s="10"/>
     </row>
-    <row r="5" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B5" s="12"/>
       <c r="C5" s="24"/>
       <c r="D5" s="24"/>
@@ -1854,7 +4978,7 @@
       <c r="J5" s="24"/>
       <c r="K5" s="13"/>
     </row>
-    <row r="6" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B6" s="12"/>
       <c r="C6" s="24"/>
       <c r="D6" s="24"/>
@@ -1866,7 +4990,7 @@
       <c r="J6" s="24"/>
       <c r="K6" s="13"/>
     </row>
-    <row r="7" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B7" s="12"/>
       <c r="C7" s="24"/>
       <c r="D7" s="24"/>
@@ -1878,7 +5002,7 @@
       <c r="J7" s="24"/>
       <c r="K7" s="13"/>
     </row>
-    <row r="8" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B8" s="12"/>
       <c r="C8" s="24"/>
       <c r="D8" s="24"/>
@@ -1890,7 +5014,7 @@
       <c r="J8" s="24"/>
       <c r="K8" s="13"/>
     </row>
-    <row r="9" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B9" s="12"/>
       <c r="C9" s="24"/>
       <c r="D9" s="24"/>
@@ -1902,7 +5026,7 @@
       <c r="J9" s="24"/>
       <c r="K9" s="13"/>
     </row>
-    <row r="10" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B10" s="12"/>
       <c r="C10" s="24"/>
       <c r="D10" s="24"/>
@@ -1914,7 +5038,7 @@
       <c r="J10" s="24"/>
       <c r="K10" s="13"/>
     </row>
-    <row r="11" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B11" s="12"/>
       <c r="C11" s="24"/>
       <c r="D11" s="24"/>
@@ -1926,7 +5050,7 @@
       <c r="J11" s="24"/>
       <c r="K11" s="13"/>
     </row>
-    <row r="12" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B12" s="12"/>
       <c r="C12" s="24"/>
       <c r="D12" s="24"/>
@@ -1938,7 +5062,7 @@
       <c r="J12" s="24"/>
       <c r="K12" s="13"/>
     </row>
-    <row r="13" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B13" s="12"/>
       <c r="C13" s="24"/>
       <c r="D13" s="24"/>
@@ -1950,7 +5074,7 @@
       <c r="J13" s="24"/>
       <c r="K13" s="13"/>
     </row>
-    <row r="14" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B14" s="12"/>
       <c r="C14" s="24"/>
       <c r="D14" s="24"/>
@@ -1962,7 +5086,7 @@
       <c r="J14" s="24"/>
       <c r="K14" s="13"/>
     </row>
-    <row r="15" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B15" s="12"/>
       <c r="C15" s="24"/>
       <c r="D15" s="24"/>
@@ -1974,7 +5098,7 @@
       <c r="J15" s="24"/>
       <c r="K15" s="13"/>
     </row>
-    <row r="16" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B16" s="12"/>
       <c r="C16" s="24"/>
       <c r="D16" s="24"/>
@@ -1986,7 +5110,7 @@
       <c r="J16" s="24"/>
       <c r="K16" s="13"/>
     </row>
-    <row r="17" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B17" s="12"/>
       <c r="C17" s="24"/>
       <c r="D17" s="24"/>
@@ -1998,7 +5122,7 @@
       <c r="J17" s="24"/>
       <c r="K17" s="13"/>
     </row>
-    <row r="18" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B18" s="12"/>
       <c r="C18" s="24"/>
       <c r="D18" s="24"/>
@@ -2010,7 +5134,7 @@
       <c r="J18" s="24"/>
       <c r="K18" s="13"/>
     </row>
-    <row r="19" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B19" s="12"/>
       <c r="C19" s="24"/>
       <c r="D19" s="24"/>
@@ -2022,7 +5146,7 @@
       <c r="J19" s="24"/>
       <c r="K19" s="13"/>
     </row>
-    <row r="20" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B20" s="12"/>
       <c r="C20" s="24"/>
       <c r="D20" s="24"/>
@@ -2034,7 +5158,7 @@
       <c r="J20" s="24"/>
       <c r="K20" s="13"/>
     </row>
-    <row r="21" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B21" s="12"/>
       <c r="C21" s="24"/>
       <c r="D21" s="24"/>
@@ -2046,7 +5170,7 @@
       <c r="J21" s="24"/>
       <c r="K21" s="13"/>
     </row>
-    <row r="22" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B22" s="12"/>
       <c r="C22" s="24"/>
       <c r="D22" s="24"/>
@@ -2058,7 +5182,7 @@
       <c r="J22" s="24"/>
       <c r="K22" s="13"/>
     </row>
-    <row r="23" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B23" s="12"/>
       <c r="C23" s="24"/>
       <c r="D23" s="24"/>
@@ -2070,7 +5194,7 @@
       <c r="J23" s="24"/>
       <c r="K23" s="13"/>
     </row>
-    <row r="24" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B24" s="12"/>
       <c r="C24" s="24"/>
       <c r="D24" s="24"/>
@@ -2082,7 +5206,7 @@
       <c r="J24" s="24"/>
       <c r="K24" s="13"/>
     </row>
-    <row r="25" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B25" s="12"/>
       <c r="C25" s="24"/>
       <c r="D25" s="24"/>
@@ -2094,7 +5218,7 @@
       <c r="J25" s="24"/>
       <c r="K25" s="13"/>
     </row>
-    <row r="26" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B26" s="12"/>
       <c r="C26" s="24"/>
       <c r="D26" s="24"/>
@@ -2107,11 +5231,11 @@
       <c r="K26" s="13"/>
       <c r="M26" s="14"/>
     </row>
-    <row r="27" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B27" s="12"/>
       <c r="K27" s="13"/>
     </row>
-    <row r="28" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B28" s="6"/>
       <c r="D28" s="8" t="s">
         <v>18</v>
@@ -2128,7 +5252,7 @@
       <c r="L28" s="23"/>
       <c r="M28" s="15"/>
     </row>
-    <row r="29" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B29" s="12"/>
       <c r="D29" s="2" t="s">
         <v>16</v>
@@ -2141,7 +5265,7 @@
       <c r="L29" s="23"/>
       <c r="M29" s="16"/>
     </row>
-    <row r="30" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B30" s="12"/>
       <c r="H30" s="2" t="s">
         <v>23</v>
@@ -2153,7 +5277,7 @@
       <c r="N30" s="17"/>
       <c r="O30" s="17"/>
     </row>
-    <row r="31" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B31" s="12"/>
       <c r="D31" s="2" t="s">
         <v>15</v>
@@ -2168,7 +5292,7 @@
       <c r="N31" s="17"/>
       <c r="O31" s="17"/>
     </row>
-    <row r="32" spans="2:15" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:15" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B32" s="6"/>
       <c r="D32" s="2" t="s">
         <v>13</v>
@@ -2189,7 +5313,7 @@
       <c r="N32" s="17"/>
       <c r="O32" s="17"/>
     </row>
-    <row r="33" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B33" s="12"/>
       <c r="H33" s="2" t="s">
         <v>25</v>
@@ -2204,7 +5328,7 @@
       <c r="N33" s="17"/>
       <c r="O33" s="17"/>
     </row>
-    <row r="34" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B34" s="12"/>
       <c r="H34" s="2" t="s">
         <v>10</v>
@@ -2219,7 +5343,7 @@
       <c r="N34" s="17"/>
       <c r="O34" s="17"/>
     </row>
-    <row r="35" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B35" s="12"/>
       <c r="H35" s="2" t="s">
         <v>8</v>
@@ -2231,7 +5355,7 @@
       <c r="N35" s="17"/>
       <c r="O35" s="17"/>
     </row>
-    <row r="36" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B36" s="12"/>
       <c r="D36" s="2" t="s">
         <v>9</v>
@@ -2246,7 +5370,7 @@
       <c r="N36" s="17"/>
       <c r="O36" s="17"/>
     </row>
-    <row r="37" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B37" s="12"/>
       <c r="D37" s="2" t="s">
         <v>7</v>
@@ -2261,7 +5385,7 @@
       <c r="N37" s="17"/>
       <c r="O37" s="17"/>
     </row>
-    <row r="38" spans="2:15" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:15" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B38" s="6"/>
       <c r="D38" s="8" t="s">
         <v>4</v>
@@ -2272,7 +5396,7 @@
       <c r="N38" s="17"/>
       <c r="O38" s="17"/>
     </row>
-    <row r="39" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B39" s="12"/>
       <c r="D39" s="27" t="s">
         <v>20</v>
@@ -2289,7 +5413,7 @@
       <c r="N39" s="17"/>
       <c r="O39" s="17"/>
     </row>
-    <row r="40" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B40" s="12"/>
       <c r="K40" s="13"/>
       <c r="L40" s="17"/>
@@ -2297,7 +5421,7 @@
       <c r="N40" s="17"/>
       <c r="O40" s="17"/>
     </row>
-    <row r="41" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B41" s="12"/>
       <c r="C41" s="2">
         <v>1</v>
@@ -2315,7 +5439,7 @@
       <c r="N41" s="17"/>
       <c r="O41" s="17"/>
     </row>
-    <row r="42" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B42" s="12"/>
       <c r="K42" s="13"/>
       <c r="L42" s="17"/>
@@ -2323,7 +5447,7 @@
       <c r="N42" s="17"/>
       <c r="O42" s="17"/>
     </row>
-    <row r="43" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B43" s="12"/>
       <c r="K43" s="13"/>
       <c r="L43" s="17"/>
@@ -2331,7 +5455,7 @@
       <c r="N43" s="17"/>
       <c r="O43" s="17"/>
     </row>
-    <row r="44" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B44" s="12"/>
       <c r="K44" s="13"/>
       <c r="L44" s="17"/>
@@ -2339,7 +5463,7 @@
       <c r="N44" s="17"/>
       <c r="O44" s="17"/>
     </row>
-    <row r="45" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B45" s="12"/>
       <c r="K45" s="13"/>
       <c r="L45" s="17"/>
@@ -2347,7 +5471,7 @@
       <c r="N45" s="17"/>
       <c r="O45" s="17"/>
     </row>
-    <row r="46" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B46" s="12"/>
       <c r="K46" s="13"/>
       <c r="L46" s="17"/>
@@ -2355,7 +5479,7 @@
       <c r="N46" s="17"/>
       <c r="O46" s="17"/>
     </row>
-    <row r="47" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B47" s="12"/>
       <c r="K47" s="13"/>
       <c r="L47" s="17"/>
@@ -2363,7 +5487,7 @@
       <c r="N47" s="17"/>
       <c r="O47" s="17"/>
     </row>
-    <row r="48" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B48" s="12"/>
       <c r="K48" s="13"/>
       <c r="L48" s="17"/>
@@ -2371,7 +5495,7 @@
       <c r="N48" s="17"/>
       <c r="O48" s="17"/>
     </row>
-    <row r="49" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B49" s="12"/>
       <c r="K49" s="13"/>
       <c r="L49" s="17"/>
@@ -2379,7 +5503,7 @@
       <c r="N49" s="17"/>
       <c r="O49" s="17"/>
     </row>
-    <row r="50" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B50" s="12"/>
       <c r="K50" s="13"/>
       <c r="L50" s="17"/>
@@ -2387,7 +5511,7 @@
       <c r="N50" s="17"/>
       <c r="O50" s="17"/>
     </row>
-    <row r="51" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B51" s="12"/>
       <c r="K51" s="13"/>
       <c r="L51" s="17"/>
@@ -2395,7 +5519,7 @@
       <c r="N51" s="17"/>
       <c r="O51" s="17"/>
     </row>
-    <row r="52" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B52" s="12"/>
       <c r="K52" s="13"/>
       <c r="L52" s="17"/>
@@ -2403,7 +5527,7 @@
       <c r="N52" s="17"/>
       <c r="O52" s="17"/>
     </row>
-    <row r="53" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B53" s="12"/>
       <c r="K53" s="13"/>
       <c r="L53" s="17"/>
@@ -2411,7 +5535,7 @@
       <c r="N53" s="17"/>
       <c r="O53" s="17"/>
     </row>
-    <row r="54" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B54" s="12"/>
       <c r="K54" s="13"/>
       <c r="L54" s="17"/>
@@ -2419,7 +5543,7 @@
       <c r="N54" s="17"/>
       <c r="O54" s="17"/>
     </row>
-    <row r="55" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B55" s="12"/>
       <c r="K55" s="13"/>
       <c r="L55" s="17"/>
@@ -2427,7 +5551,7 @@
       <c r="N55" s="17"/>
       <c r="O55" s="17"/>
     </row>
-    <row r="56" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B56" s="12"/>
       <c r="K56" s="13"/>
       <c r="L56" s="17"/>
@@ -2435,7 +5559,7 @@
       <c r="N56" s="17"/>
       <c r="O56" s="17"/>
     </row>
-    <row r="57" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B57" s="12"/>
       <c r="K57" s="13"/>
       <c r="L57" s="17"/>
@@ -2443,7 +5567,7 @@
       <c r="N57" s="17"/>
       <c r="O57" s="17"/>
     </row>
-    <row r="58" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B58" s="12"/>
       <c r="K58" s="13"/>
       <c r="L58" s="17"/>
@@ -2451,7 +5575,7 @@
       <c r="N58" s="17"/>
       <c r="O58" s="17"/>
     </row>
-    <row r="59" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B59" s="12"/>
       <c r="K59" s="13"/>
       <c r="L59" s="17"/>
@@ -2459,7 +5583,7 @@
       <c r="N59" s="17"/>
       <c r="O59" s="17"/>
     </row>
-    <row r="60" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B60" s="12"/>
       <c r="K60" s="13"/>
       <c r="L60" s="17"/>
@@ -2467,7 +5591,7 @@
       <c r="N60" s="17"/>
       <c r="O60" s="17"/>
     </row>
-    <row r="61" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B61" s="12"/>
       <c r="K61" s="13"/>
       <c r="L61" s="17"/>
@@ -2475,7 +5599,7 @@
       <c r="N61" s="17"/>
       <c r="O61" s="17"/>
     </row>
-    <row r="62" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B62" s="12"/>
       <c r="K62" s="13"/>
       <c r="L62" s="17"/>
@@ -2483,7 +5607,7 @@
       <c r="N62" s="17"/>
       <c r="O62" s="17"/>
     </row>
-    <row r="63" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B63" s="12"/>
       <c r="K63" s="13"/>
       <c r="L63" s="17"/>
@@ -2491,7 +5615,7 @@
       <c r="N63" s="17"/>
       <c r="O63" s="17"/>
     </row>
-    <row r="64" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B64" s="12"/>
       <c r="K64" s="13"/>
       <c r="L64" s="17"/>
@@ -2499,7 +5623,7 @@
       <c r="N64" s="17"/>
       <c r="O64" s="17"/>
     </row>
-    <row r="65" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B65" s="12"/>
       <c r="K65" s="13"/>
       <c r="L65" s="17"/>
@@ -2507,7 +5631,7 @@
       <c r="N65" s="17"/>
       <c r="O65" s="17"/>
     </row>
-    <row r="66" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B66" s="12"/>
       <c r="K66" s="13"/>
       <c r="L66" s="17"/>
@@ -2515,7 +5639,7 @@
       <c r="N66" s="17"/>
       <c r="O66" s="17"/>
     </row>
-    <row r="67" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B67" s="12"/>
       <c r="K67" s="13"/>
       <c r="L67" s="17"/>
@@ -2523,7 +5647,7 @@
       <c r="N67" s="17"/>
       <c r="O67" s="17"/>
     </row>
-    <row r="68" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B68" s="12"/>
       <c r="K68" s="13"/>
       <c r="L68" s="17"/>
@@ -2531,7 +5655,7 @@
       <c r="N68" s="17"/>
       <c r="O68" s="17"/>
     </row>
-    <row r="69" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B69" s="12"/>
       <c r="K69" s="13"/>
       <c r="L69" s="17"/>
@@ -2539,7 +5663,7 @@
       <c r="N69" s="17"/>
       <c r="O69" s="17"/>
     </row>
-    <row r="70" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B70" s="12"/>
       <c r="K70" s="13"/>
       <c r="L70" s="17"/>
@@ -2547,7 +5671,7 @@
       <c r="N70" s="17"/>
       <c r="O70" s="17"/>
     </row>
-    <row r="71" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B71" s="12"/>
       <c r="K71" s="13"/>
       <c r="L71" s="17"/>
@@ -2555,7 +5679,7 @@
       <c r="N71" s="17"/>
       <c r="O71" s="17"/>
     </row>
-    <row r="72" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B72" s="12"/>
       <c r="K72" s="13"/>
       <c r="L72" s="17"/>
@@ -2563,7 +5687,7 @@
       <c r="N72" s="17"/>
       <c r="O72" s="17"/>
     </row>
-    <row r="73" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B73" s="12"/>
       <c r="K73" s="13"/>
       <c r="L73" s="17"/>
@@ -2571,7 +5695,7 @@
       <c r="N73" s="17"/>
       <c r="O73" s="17"/>
     </row>
-    <row r="74" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="74" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B74" s="12"/>
       <c r="K74" s="13"/>
       <c r="L74" s="17"/>
@@ -2579,7 +5703,7 @@
       <c r="N74" s="17"/>
       <c r="O74" s="17"/>
     </row>
-    <row r="75" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="75" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B75" s="12"/>
       <c r="K75" s="13"/>
       <c r="L75" s="17"/>
@@ -2587,7 +5711,7 @@
       <c r="N75" s="17"/>
       <c r="O75" s="17"/>
     </row>
-    <row r="76" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="76" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B76" s="12"/>
       <c r="K76" s="13"/>
       <c r="L76" s="17"/>
@@ -2595,7 +5719,7 @@
       <c r="N76" s="17"/>
       <c r="O76" s="17"/>
     </row>
-    <row r="77" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B77" s="19"/>
       <c r="C77" s="20"/>
       <c r="D77" s="20"/>
@@ -2609,7 +5733,7 @@
       <c r="L77" s="23"/>
       <c r="M77" s="22"/>
     </row>
-    <row r="78" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="78" spans="2:15" x14ac:dyDescent="0.3">
       <c r="H78" s="8"/>
       <c r="I78" s="8"/>
       <c r="J78" s="8"/>
@@ -2627,18 +5751,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BE78AA8-3E87-47A3-991D-56AC1DEC39E3}">
   <dimension ref="A1:K19"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.85546875" style="1" customWidth="1"/>
-    <col min="2" max="3" width="16.42578125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="15.85546875" style="1" customWidth="1"/>
-    <col min="5" max="5" width="22.5703125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="13.140625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="13.28515625" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="18.88671875" style="1" customWidth="1"/>
+    <col min="2" max="3" width="16.44140625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="15.88671875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="22.5546875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="13.109375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="13.33203125" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="26" t="s">
         <v>27</v>
       </c>
@@ -2661,7 +5785,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>0</v>
       </c>
@@ -2684,7 +5808,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="11:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K19" s="2"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
dowload reports - fix start time (local), results in db (local instead of UTC)
</commit_message>
<xml_diff>
--- a/web-console/server/assets/excel_template.xlsx
+++ b/web-console/server/assets/excel_template.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr defaultThemeVersion="166925"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\DEV\UBA6\web-console\server\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A0BE590-A765-4F8F-ACFA-417049B22B4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5033F18F-FF5E-48AD-96C7-D27BE9A8C527}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3E3B58E4-0181-4207-8002-E1D914CEBC2E}"/>
   </bookViews>
@@ -429,6 +429,14 @@
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFCC0000"/>
+      <color rgb="FF009999"/>
+      <color rgb="FF0066FF"/>
+      <color rgb="FF009900"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -441,923 +449,6 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
-  <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="2"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
-  <c:chart>
-    <c:autoTitleDeleted val="1"/>
-    <c:plotArea>
-      <c:layout>
-        <c:manualLayout>
-          <c:layoutTarget val="inner"/>
-          <c:xMode val="edge"/>
-          <c:yMode val="edge"/>
-          <c:x val="2.4483389978238169E-2"/>
-          <c:y val="4.7792374087071994E-2"/>
-          <c:w val="0.94714843493388978"/>
-          <c:h val="0.89839320293349512"/>
-        </c:manualLayout>
-      </c:layout>
-      <c:scatterChart>
-        <c:scatterStyle val="lineMarker"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="2"/>
-          <c:order val="2"/>
-          <c:tx>
-            <c:v>Temprture </c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:srgbClr val="0070C0"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>[0]!Time</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>[0]!Temp</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-D4ED-46DC-869B-EE0C9C2EF0E9}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:axId val="538752176"/>
-        <c:axId val="538753616"/>
-        <c:extLst>
-          <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-            <c15:filteredScatterSeries>
-              <c15:ser>
-                <c:idx val="0"/>
-                <c:order val="0"/>
-                <c:tx>
-                  <c:v>Voltage</c:v>
-                </c:tx>
-                <c:spPr>
-                  <a:ln w="38100" cap="rnd">
-                    <a:solidFill>
-                      <a:schemeClr val="accent1"/>
-                    </a:solidFill>
-                    <a:round/>
-                  </a:ln>
-                  <a:effectLst/>
-                </c:spPr>
-                <c:marker>
-                  <c:symbol val="none"/>
-                </c:marker>
-                <c:xVal>
-                  <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Time</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:xVal>
-                <c:yVal>
-                  <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Voltage</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:yVal>
-                <c:smooth val="0"/>
-                <c:extLst>
-                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                    <c16:uniqueId val="{00000001-D4ED-46DC-869B-EE0C9C2EF0E9}"/>
-                  </c:ext>
-                </c:extLst>
-              </c15:ser>
-            </c15:filteredScatterSeries>
-          </c:ext>
-        </c:extLst>
-      </c:scatterChart>
-      <c:scatterChart>
-        <c:scatterStyle val="lineMarker"/>
-        <c:varyColors val="0"/>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:axId val="548909984"/>
-        <c:axId val="572448592"/>
-        <c:extLst>
-          <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-            <c15:filteredScatterSeries>
-              <c15:ser>
-                <c:idx val="1"/>
-                <c:order val="1"/>
-                <c:tx>
-                  <c:v>Current</c:v>
-                </c:tx>
-                <c:spPr>
-                  <a:ln w="38100" cap="rnd">
-                    <a:solidFill>
-                      <a:schemeClr val="accent2"/>
-                    </a:solidFill>
-                    <a:round/>
-                  </a:ln>
-                  <a:effectLst/>
-                </c:spPr>
-                <c:marker>
-                  <c:symbol val="none"/>
-                </c:marker>
-                <c:xVal>
-                  <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Time</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:xVal>
-                <c:yVal>
-                  <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Cur</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:yVal>
-                <c:smooth val="0"/>
-                <c:extLst>
-                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                    <c16:uniqueId val="{00000002-D4ED-46DC-869B-EE0C9C2EF0E9}"/>
-                  </c:ext>
-                </c:extLst>
-              </c15:ser>
-            </c15:filteredScatterSeries>
-          </c:ext>
-        </c:extLst>
-      </c:scatterChart>
-      <c:valAx>
-        <c:axId val="538752176"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="1"/>
-        <c:axPos val="b"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:minorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="5000"/>
-                  <a:lumOff val="95000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:minorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="538753616"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:valAx>
-        <c:axId val="538753616"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-          <c:max val="40"/>
-          <c:min val="10"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="low"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="accent5">
-                    <a:lumMod val="75000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-IL"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="538752176"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-        <c:majorUnit val="3"/>
-      </c:valAx>
-      <c:valAx>
-        <c:axId val="572448592"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-          <c:max val="1"/>
-        </c:scaling>
-        <c:delete val="1"/>
-        <c:axPos val="r"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="high"/>
-        <c:crossAx val="548909984"/>
-        <c:crosses val="max"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:valAx>
-        <c:axId val="548909984"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-          <c:max val="1"/>
-        </c:scaling>
-        <c:delete val="1"/>
-        <c:axPos val="b"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="572448592"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-    </c:plotArea>
-    <c:legend>
-      <c:legendPos val="t"/>
-      <c:layout>
-        <c:manualLayout>
-          <c:xMode val="edge"/>
-          <c:yMode val="edge"/>
-          <c:x val="0.7998643672420106"/>
-          <c:y val="0.78767517625973249"/>
-          <c:w val="0.10907123241506654"/>
-          <c:h val="5.2467796107256472E-2"/>
-        </c:manualLayout>
-      </c:layout>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-IL"/>
-        </a:p>
-      </c:txPr>
-    </c:legend>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
-    <c:extLst>
-      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
-        <c16r3:dataDisplayOptions16>
-          <c16r3:dispNaAsBlank val="1"/>
-        </c16r3:dataDisplayOptions16>
-      </c:ext>
-    </c:extLst>
-  </c:chart>
-  <c:spPr>
-    <a:solidFill>
-      <a:schemeClr val="bg1"/>
-    </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:noFill/>
-      <a:round/>
-    </a:ln>
-    <a:effectLst/>
-  </c:spPr>
-  <c:txPr>
-    <a:bodyPr/>
-    <a:lstStyle/>
-    <a:p>
-      <a:pPr>
-        <a:defRPr/>
-      </a:pPr>
-      <a:endParaRPr lang="en-IL"/>
-    </a:p>
-  </c:txPr>
-  <c:printSettings>
-    <c:headerFooter/>
-    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
-    <c:pageSetup/>
-  </c:printSettings>
-</c:chartSpace>
-</file>
-
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
-  <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="2"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
-  <c:chart>
-    <c:autoTitleDeleted val="1"/>
-    <c:plotArea>
-      <c:layout>
-        <c:manualLayout>
-          <c:layoutTarget val="inner"/>
-          <c:xMode val="edge"/>
-          <c:yMode val="edge"/>
-          <c:x val="1.8390346032920592E-2"/>
-          <c:y val="3.498752828110973E-2"/>
-          <c:w val="0.92124839634892319"/>
-          <c:h val="0.90635983893333416"/>
-        </c:manualLayout>
-      </c:layout>
-      <c:scatterChart>
-        <c:scatterStyle val="lineMarker"/>
-        <c:varyColors val="0"/>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:axId val="538752176"/>
-        <c:axId val="538753616"/>
-        <c:extLst>
-          <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-            <c15:filteredScatterSeries>
-              <c15:ser>
-                <c:idx val="0"/>
-                <c:order val="0"/>
-                <c:tx>
-                  <c:v>Voltage</c:v>
-                </c:tx>
-                <c:spPr>
-                  <a:ln w="28575" cap="rnd">
-                    <a:solidFill>
-                      <a:schemeClr val="accent1"/>
-                    </a:solidFill>
-                    <a:round/>
-                  </a:ln>
-                  <a:effectLst/>
-                </c:spPr>
-                <c:marker>
-                  <c:symbol val="none"/>
-                </c:marker>
-                <c:xVal>
-                  <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Time</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:xVal>
-                <c:yVal>
-                  <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Voltage</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:yVal>
-                <c:smooth val="0"/>
-                <c:extLst>
-                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                    <c16:uniqueId val="{00000000-3E5E-4D86-A6D8-00C02409DB60}"/>
-                  </c:ext>
-                </c:extLst>
-              </c15:ser>
-            </c15:filteredScatterSeries>
-            <c15:filteredScatterSeries>
-              <c15:ser>
-                <c:idx val="2"/>
-                <c:order val="2"/>
-                <c:tx>
-                  <c:v>Temprture </c:v>
-                </c:tx>
-                <c:spPr>
-                  <a:ln w="28575" cap="rnd">
-                    <a:solidFill>
-                      <a:schemeClr val="accent3"/>
-                    </a:solidFill>
-                    <a:round/>
-                  </a:ln>
-                  <a:effectLst/>
-                </c:spPr>
-                <c:marker>
-                  <c:symbol val="none"/>
-                </c:marker>
-                <c:xVal>
-                  <c:numRef>
-                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Time</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:xVal>
-                <c:yVal>
-                  <c:numRef>
-                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Temp</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:yVal>
-                <c:smooth val="0"/>
-                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                    <c16:uniqueId val="{00000001-3E5E-4D86-A6D8-00C02409DB60}"/>
-                  </c:ext>
-                </c:extLst>
-              </c15:ser>
-            </c15:filteredScatterSeries>
-          </c:ext>
-        </c:extLst>
-      </c:scatterChart>
-      <c:scatterChart>
-        <c:scatterStyle val="lineMarker"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
-          <c:tx>
-            <c:v>Current</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:srgbClr val="FF0000"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>[0]!Time</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>[0]!Cur</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-3E5E-4D86-A6D8-00C02409DB60}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:axId val="548909984"/>
-        <c:axId val="572448592"/>
-      </c:scatterChart>
-      <c:valAx>
-        <c:axId val="538752176"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-          <c:max val="1"/>
-        </c:scaling>
-        <c:delete val="1"/>
-        <c:axPos val="b"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="538753616"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:valAx>
-        <c:axId val="538753616"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-          <c:min val="0"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="high"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="bg1"/>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-IL"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="538752176"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:valAx>
-        <c:axId val="572448592"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="r"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:srgbClr val="FF0000"/>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-IL"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="548909984"/>
-        <c:crosses val="max"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:valAx>
-        <c:axId val="548909984"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="bg1"/>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-IL"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="572448592"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-        <c:majorUnit val="0.1"/>
-        <c:minorUnit val="1.0000000000000002E-2"/>
-      </c:valAx>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-    </c:plotArea>
-    <c:legend>
-      <c:legendPos val="r"/>
-      <c:layout>
-        <c:manualLayout>
-          <c:xMode val="edge"/>
-          <c:yMode val="edge"/>
-          <c:x val="0.80566647533210101"/>
-          <c:y val="0.81655369968699099"/>
-          <c:w val="8.0866861773946044E-2"/>
-          <c:h val="5.3625314899907628E-2"/>
-        </c:manualLayout>
-      </c:layout>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-IL"/>
-        </a:p>
-      </c:txPr>
-    </c:legend>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
-    <c:extLst>
-      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
-        <c16r3:dataDisplayOptions16>
-          <c16r3:dispNaAsBlank val="1"/>
-        </c16r3:dataDisplayOptions16>
-      </c:ext>
-    </c:extLst>
-  </c:chart>
-  <c:spPr>
-    <a:noFill/>
-    <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
-      <a:solidFill>
-        <a:schemeClr val="tx1"/>
-      </a:solidFill>
-      <a:round/>
-    </a:ln>
-    <a:effectLst/>
-  </c:spPr>
-  <c:txPr>
-    <a:bodyPr/>
-    <a:lstStyle/>
-    <a:p>
-      <a:pPr>
-        <a:defRPr/>
-      </a:pPr>
-      <a:endParaRPr lang="en-IL"/>
-    </a:p>
-  </c:txPr>
-  <c:printSettings>
-    <c:headerFooter/>
-    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
-    <c:pageSetup/>
-  </c:printSettings>
-</c:chartSpace>
-</file>
-
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -1786,6 +877,917 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="2.4483389978238169E-2"/>
+          <c:y val="4.7792374087071994E-2"/>
+          <c:w val="0.94714843493388978"/>
+          <c:h val="0.89839320293349512"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:v>Temprture [°C]</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="12700" cap="rnd">
+              <a:solidFill>
+                <a:srgbClr val="CC0000"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>[0]!Time</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>[0]!Temp</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-D4ED-46DC-869B-EE0C9C2EF0E9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="538752176"/>
+        <c:axId val="538753616"/>
+        <c:extLst>
+          <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+            <c15:filteredScatterSeries>
+              <c15:ser>
+                <c:idx val="0"/>
+                <c:order val="0"/>
+                <c:tx>
+                  <c:v>Voltage [V]</c:v>
+                </c:tx>
+                <c:spPr>
+                  <a:ln w="38100" cap="rnd">
+                    <a:solidFill>
+                      <a:schemeClr val="accent1"/>
+                    </a:solidFill>
+                    <a:round/>
+                  </a:ln>
+                  <a:effectLst/>
+                </c:spPr>
+                <c:marker>
+                  <c:symbol val="none"/>
+                </c:marker>
+                <c:xVal>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Time</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:xVal>
+                <c:yVal>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Voltage</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:yVal>
+                <c:smooth val="0"/>
+                <c:extLst>
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000001-D4ED-46DC-869B-EE0C9C2EF0E9}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredScatterSeries>
+          </c:ext>
+        </c:extLst>
+      </c:scatterChart>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="548909984"/>
+        <c:axId val="572448592"/>
+        <c:extLst>
+          <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+            <c15:filteredScatterSeries>
+              <c15:ser>
+                <c:idx val="1"/>
+                <c:order val="1"/>
+                <c:tx>
+                  <c:v>Current [mA]</c:v>
+                </c:tx>
+                <c:spPr>
+                  <a:ln w="38100" cap="rnd">
+                    <a:solidFill>
+                      <a:schemeClr val="accent2"/>
+                    </a:solidFill>
+                    <a:round/>
+                  </a:ln>
+                  <a:effectLst/>
+                </c:spPr>
+                <c:marker>
+                  <c:symbol val="none"/>
+                </c:marker>
+                <c:xVal>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Time</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:xVal>
+                <c:yVal>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Cur</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:yVal>
+                <c:smooth val="0"/>
+                <c:extLst>
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000002-D4ED-46DC-869B-EE0C9C2EF0E9}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredScatterSeries>
+          </c:ext>
+        </c:extLst>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="538752176"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:minorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="5000"/>
+                  <a:lumOff val="95000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:minorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="538753616"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="538753616"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="40"/>
+          <c:min val="10"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="low"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:srgbClr val="C00000"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-IL"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="538752176"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+        <c:majorUnit val="3"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="572448592"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="1"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="r"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="high"/>
+        <c:crossAx val="548909984"/>
+        <c:crosses val="max"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="548909984"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="1"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="572448592"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.81801116030075538"/>
+          <c:y val="0.89087012680713484"/>
+          <c:w val="0.1187560047174363"/>
+          <c:h val="5.2573014805340469E-2"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="CC0000"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-IL"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:noFill/>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-IL"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="2.9449730317721565E-2"/>
+          <c:y val="3.4988307114440113E-2"/>
+          <c:w val="0.9115746029438424"/>
+          <c:h val="0.90635983893333416"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="538752176"/>
+        <c:axId val="538753616"/>
+        <c:extLst>
+          <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+            <c15:filteredScatterSeries>
+              <c15:ser>
+                <c:idx val="0"/>
+                <c:order val="0"/>
+                <c:tx>
+                  <c:v>Voltage</c:v>
+                </c:tx>
+                <c:spPr>
+                  <a:ln w="28575" cap="rnd">
+                    <a:solidFill>
+                      <a:schemeClr val="accent1"/>
+                    </a:solidFill>
+                    <a:round/>
+                  </a:ln>
+                  <a:effectLst/>
+                </c:spPr>
+                <c:marker>
+                  <c:symbol val="none"/>
+                </c:marker>
+                <c:xVal>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Time</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:xVal>
+                <c:yVal>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Voltage</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:yVal>
+                <c:smooth val="0"/>
+                <c:extLst>
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000001-27BB-4E04-B76C-393CC8BFB84A}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredScatterSeries>
+            <c15:filteredScatterSeries>
+              <c15:ser>
+                <c:idx val="2"/>
+                <c:order val="2"/>
+                <c:tx>
+                  <c:v>Temprture </c:v>
+                </c:tx>
+                <c:spPr>
+                  <a:ln w="28575" cap="rnd">
+                    <a:solidFill>
+                      <a:schemeClr val="accent3"/>
+                    </a:solidFill>
+                    <a:round/>
+                  </a:ln>
+                  <a:effectLst/>
+                </c:spPr>
+                <c:marker>
+                  <c:symbol val="none"/>
+                </c:marker>
+                <c:xVal>
+                  <c:numRef>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Time</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:xVal>
+                <c:yVal>
+                  <c:numRef>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Temp</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:yVal>
+                <c:smooth val="0"/>
+                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000002-27BB-4E04-B76C-393CC8BFB84A}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredScatterSeries>
+          </c:ext>
+        </c:extLst>
+      </c:scatterChart>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Current [mA]</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="12700" cap="rnd">
+              <a:solidFill>
+                <a:srgbClr val="0070C0"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>[0]!Time</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>[0]!Cur</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-27BB-4E04-B76C-393CC8BFB84A}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="548909984"/>
+        <c:axId val="572448592"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="538752176"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="1"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="538753616"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="538753616"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:min val="0"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="high"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="bg1"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-IL"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="538752176"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="572448592"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="r"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:srgbClr val="1134E5"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-IL"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="548909984"/>
+        <c:crosses val="max"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="548909984"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="low"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="bg1"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-IL"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="572448592"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+        <c:majorUnit val="0.1"/>
+        <c:minorUnit val="1.0000000000000002E-2"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst>
+          <a:softEdge rad="0"/>
+        </a:effectLst>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.81026726999333876"/>
+          <c:y val="0.80315839279030921"/>
+          <c:w val="0.10803954187413875"/>
+          <c:h val="5.2905920262186892E-2"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="3366FF"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-IL"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:noFill/>
+    <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-IL"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
@@ -1808,9 +1810,9 @@
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
           <c:x val="1.3042762160857644E-2"/>
-          <c:y val="3.9135691333752574E-2"/>
-          <c:w val="0.93216865552763761"/>
-          <c:h val="0.90009773498387535"/>
+          <c:y val="4.8651119114099188E-2"/>
+          <c:w val="0.94670208851992088"/>
+          <c:h val="0.89058230895640922"/>
         </c:manualLayout>
       </c:layout>
       <c:scatterChart>
@@ -1820,10 +1822,10 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:v>Voltage</c:v>
+            <c:v>Voltage [V]</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln w="19050" cap="rnd">
+            <a:ln w="12700" cap="rnd">
               <a:solidFill>
                 <a:srgbClr val="00B050"/>
               </a:solidFill>
@@ -2069,6 +2071,7 @@
         <c:axId val="538753616"/>
         <c:scaling>
           <c:orientation val="minMax"/>
+          <c:min val="3"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
@@ -2141,24 +2144,46 @@
       </c:valAx>
       <c:spPr>
         <a:noFill/>
-        <a:ln w="19050">
+        <a:ln w="12700">
           <a:solidFill>
             <a:sysClr val="windowText" lastClr="000000"/>
           </a:solidFill>
         </a:ln>
-        <a:effectLst/>
+        <a:effectLst>
+          <a:softEdge rad="1270000"/>
+        </a:effectLst>
       </c:spPr>
     </c:plotArea>
     <c:legend>
       <c:legendPos val="r"/>
+      <c:legendEntry>
+        <c:idx val="0"/>
+        <c:txPr>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:srgbClr val="008000"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-IL"/>
+          </a:p>
+        </c:txPr>
+      </c:legendEntry>
       <c:layout>
         <c:manualLayout>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.82691141849951322"/>
-          <c:y val="0.85637522606985139"/>
-          <c:w val="8.436597058502586E-2"/>
-          <c:h val="5.2249736939881872E-2"/>
+          <c:x val="0.83692512917620809"/>
+          <c:y val="0.84840430666972655"/>
+          <c:w val="0.10284715188479832"/>
+          <c:h val="5.2306152832353021E-2"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="0"/>
@@ -2388,7 +2413,7 @@
 </file>
 
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="225">
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
@@ -2399,7 +2424,7 @@
         <a:lumOff val="35000"/>
       </a:schemeClr>
     </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200" cap="all"/>
+    <cs:defRPr sz="1000" kern="1200"/>
   </cs:axisTitle>
   <cs:categoryAxis>
     <cs:lnRef idx="0"/>
@@ -2415,21 +2440,21 @@
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
           <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
       </a:ln>
     </cs:spPr>
-    <cs:defRPr sz="900" b="0" kern="1200" cap="none" spc="0" normalizeH="0" baseline="0"/>
+    <cs:defRPr sz="900" kern="1200"/>
   </cs:categoryAxis>
   <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:solidFill>
@@ -2445,7 +2470,7 @@
         <a:round/>
       </a:ln>
     </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
+    <cs:defRPr sz="1000" kern="1200"/>
   </cs:chartArea>
   <cs:dataLabel>
     <cs:lnRef idx="0"/>
@@ -2465,17 +2490,22 @@
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
       <a:schemeClr val="dk1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:spPr>
       <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
+        <a:schemeClr val="lt1"/>
       </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
     </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
     <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
@@ -2484,511 +2514,6 @@
   </cs:dataLabelCallout>
   <cs:dataPoint>
     <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="phClr"/>
-      </a:solidFill>
-    </cs:spPr>
-  </cs:dataPoint>
-  <cs:dataPoint3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="phClr"/>
-      </a:solidFill>
-    </cs:spPr>
-  </cs:dataPoint3D>
-  <cs:dataPointLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="38100" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointLine>
-  <cs:dataPointMarker>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="phClr"/>
-      </a:solidFill>
-    </cs:spPr>
-  </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="8"/>
-  <cs:dataPointWireframe>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointWireframe>
-  <cs:dataTable>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataTable>
-  <cs:downBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="75000"/>
-          <a:lumOff val="25000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:downBar>
-  <cs:dropLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:prstDash val="dash"/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dropLine>
-  <cs:errorBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:errorBar>
-  <cs:floor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-  </cs:floor>
-  <cs:gridlineMajor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMajor>
-  <cs:gridlineMinor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="5000"/>
-            <a:lumOff val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:prstDash val="dash"/>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:legend>
-  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-  </cs:plotArea>
-  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:seriesLine>
-  <cs:title>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="major">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="2000" b="0" kern="1200" cap="none" spc="0" normalizeH="0" baseline="0"/>
-  </cs:title>
-  <cs:trendline>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:trendline>
-  <cs:trendlineLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:trendlineLabel>
-  <cs:upBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:upBar>
-  <cs:valueAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:valueAxis>
-  <cs:wall>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-  </cs:wall>
-</cs:chartStyle>
-</file>
-
-<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="322">
-  <cs:axisTitle>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:axisTitle>
-  <cs:categoryAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:categoryAxis>
-  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="bg1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:chartArea>
-  <cs:dataLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataLabel>
-  <cs:dataLabelCallout>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
-      <a:spAutoFit/>
-    </cs:bodyPr>
-  </cs:dataLabelCallout>
-  <cs:dataPoint>
-    <cs:lnRef idx="0"/>
     <cs:fillRef idx="1">
       <cs:styleClr val="auto"/>
     </cs:fillRef>
@@ -3017,7 +2542,7 @@
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="28575" cap="rnd">
+      <a:ln w="19050" cap="rnd">
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
@@ -3049,10 +2574,10 @@
     <cs:lnRef idx="0">
       <cs:styleClr val="auto"/>
     </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="9525" cap="rnd">
@@ -3213,8 +2738,8 @@
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
           <a:schemeClr val="tx1">
-            <a:lumMod val="75000"/>
-            <a:lumOff val="25000"/>
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -3278,17 +2803,6 @@
         <a:lumOff val="35000"/>
       </a:schemeClr>
     </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
   </cs:seriesAxis>
   <cs:seriesLine>
@@ -3384,6 +2898,17 @@
         <a:lumOff val="35000"/>
       </a:schemeClr>
     </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
   </cs:valueAxis>
   <cs:wall>
@@ -3403,8 +2928,8 @@
 </cs:chartStyle>
 </file>
 
-<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="225">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
@@ -3415,7 +2940,7 @@
         <a:lumOff val="35000"/>
       </a:schemeClr>
     </cs:fontRef>
-    <cs:defRPr sz="1000" kern="1200"/>
+    <cs:defRPr sz="900" kern="1200" cap="all"/>
   </cs:axisTitle>
   <cs:categoryAxis>
     <cs:lnRef idx="0"/>
@@ -3431,21 +2956,21 @@
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
           <a:schemeClr val="tx1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
       </a:ln>
     </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
+    <cs:defRPr sz="900" b="0" kern="1200" cap="none" spc="0" normalizeH="0" baseline="0"/>
   </cs:categoryAxis>
   <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="dk1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:solidFill>
@@ -3461,7 +2986,7 @@
         <a:round/>
       </a:ln>
     </cs:spPr>
-    <cs:defRPr sz="1000" kern="1200"/>
+    <cs:defRPr sz="900" kern="1200"/>
   </cs:chartArea>
   <cs:dataLabel>
     <cs:lnRef idx="0"/>
@@ -3481,22 +3006,17 @@
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
       <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:spPr>
       <a:solidFill>
-        <a:schemeClr val="lt1"/>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
       </a:solidFill>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
     </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
     <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
@@ -3505,6 +3025,511 @@
   </cs:dataLabelCallout>
   <cs:dataPoint>
     <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="38100" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="8"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="major">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="2000" b="0" kern="1200" cap="none" spc="0" normalizeH="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="322">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
     <cs:fillRef idx="1">
       <cs:styleClr val="auto"/>
     </cs:fillRef>
@@ -3533,7 +3558,7 @@
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="19050" cap="rnd">
+      <a:ln w="28575" cap="rnd">
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
@@ -3565,10 +3590,10 @@
     <cs:lnRef idx="0">
       <cs:styleClr val="auto"/>
     </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="9525" cap="rnd">
@@ -3729,8 +3754,8 @@
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
           <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -3794,6 +3819,17 @@
         <a:lumOff val="35000"/>
       </a:schemeClr>
     </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
   </cs:seriesAxis>
   <cs:seriesLine>
@@ -3889,17 +3925,6 @@
         <a:lumOff val="35000"/>
       </a:schemeClr>
     </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
   </cs:valueAxis>
   <cs:wall>
@@ -4437,82 +4462,6 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>105131</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>179053</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>178224</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>151825</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="7" name="Chart 6">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{80F85B0E-700A-4724-8B40-68BD122674AB}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr>
-          <a:graphicFrameLocks/>
-        </xdr:cNvGraphicFramePr>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>78038</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>7327</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>169546</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>20956</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="8" name="Chart 7">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3F2436C3-92FD-47C1-AC85-E4ADC3EC8563}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr>
-          <a:graphicFrameLocks/>
-        </xdr:cNvGraphicFramePr>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>2</xdr:col>
@@ -4543,7 +4492,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -4551,40 +4500,126 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>79813</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>26372</xdr:rowOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>97167</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>7781</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>556126</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>10886</xdr:rowOff>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>1722839</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>162711</xdr:rowOff>
     </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="6" name="Chart 5">
+    <xdr:grpSp>
+      <xdr:nvGrpSpPr>
+        <xdr:cNvPr id="4" name="Group 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A342E69C-40E3-4049-92C5-8B4CFE72E6B5}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{866F844E-F3BE-594D-7AB0-3062BC36413A}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr>
-          <a:graphicFrameLocks/>
-        </xdr:cNvGraphicFramePr>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
+        <xdr:cNvGrpSpPr/>
+      </xdr:nvGrpSpPr>
+      <xdr:grpSpPr>
+        <a:xfrm>
+          <a:off x="607707" y="533561"/>
+          <a:ext cx="11594537" cy="6308080"/>
+          <a:chOff x="658053" y="598165"/>
+          <a:chExt cx="11594119" cy="6392357"/>
+        </a:xfrm>
+      </xdr:grpSpPr>
+      <xdr:graphicFrame macro="">
+        <xdr:nvGraphicFramePr>
+          <xdr:cNvPr id="7" name="Chart 6">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{80F85B0E-700A-4724-8B40-68BD122674AB}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvGraphicFramePr>
+            <a:graphicFrameLocks/>
+          </xdr:cNvGraphicFramePr>
+        </xdr:nvGraphicFramePr>
+        <xdr:xfrm>
+          <a:off x="1601799" y="1962648"/>
+          <a:ext cx="9057462" cy="4074613"/>
+        </xdr:xfrm>
+        <a:graphic>
+          <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+            <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          </a:graphicData>
+        </a:graphic>
+      </xdr:graphicFrame>
+      <xdr:grpSp>
+        <xdr:nvGrpSpPr>
+          <xdr:cNvPr id="2" name="Group 1">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9619185F-13F1-B981-85AF-A15E2E36AA7E}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvGrpSpPr/>
+        </xdr:nvGrpSpPr>
+        <xdr:grpSpPr>
+          <a:xfrm>
+            <a:off x="658053" y="598165"/>
+            <a:ext cx="11594119" cy="6392357"/>
+            <a:chOff x="658053" y="601929"/>
+            <a:chExt cx="11594119" cy="6386434"/>
+          </a:xfrm>
+        </xdr:grpSpPr>
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="3" name="Chart 2">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{04634C5F-9538-4DAD-82D1-B1CF33C71DB0}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr>
+              <a:graphicFrameLocks/>
+            </xdr:cNvGraphicFramePr>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="658053" y="601929"/>
+            <a:ext cx="9169604" cy="4045222"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+              <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="6" name="Chart 5">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A342E69C-40E3-4049-92C5-8B4CFE72E6B5}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr>
+              <a:graphicFrameLocks/>
+            </xdr:cNvGraphicFramePr>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="3532300" y="2896756"/>
+            <a:ext cx="8719872" cy="4091607"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+              <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </xdr:grpSp>
+    </xdr:grpSp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -4609,7 +4644,7 @@
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Red">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -4617,34 +4652,34 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546A"/>
+        <a:srgbClr val="323232"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
+        <a:srgbClr val="E5C243"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="A5300F"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ED7D31"/>
+        <a:srgbClr val="D55816"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A5A5A5"/>
+        <a:srgbClr val="E19825"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="FFC000"/>
+        <a:srgbClr val="B19C7D"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="7F5F52"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70AD47"/>
+        <a:srgbClr val="B27D49"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563C1"/>
+        <a:srgbClr val="6B9F25"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954F72"/>
+        <a:srgbClr val="B26B02"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">

</xml_diff>

<commit_message>
download xlsx/pdf reports, display live report - relative time [sec]
</commit_message>
<xml_diff>
--- a/web-console/server/assets/excel_template.xlsx
+++ b/web-console/server/assets/excel_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\DEV\UBA6\web-console\server\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5033F18F-FF5E-48AD-96C7-D27BE9A8C527}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15B1A060-BCEB-4196-BBBB-47CFEADD345D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3E3B58E4-0181-4207-8002-E1D914CEBC2E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{3E3B58E4-0181-4207-8002-E1D914CEBC2E}"/>
   </bookViews>
   <sheets>
     <sheet name="Report" sheetId="1" r:id="rId1"/>
@@ -359,7 +359,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
@@ -399,6 +399,7 @@
     </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="3" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -431,9 +432,10 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FF000000"/>
+      <color rgb="FF0066FF"/>
       <color rgb="FFCC0000"/>
       <color rgb="FF009999"/>
-      <color rgb="FF0066FF"/>
       <color rgb="FF009900"/>
     </mruColors>
   </colors>
@@ -462,435 +464,6 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:chart>
-    <c:autoTitleDeleted val="0"/>
-    <c:plotArea>
-      <c:layout/>
-      <c:scatterChart>
-        <c:scatterStyle val="lineMarker"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:tx>
-            <c:v>Voltage</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent1"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>[0]!Time</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>[0]!Voltage</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-E875-4C8B-836C-C00ED46E82DB}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="2"/>
-          <c:order val="2"/>
-          <c:tx>
-            <c:v>Temprture </c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent3"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>[0]!Time</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>[0]!Temp</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-E875-4C8B-836C-C00ED46E82DB}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:axId val="538752176"/>
-        <c:axId val="538753616"/>
-      </c:scatterChart>
-      <c:scatterChart>
-        <c:scatterStyle val="lineMarker"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
-          <c:tx>
-            <c:v>Current</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent2"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>[0]!Time</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>[0]!Cur</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-E875-4C8B-836C-C00ED46E82DB}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:axId val="548909984"/>
-        <c:axId val="572448592"/>
-      </c:scatterChart>
-      <c:valAx>
-        <c:axId val="538752176"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="25000"/>
-                <a:lumOff val="75000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-IL"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="538753616"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:valAx>
-        <c:axId val="538753616"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-          <c:min val="20"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="25000"/>
-                <a:lumOff val="75000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-IL"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="538752176"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:valAx>
-        <c:axId val="572448592"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="r"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="out"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="25000"/>
-                <a:lumOff val="75000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-IL"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="548909984"/>
-        <c:crosses val="max"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:valAx>
-        <c:axId val="548909984"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="1"/>
-        <c:axPos val="b"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="out"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="572448592"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-    </c:plotArea>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
-    <c:extLst>
-      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
-        <c16r3:dataDisplayOptions16>
-          <c16r3:dispNaAsBlank val="1"/>
-        </c16r3:dataDisplayOptions16>
-      </c:ext>
-    </c:extLst>
-  </c:chart>
-  <c:spPr>
-    <a:solidFill>
-      <a:schemeClr val="bg1"/>
-    </a:solidFill>
-    <a:ln w="31750" cap="flat" cmpd="sng" algn="ctr">
-      <a:solidFill>
-        <a:schemeClr val="tx1"/>
-      </a:solidFill>
-      <a:round/>
-    </a:ln>
-    <a:effectLst/>
-  </c:spPr>
-  <c:txPr>
-    <a:bodyPr/>
-    <a:lstStyle/>
-    <a:p>
-      <a:pPr>
-        <a:defRPr/>
-      </a:pPr>
-      <a:endParaRPr lang="en-IL"/>
-    </a:p>
-  </c:txPr>
-  <c:printSettings>
-    <c:headerFooter/>
-    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
-    <c:pageSetup/>
-  </c:printSettings>
-</c:chartSpace>
-</file>
-
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
-  <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="2"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
-  <c:chart>
     <c:autoTitleDeleted val="1"/>
     <c:plotArea>
       <c:layout>
@@ -900,8 +473,8 @@
           <c:yMode val="edge"/>
           <c:x val="2.4483389978238169E-2"/>
           <c:y val="4.7792374087071994E-2"/>
-          <c:w val="0.94714843493388978"/>
-          <c:h val="0.89839320293349512"/>
+          <c:w val="0.91768132307048078"/>
+          <c:h val="0.8952059492518637"/>
         </c:manualLayout>
       </c:layout>
       <c:scatterChart>
@@ -927,10 +500,10 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>[0]!Time</c:f>
+              <c:f>Data!$A$2:$A$500</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
+                <c:ptCount val="499"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -939,10 +512,10 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>[0]!Temp</c:f>
+              <c:f>Data!$E$2:$E$500</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
+                <c:ptCount val="499"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -1260,10 +833,10 @@
         <c:manualLayout>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.81801116030075538"/>
-          <c:y val="0.89087012680713484"/>
-          <c:w val="0.1187560047174363"/>
-          <c:h val="5.2573014805340469E-2"/>
+          <c:x val="0.8259853931802642"/>
+          <c:y val="0.88814860455055555"/>
+          <c:w val="0.11904422240503133"/>
+          <c:h val="5.4274502653401564E-2"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="0"/>
@@ -1281,7 +854,7 @@
           <a:pPr>
             <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
-                <a:srgbClr val="CC0000"/>
+                <a:srgbClr val="C00000"/>
               </a:solidFill>
               <a:latin typeface="+mn-lt"/>
               <a:ea typeface="+mn-ea"/>
@@ -1331,7 +904,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -1352,10 +925,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="2.9449730317721565E-2"/>
-          <c:y val="3.4988307114440113E-2"/>
-          <c:w val="0.9115746029438424"/>
-          <c:h val="0.90635983893333416"/>
+          <c:x val="3.8413754861339688E-2"/>
+          <c:y val="3.1809769929148149E-2"/>
+          <c:w val="0.88619754950669771"/>
+          <c:h val="0.88484152408937922"/>
         </c:manualLayout>
       </c:layout>
       <c:scatterChart>
@@ -1525,10 +1098,10 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>[0]!Time</c:f>
+              <c:f>Data!$A$2:$A$500</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
+                <c:ptCount val="499"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -1537,10 +1110,10 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>[0]!Cur</c:f>
+              <c:f>Data!$D$2:$D$500</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
+                <c:ptCount val="499"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -1569,14 +1142,40 @@
         <c:axId val="538752176"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:max val="1"/>
         </c:scaling>
-        <c:delete val="1"/>
+        <c:delete val="0"/>
         <c:axPos val="b"/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
+        <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
+        <c:tickLblPos val="none"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-IL"/>
+          </a:p>
+        </c:txPr>
         <c:crossAx val="538753616"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
@@ -1585,12 +1184,11 @@
         <c:axId val="538753616"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:min val="0"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
+        <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="high"/>
         <c:spPr>
@@ -1629,7 +1227,7 @@
         <c:delete val="0"/>
         <c:axPos val="r"/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
+        <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
@@ -1666,9 +1264,9 @@
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
-        <c:axPos val="b"/>
+        <c:axPos val="t"/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
+        <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="low"/>
         <c:spPr>
@@ -1696,19 +1294,17 @@
           </a:p>
         </c:txPr>
         <c:crossAx val="572448592"/>
-        <c:crosses val="autoZero"/>
+        <c:crosses val="max"/>
         <c:crossBetween val="midCat"/>
-        <c:majorUnit val="0.1"/>
-        <c:minorUnit val="1.0000000000000002E-2"/>
       </c:valAx>
       <c:spPr>
         <a:noFill/>
-        <a:ln cmpd="sng">
-          <a:noFill/>
+        <a:ln>
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
         </a:ln>
-        <a:effectLst>
-          <a:softEdge rad="0"/>
-        </a:effectLst>
+        <a:effectLst/>
       </c:spPr>
     </c:plotArea>
     <c:legend>
@@ -1717,10 +1313,10 @@
         <c:manualLayout>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.81026726999333876"/>
-          <c:y val="0.80315839279030921"/>
-          <c:w val="0.10803954187413875"/>
-          <c:h val="5.2905920262186892E-2"/>
+          <c:x val="0.81091573854013277"/>
+          <c:y val="0.7965441225698342"/>
+          <c:w val="0.10600533583115072"/>
+          <c:h val="5.361499841016773E-2"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="0"/>
@@ -1738,7 +1334,7 @@
           <a:pPr>
             <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
-                <a:srgbClr val="3366FF"/>
+                <a:srgbClr val="0070C0"/>
               </a:solidFill>
               <a:latin typeface="+mn-lt"/>
               <a:ea typeface="+mn-ea"/>
@@ -1788,7 +1384,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -1809,17 +1405,17 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="1.3042762160857644E-2"/>
-          <c:y val="4.8651119114099188E-2"/>
-          <c:w val="0.94670208851992088"/>
-          <c:h val="0.89058230895640922"/>
+          <c:x val="1.3154584557626622E-2"/>
+          <c:y val="1.7806536670153209E-2"/>
+          <c:w val="0.92413817547012744"/>
+          <c:h val="0.89161032223878844"/>
         </c:manualLayout>
       </c:layout>
       <c:scatterChart>
         <c:scatterStyle val="lineMarker"/>
         <c:varyColors val="0"/>
         <c:ser>
-          <c:idx val="0"/>
+          <c:idx val="3"/>
           <c:order val="0"/>
           <c:tx>
             <c:v>Voltage [V]</c:v>
@@ -1838,34 +1434,32 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>[0]!Time</c:f>
+              <c:f>Data!$A$2:$A$500</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
+                <c:ptCount val="499"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
-              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>[0]!Voltage</c:f>
+              <c:f>Data!$C$2:$C$500</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
+                <c:ptCount val="499"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
-              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-9AAC-4A56-A8F3-EE39410B3FD8}"/>
+              <c16:uniqueId val="{00000006-AD78-4094-AE9E-5F088A45CD90}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1883,15 +1477,15 @@
           <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
             <c15:filteredScatterSeries>
               <c15:ser>
-                <c:idx val="2"/>
-                <c:order val="2"/>
+                <c:idx val="4"/>
+                <c:order val="1"/>
                 <c:tx>
                   <c:v>Temprture </c:v>
                 </c:tx>
                 <c:spPr>
                   <a:ln w="28575" cap="rnd">
                     <a:solidFill>
-                      <a:schemeClr val="accent3"/>
+                      <a:schemeClr val="accent5"/>
                     </a:solidFill>
                     <a:round/>
                   </a:ln>
@@ -1939,40 +1533,22 @@
                 <c:smooth val="0"/>
                 <c:extLst>
                   <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                    <c16:uniqueId val="{00000000-9AAC-4A56-A8F3-EE39410B3FD8}"/>
+                    <c16:uniqueId val="{00000007-AD78-4094-AE9E-5F088A45CD90}"/>
                   </c:ext>
                 </c:extLst>
               </c15:ser>
             </c15:filteredScatterSeries>
-          </c:ext>
-        </c:extLst>
-      </c:scatterChart>
-      <c:scatterChart>
-        <c:scatterStyle val="lineMarker"/>
-        <c:varyColors val="0"/>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:axId val="548909984"/>
-        <c:axId val="572448592"/>
-        <c:extLst>
-          <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
             <c15:filteredScatterSeries>
               <c15:ser>
-                <c:idx val="1"/>
-                <c:order val="1"/>
+                <c:idx val="5"/>
+                <c:order val="2"/>
                 <c:tx>
                   <c:v>Current</c:v>
                 </c:tx>
                 <c:spPr>
                   <a:ln w="9525" cap="rnd">
                     <a:solidFill>
-                      <a:schemeClr val="accent2"/>
+                      <a:schemeClr val="accent6"/>
                     </a:solidFill>
                     <a:round/>
                   </a:ln>
@@ -1983,8 +1559,8 @@
                 </c:marker>
                 <c:xVal>
                   <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:formulaRef>
                           <c15:sqref>[0]!Time</c15:sqref>
                         </c15:formulaRef>
@@ -2001,8 +1577,8 @@
                 </c:xVal>
                 <c:yVal>
                   <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:formulaRef>
                           <c15:sqref>[0]!Cur</c15:sqref>
                         </c15:formulaRef>
@@ -2018,9 +1594,135 @@
                   </c:numRef>
                 </c:yVal>
                 <c:smooth val="0"/>
-                <c:extLst>
+                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
                   <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                    <c16:uniqueId val="{00000002-9AAC-4A56-A8F3-EE39410B3FD8}"/>
+                    <c16:uniqueId val="{00000008-AD78-4094-AE9E-5F088A45CD90}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredScatterSeries>
+            <c15:filteredScatterSeries>
+              <c15:ser>
+                <c:idx val="0"/>
+                <c:order val="3"/>
+                <c:tx>
+                  <c:v>Voltage [V]</c:v>
+                </c:tx>
+                <c:spPr>
+                  <a:ln w="12700" cap="rnd">
+                    <a:solidFill>
+                      <a:srgbClr val="00B050"/>
+                    </a:solidFill>
+                    <a:round/>
+                  </a:ln>
+                  <a:effectLst/>
+                </c:spPr>
+                <c:marker>
+                  <c:symbol val="none"/>
+                </c:marker>
+                <c:xVal>
+                  <c:numRef>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>Data!$A$2:$A$500</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="499"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:xVal>
+                <c:yVal>
+                  <c:numRef>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>Data!$C$2:$C$500</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="499"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:yVal>
+                <c:smooth val="0"/>
+                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000001-AD78-4094-AE9E-5F088A45CD90}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredScatterSeries>
+            <c15:filteredScatterSeries>
+              <c15:ser>
+                <c:idx val="2"/>
+                <c:order val="4"/>
+                <c:tx>
+                  <c:v>Temprture </c:v>
+                </c:tx>
+                <c:spPr>
+                  <a:ln w="28575" cap="rnd">
+                    <a:solidFill>
+                      <a:schemeClr val="accent3"/>
+                    </a:solidFill>
+                    <a:round/>
+                  </a:ln>
+                  <a:effectLst/>
+                </c:spPr>
+                <c:marker>
+                  <c:symbol val="none"/>
+                </c:marker>
+                <c:xVal>
+                  <c:numRef>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Time</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:xVal>
+                <c:yVal>
+                  <c:numRef>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Temp</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:yVal>
+                <c:smooth val="0"/>
+                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000005-AD78-4094-AE9E-5F088A45CD90}"/>
                   </c:ext>
                 </c:extLst>
               </c15:ser>
@@ -2082,9 +1784,7 @@
         <c:spPr>
           <a:noFill/>
           <a:ln>
-            <a:solidFill>
-              <a:schemeClr val="tx1"/>
-            </a:solidFill>
+            <a:noFill/>
           </a:ln>
           <a:effectLst/>
         </c:spPr>
@@ -2109,45 +1809,10 @@
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
-      <c:valAx>
-        <c:axId val="572448592"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-          <c:max val="1"/>
-          <c:min val="0"/>
-        </c:scaling>
-        <c:delete val="1"/>
-        <c:axPos val="r"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="548909984"/>
-        <c:crosses val="max"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:valAx>
-        <c:axId val="548909984"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-          <c:max val="1"/>
-        </c:scaling>
-        <c:delete val="1"/>
-        <c:axPos val="b"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="572448592"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
       <c:spPr>
         <a:noFill/>
         <a:ln w="12700">
-          <a:solidFill>
-            <a:sysClr val="windowText" lastClr="000000"/>
-          </a:solidFill>
+          <a:noFill/>
         </a:ln>
         <a:effectLst>
           <a:softEdge rad="1270000"/>
@@ -2156,34 +1821,14 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="r"/>
-      <c:legendEntry>
-        <c:idx val="0"/>
-        <c:txPr>
-          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:srgbClr val="008000"/>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-IL"/>
-          </a:p>
-        </c:txPr>
-      </c:legendEntry>
       <c:layout>
         <c:manualLayout>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.83692512917620809"/>
-          <c:y val="0.84840430666972655"/>
-          <c:w val="0.10284715188479832"/>
-          <c:h val="5.2306152832353021E-2"/>
+          <c:x val="0.8231257513820065"/>
+          <c:y val="0.81824603170531074"/>
+          <c:w val="0.10014027011991856"/>
+          <c:h val="5.3611631988568942E-2"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="0"/>
@@ -2201,10 +1846,7 @@
           <a:pPr>
             <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
+                <a:srgbClr val="00B050"/>
               </a:solidFill>
               <a:latin typeface="+mn-lt"/>
               <a:ea typeface="+mn-ea"/>
@@ -2218,13 +1860,7 @@
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
-    <c:extLst>
-      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
-        <c16r3:dataDisplayOptions16>
-          <c16r3:dispNaAsBlank val="1"/>
-        </c16r3:dataDisplayOptions16>
-      </c:ext>
-    </c:extLst>
+    <c:extLst/>
   </c:chart>
   <c:spPr>
     <a:noFill/>
@@ -2372,48 +2008,8 @@
 </cs:colorStyle>
 </file>
 
-<file path=xl/charts/colors4.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
-  <a:schemeClr val="accent1"/>
-  <a:schemeClr val="accent2"/>
-  <a:schemeClr val="accent3"/>
-  <a:schemeClr val="accent4"/>
-  <a:schemeClr val="accent5"/>
-  <a:schemeClr val="accent6"/>
-  <cs:variation/>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-    <a:lumOff val="20000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-    <a:lumOff val="40000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-    <a:lumOff val="30000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-    <a:lumOff val="50000"/>
-  </cs:variation>
-</cs:colorStyle>
-</file>
-
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="225">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
@@ -2424,7 +2020,7 @@
         <a:lumOff val="35000"/>
       </a:schemeClr>
     </cs:fontRef>
-    <cs:defRPr sz="1000" kern="1200"/>
+    <cs:defRPr sz="900" kern="1200" cap="all"/>
   </cs:axisTitle>
   <cs:categoryAxis>
     <cs:lnRef idx="0"/>
@@ -2440,21 +2036,21 @@
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
           <a:schemeClr val="tx1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
       </a:ln>
     </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
+    <cs:defRPr sz="900" b="0" kern="1200" cap="none" spc="0" normalizeH="0" baseline="0"/>
   </cs:categoryAxis>
   <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="dk1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:solidFill>
@@ -2470,7 +2066,7 @@
         <a:round/>
       </a:ln>
     </cs:spPr>
-    <cs:defRPr sz="1000" kern="1200"/>
+    <cs:defRPr sz="900" kern="1200"/>
   </cs:chartArea>
   <cs:dataLabel>
     <cs:lnRef idx="0"/>
@@ -2490,22 +2086,17 @@
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
       <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:spPr>
       <a:solidFill>
-        <a:schemeClr val="lt1"/>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
       </a:solidFill>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
     </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
     <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
@@ -2514,6 +2105,511 @@
   </cs:dataLabelCallout>
   <cs:dataPoint>
     <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="38100" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="8"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="major">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="2000" b="0" kern="1200" cap="none" spc="0" normalizeH="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="322">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
     <cs:fillRef idx="1">
       <cs:styleClr val="auto"/>
     </cs:fillRef>
@@ -2542,7 +2638,7 @@
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="19050" cap="rnd">
+      <a:ln w="28575" cap="rnd">
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
@@ -2574,10 +2670,10 @@
     <cs:lnRef idx="0">
       <cs:styleClr val="auto"/>
     </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="9525" cap="rnd">
@@ -2738,8 +2834,8 @@
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
           <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -2803,6 +2899,17 @@
         <a:lumOff val="35000"/>
       </a:schemeClr>
     </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
   </cs:seriesAxis>
   <cs:seriesLine>
@@ -2898,17 +3005,6 @@
         <a:lumOff val="35000"/>
       </a:schemeClr>
     </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
   </cs:valueAxis>
   <cs:wall>
@@ -2924,506 +3020,6 @@
         <a:noFill/>
       </a:ln>
     </cs:spPr>
-  </cs:wall>
-</cs:chartStyle>
-</file>
-
-<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="225">
-  <cs:axisTitle>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200" cap="all"/>
-  </cs:axisTitle>
-  <cs:categoryAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" b="0" kern="1200" cap="none" spc="0" normalizeH="0" baseline="0"/>
-  </cs:categoryAxis>
-  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="bg1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:chartArea>
-  <cs:dataLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataLabel>
-  <cs:dataLabelCallout>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
-      </a:solidFill>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
-      <a:spAutoFit/>
-    </cs:bodyPr>
-  </cs:dataLabelCallout>
-  <cs:dataPoint>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="phClr"/>
-      </a:solidFill>
-    </cs:spPr>
-  </cs:dataPoint>
-  <cs:dataPoint3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="phClr"/>
-      </a:solidFill>
-    </cs:spPr>
-  </cs:dataPoint3D>
-  <cs:dataPointLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="38100" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointLine>
-  <cs:dataPointMarker>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="phClr"/>
-      </a:solidFill>
-    </cs:spPr>
-  </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="8"/>
-  <cs:dataPointWireframe>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointWireframe>
-  <cs:dataTable>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataTable>
-  <cs:downBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="75000"/>
-          <a:lumOff val="25000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:downBar>
-  <cs:dropLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:prstDash val="dash"/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dropLine>
-  <cs:errorBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:errorBar>
-  <cs:floor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-  </cs:floor>
-  <cs:gridlineMajor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMajor>
-  <cs:gridlineMinor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="5000"/>
-            <a:lumOff val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:prstDash val="dash"/>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:legend>
-  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-  </cs:plotArea>
-  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:seriesLine>
-  <cs:title>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="major">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="2000" b="0" kern="1200" cap="none" spc="0" normalizeH="0" baseline="0"/>
-  </cs:title>
-  <cs:trendline>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:trendline>
-  <cs:trendlineLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:trendlineLabel>
-  <cs:upBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:upBar>
-  <cs:valueAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:valueAxis>
-  <cs:wall>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
   </cs:wall>
 </cs:chartStyle>
 </file>
@@ -3944,579 +3540,27 @@
 </cs:chartStyle>
 </file>
 
-<file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="322">
-  <cs:axisTitle>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:axisTitle>
-  <cs:categoryAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:categoryAxis>
-  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="bg1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:chartArea>
-  <cs:dataLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataLabel>
-  <cs:dataLabelCallout>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
-      <a:spAutoFit/>
-    </cs:bodyPr>
-  </cs:dataLabelCallout>
-  <cs:dataPoint>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint>
-  <cs:dataPoint3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint3D>
-  <cs:dataPointLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="28575" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointLine>
-  <cs:dataPointMarker>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
-  <cs:dataPointWireframe>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointWireframe>
-  <cs:dataTable>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataTable>
-  <cs:downBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="75000"/>
-          <a:lumOff val="25000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:downBar>
-  <cs:dropLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dropLine>
-  <cs:errorBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:errorBar>
-  <cs:floor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:floor>
-  <cs:gridlineMajor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMajor>
-  <cs:gridlineMinor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="5000"/>
-            <a:lumOff val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="75000"/>
-            <a:lumOff val="25000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:legend>
-  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea>
-  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:seriesLine>
-  <cs:title>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
-  </cs:title>
-  <cs:trendline>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:prstDash val="sysDot"/>
-      </a:ln>
-    </cs:spPr>
-  </cs:trendline>
-  <cs:trendlineLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:trendlineLabel>
-  <cs:upBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:upBar>
-  <cs:valueAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:valueAxis>
-  <cs:wall>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:wall>
-</cs:chartStyle>
-</file>
-
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>8563</xdr:colOff>
-      <xdr:row>78</xdr:row>
-      <xdr:rowOff>12937</xdr:rowOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>15241</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>28578</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>633254</xdr:colOff>
-      <xdr:row>100</xdr:row>
-      <xdr:rowOff>18651</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="5" name="Chart 4">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C12528C4-E76A-79C2-7F52-3D002A97EFD8}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr/>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>97167</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>7781</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>1722839</xdr:colOff>
-      <xdr:row>38</xdr:row>
-      <xdr:rowOff>162711</xdr:rowOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>259081</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>135392</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
-        <xdr:cNvPr id="4" name="Group 3">
+        <xdr:cNvPr id="2" name="Group 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{866F844E-F3BE-594D-7AB0-3062BC36413A}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F11F62E5-A91C-56A4-A813-ABF1C82C1850}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4524,10 +3568,10 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="607707" y="533561"/>
-          <a:ext cx="11594537" cy="6308080"/>
-          <a:chOff x="658053" y="598165"/>
-          <a:chExt cx="11594119" cy="6392357"/>
+          <a:off x="525781" y="501018"/>
+          <a:ext cx="9273540" cy="4191134"/>
+          <a:chOff x="730729" y="746776"/>
+          <a:chExt cx="9247665" cy="4240098"/>
         </a:xfrm>
       </xdr:grpSpPr>
       <xdr:graphicFrame macro="">
@@ -4544,8 +3588,31 @@
           </xdr:cNvGraphicFramePr>
         </xdr:nvGraphicFramePr>
         <xdr:xfrm>
-          <a:off x="1601799" y="1962648"/>
-          <a:ext cx="9057462" cy="4074613"/>
+          <a:off x="773238" y="746776"/>
+          <a:ext cx="9022790" cy="4071124"/>
+        </xdr:xfrm>
+        <a:graphic>
+          <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+            <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          </a:graphicData>
+        </a:graphic>
+      </xdr:graphicFrame>
+      <xdr:graphicFrame macro="">
+        <xdr:nvGraphicFramePr>
+          <xdr:cNvPr id="3" name="Chart 2">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{04634C5F-9538-4DAD-82D1-B1CF33C71DB0}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvGraphicFramePr>
+            <a:graphicFrameLocks/>
+          </xdr:cNvGraphicFramePr>
+        </xdr:nvGraphicFramePr>
+        <xdr:xfrm>
+          <a:off x="730729" y="806482"/>
+          <a:ext cx="9247665" cy="4121202"/>
         </xdr:xfrm>
         <a:graphic>
           <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -4553,73 +3620,122 @@
           </a:graphicData>
         </a:graphic>
       </xdr:graphicFrame>
-      <xdr:grpSp>
-        <xdr:nvGrpSpPr>
-          <xdr:cNvPr id="2" name="Group 1">
+      <xdr:graphicFrame macro="">
+        <xdr:nvGraphicFramePr>
+          <xdr:cNvPr id="6" name="Chart 5">
             <a:extLst>
               <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9619185F-13F1-B981-85AF-A15E2E36AA7E}"/>
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A342E69C-40E3-4049-92C5-8B4CFE72E6B5}"/>
               </a:ext>
             </a:extLst>
           </xdr:cNvPr>
-          <xdr:cNvGrpSpPr/>
-        </xdr:nvGrpSpPr>
-        <xdr:grpSpPr>
-          <a:xfrm>
-            <a:off x="658053" y="598165"/>
-            <a:ext cx="11594119" cy="6392357"/>
-            <a:chOff x="658053" y="601929"/>
-            <a:chExt cx="11594119" cy="6386434"/>
-          </a:xfrm>
-        </xdr:grpSpPr>
-        <xdr:graphicFrame macro="">
-          <xdr:nvGraphicFramePr>
-            <xdr:cNvPr id="3" name="Chart 2">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{04634C5F-9538-4DAD-82D1-B1CF33C71DB0}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvGraphicFramePr>
-              <a:graphicFrameLocks/>
-            </xdr:cNvGraphicFramePr>
-          </xdr:nvGraphicFramePr>
-          <xdr:xfrm>
-            <a:off x="658053" y="601929"/>
-            <a:ext cx="9169604" cy="4045222"/>
-          </xdr:xfrm>
-          <a:graphic>
-            <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-              <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
-            </a:graphicData>
-          </a:graphic>
-        </xdr:graphicFrame>
-        <xdr:graphicFrame macro="">
-          <xdr:nvGraphicFramePr>
-            <xdr:cNvPr id="6" name="Chart 5">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A342E69C-40E3-4049-92C5-8B4CFE72E6B5}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvGraphicFramePr>
-              <a:graphicFrameLocks/>
-            </xdr:cNvGraphicFramePr>
-          </xdr:nvGraphicFramePr>
-          <xdr:xfrm>
-            <a:off x="3532300" y="2896756"/>
-            <a:ext cx="8719872" cy="4091607"/>
-          </xdr:xfrm>
-          <a:graphic>
-            <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-              <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
-            </a:graphicData>
-          </a:graphic>
-        </xdr:graphicFrame>
-      </xdr:grpSp>
+          <xdr:cNvGraphicFramePr>
+            <a:graphicFrameLocks/>
+          </xdr:cNvGraphicFramePr>
+        </xdr:nvGraphicFramePr>
+        <xdr:xfrm>
+          <a:off x="864424" y="865413"/>
+          <a:ext cx="8942947" cy="4121461"/>
+        </xdr:xfrm>
+        <a:graphic>
+          <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+            <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+          </a:graphicData>
+        </a:graphic>
+      </xdr:graphicFrame>
     </xdr:grpSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>227091</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>163651</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>77602</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>71888</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="5" name="Rectangle 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C63790C8-B105-20F9-DA30-783F73975AAE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9168011" y="4279170"/>
+          <a:ext cx="497492" cy="267671"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="900">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>[</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="900" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Sec</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="900">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>]</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-IL" sz="900">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -5433,15 +4549,15 @@
     </row>
     <row r="39" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B39" s="12"/>
-      <c r="D39" s="27" t="s">
+      <c r="D39" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="E39" s="27"/>
-      <c r="F39" s="27"/>
-      <c r="G39" s="27"/>
-      <c r="H39" s="27"/>
-      <c r="I39" s="27"/>
-      <c r="J39" s="27"/>
+      <c r="E39" s="28"/>
+      <c r="F39" s="28"/>
+      <c r="G39" s="28"/>
+      <c r="H39" s="28"/>
+      <c r="I39" s="28"/>
+      <c r="J39" s="28"/>
       <c r="K39" s="13"/>
       <c r="L39" s="17"/>
       <c r="M39" s="17"/>
@@ -5754,24 +4870,23 @@
       <c r="N76" s="17"/>
       <c r="O76" s="17"/>
     </row>
-    <row r="77" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B77" s="19"/>
-      <c r="C77" s="20"/>
-      <c r="D77" s="20"/>
-      <c r="E77" s="20"/>
-      <c r="F77" s="20"/>
-      <c r="G77" s="20"/>
-      <c r="H77" s="20"/>
-      <c r="I77" s="20"/>
-      <c r="J77" s="20"/>
-      <c r="K77" s="21"/>
+    <row r="77" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="B77" s="12"/>
+      <c r="K77" s="13"/>
       <c r="L77" s="23"/>
       <c r="M77" s="22"/>
     </row>
-    <row r="78" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="H78" s="8"/>
-      <c r="I78" s="8"/>
-      <c r="J78" s="8"/>
+    <row r="78" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B78" s="19"/>
+      <c r="C78" s="20"/>
+      <c r="D78" s="20"/>
+      <c r="E78" s="20"/>
+      <c r="F78" s="20"/>
+      <c r="G78" s="20"/>
+      <c r="H78" s="27"/>
+      <c r="I78" s="27"/>
+      <c r="J78" s="27"/>
+      <c r="K78" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
file chunks transfer UBA --> service, discharge start with voltage=0 (1)
</commit_message>
<xml_diff>
--- a/web-console/server/assets/excel_template.xlsx
+++ b/web-console/server/assets/excel_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\DEV\UBA6\web-console\server\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E260C140-0872-40AA-8021-DCF244DB69E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C29B472E-0BCA-4F6C-80ED-1FA93E16EFA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{3E3B58E4-0181-4207-8002-E1D914CEBC2E}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3E3B58E4-0181-4207-8002-E1D914CEBC2E}"/>
   </bookViews>
   <sheets>
     <sheet name="Report" sheetId="1" r:id="rId1"/>
@@ -2950,6 +2950,7 @@
         <c:axId val="538753616"/>
         <c:scaling>
           <c:orientation val="minMax"/>
+          <c:min val="0"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
@@ -5859,8 +5860,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="407959" y="396023"/>
-          <a:ext cx="9435678" cy="4251259"/>
+          <a:off x="406054" y="385024"/>
+          <a:ext cx="9480823" cy="4253380"/>
           <a:chOff x="582622" y="520820"/>
           <a:chExt cx="9478578" cy="4211876"/>
         </a:xfrm>

</xml_diff>

<commit_message>
improve xlsx template, bpt timer for charge/discharge/pause
</commit_message>
<xml_diff>
--- a/web-console/server/assets/excel_template.xlsx
+++ b/web-console/server/assets/excel_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\DEV\UBA6\web-console\server\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA7B7525-60D7-4E19-B205-A097D3AECF81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{002F57DC-F906-45D9-A8E6-46C7A1E35673}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3E3B58E4-0181-4207-8002-E1D914CEBC2E}"/>
   </bookViews>
@@ -1432,7 +1432,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="700" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -1556,7 +1556,7 @@
             <c:v>Temprture [°C]</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln w="15875" cap="rnd">
+            <a:ln w="12700" cap="rnd">
               <a:solidFill>
                 <a:srgbClr val="C00000"/>
               </a:solidFill>
@@ -1857,8 +1857,8 @@
             <c:manualLayout>
               <c:xMode val="edge"/>
               <c:yMode val="edge"/>
-              <c:x val="0.96215093463589085"/>
-              <c:y val="0.43742411860274616"/>
+              <c:x val="0.9635665803108231"/>
+              <c:y val="0.4374240861470281"/>
             </c:manualLayout>
           </c:layout>
           <c:overlay val="0"/>
@@ -1906,7 +1906,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="700" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:srgbClr val="C00000"/>
                 </a:solidFill>
@@ -2021,7 +2021,7 @@
             <c:v>Voltage [V]</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln w="15875" cap="rnd">
+            <a:ln w="12700" cap="rnd">
               <a:solidFill>
                 <a:schemeClr val="tx1"/>
               </a:solidFill>
@@ -2277,7 +2277,7 @@
             <c:v>Current</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln w="15875" cap="rnd">
+            <a:ln w="12700" cap="rnd">
               <a:solidFill>
                 <a:srgbClr val="0070C0"/>
               </a:solidFill>
@@ -2406,8 +2406,8 @@
             <c:manualLayout>
               <c:xMode val="edge"/>
               <c:yMode val="edge"/>
-              <c:x val="1.9756593874322506E-2"/>
-              <c:y val="0.46379286684399923"/>
+              <c:x val="2.1191562838577517E-2"/>
+              <c:y val="0.45782005072141768"/>
             </c:manualLayout>
           </c:layout>
           <c:overlay val="0"/>
@@ -2455,7 +2455,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="700" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="50000"/>
@@ -2520,8 +2520,8 @@
             <c:manualLayout>
               <c:xMode val="edge"/>
               <c:yMode val="edge"/>
-              <c:x val="0.95537211757740326"/>
-              <c:y val="0.44523003435432329"/>
+              <c:x val="0.95680403458960617"/>
+              <c:y val="0.43909917951215816"/>
             </c:manualLayout>
           </c:layout>
           <c:overlay val="0"/>
@@ -2569,7 +2569,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="700" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:srgbClr val="0070C0"/>
                 </a:solidFill>

</xml_diff>

<commit_message>
xlsx graph - long data, file system - big files, service - concurrent activities (tasks)
</commit_message>
<xml_diff>
--- a/web-console/server/assets/excel_template.xlsx
+++ b/web-console/server/assets/excel_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\DEV\UBA6\web-console\server\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{002F57DC-F906-45D9-A8E6-46C7A1E35673}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EDCC301-41EE-446A-AA7C-09E5E889A90D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3E3B58E4-0181-4207-8002-E1D914CEBC2E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{3E3B58E4-0181-4207-8002-E1D914CEBC2E}"/>
   </bookViews>
   <sheets>
     <sheet name="Report" sheetId="1" r:id="rId1"/>
@@ -504,10 +504,10 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Data!$A$2:$A$500</c:f>
+              <c:f>Data!$A$2:$A$50000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="499"/>
+                <c:ptCount val="49999"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -516,10 +516,10 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Data!$C$2:$C$500</c:f>
+              <c:f>Data!$C$2:$C$50000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="499"/>
+                <c:ptCount val="49999"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -1015,10 +1015,10 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Data!$A$2:$A$500</c:f>
+              <c:f>Data!$A$2:$A$50000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="499"/>
+                <c:ptCount val="49999"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -1027,10 +1027,10 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Data!$H$2:$H$500</c:f>
+              <c:f>Data!$H$2:$H$50000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="499"/>
+                <c:ptCount val="49999"/>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -1569,10 +1569,10 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Data!$A$2:$A$500</c:f>
+              <c:f>Data!$A$2:$A$50000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="499"/>
+                <c:ptCount val="49999"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -1581,10 +1581,10 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Data!$E$2:$E$500</c:f>
+              <c:f>Data!$E$2:$E$50000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="499"/>
+                <c:ptCount val="49999"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -2034,10 +2034,10 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Data!$A$2:$A$500</c:f>
+              <c:f>Data!$A$2:$A$50000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="499"/>
+                <c:ptCount val="49999"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -2046,10 +2046,10 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Data!$C$2:$C$500</c:f>
+              <c:f>Data!$C$2:$C$50000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="499"/>
+                <c:ptCount val="49999"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -2290,10 +2290,10 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Data!$A$2:$A$500</c:f>
+              <c:f>Data!$A$2:$A$50000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="499"/>
+                <c:ptCount val="49999"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -2302,10 +2302,10 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Data!$D$2:$D$500</c:f>
+              <c:f>Data!$D$2:$D$50000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="499"/>
+                <c:ptCount val="49999"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -4871,8 +4871,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="612272" y="422072"/>
-          <a:ext cx="9087784" cy="4251225"/>
+          <a:off x="614350" y="423457"/>
+          <a:ext cx="9086052" cy="4244125"/>
           <a:chOff x="523959" y="465533"/>
           <a:chExt cx="9086868" cy="4291907"/>
         </a:xfrm>

</xml_diff>

<commit_message>
xlsx graph plot priorities, interface clear (Worker)
</commit_message>
<xml_diff>
--- a/web-console/server/assets/excel_template.xlsx
+++ b/web-console/server/assets/excel_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\DEV\UBA6\web-console\server\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31895CD3-2D3D-4738-BEEE-4085DA199110}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4E43470-6457-4EF9-947D-2A3CF876B303}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3E3B58E4-0181-4207-8002-E1D914CEBC2E}"/>
   </bookViews>
@@ -432,8 +432,8 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FF000000"/>
       <color rgb="FFCC0000"/>
-      <color rgb="FF000000"/>
       <color rgb="FF009999"/>
       <color rgb="FF0066FF"/>
       <color rgb="FF009900"/>
@@ -1868,7 +1868,11 @@
     </c:extLst>
   </c:chart>
   <c:spPr>
-    <a:noFill/>
+    <a:solidFill>
+      <a:srgbClr val="000000">
+        <a:alpha val="0"/>
+      </a:srgbClr>
+    </a:solidFill>
     <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:noFill/>
       <a:round/>
@@ -1894,1169 +1898,6 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
-  <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="2"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
-  <c:chart>
-    <c:autoTitleDeleted val="1"/>
-    <c:plotArea>
-      <c:layout>
-        <c:manualLayout>
-          <c:layoutTarget val="inner"/>
-          <c:xMode val="edge"/>
-          <c:yMode val="edge"/>
-          <c:x val="3.5666229321094027E-2"/>
-          <c:y val="6.6181460143433082E-2"/>
-          <c:w val="0.92413817547012744"/>
-          <c:h val="0.89478135095678857"/>
-        </c:manualLayout>
-      </c:layout>
-      <c:scatterChart>
-        <c:scatterStyle val="lineMarker"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="3"/>
-          <c:order val="0"/>
-          <c:tx>
-            <c:v>Voltage [V]</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="12700" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>Data!$A$2:$A$50000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="49999"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>Data!$C$2:$C$50000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="49999"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-D1EA-4A58-A582-9D1E456A899B}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:axId val="538752176"/>
-        <c:axId val="538753616"/>
-        <c:extLst>
-          <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-            <c15:filteredScatterSeries>
-              <c15:ser>
-                <c:idx val="4"/>
-                <c:order val="1"/>
-                <c:tx>
-                  <c:v>Temprture </c:v>
-                </c:tx>
-                <c:spPr>
-                  <a:ln w="15875" cap="rnd">
-                    <a:solidFill>
-                      <a:schemeClr val="accent5"/>
-                    </a:solidFill>
-                    <a:round/>
-                  </a:ln>
-                  <a:effectLst/>
-                </c:spPr>
-                <c:marker>
-                  <c:symbol val="none"/>
-                </c:marker>
-                <c:xVal>
-                  <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Time</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:xVal>
-                <c:yVal>
-                  <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Temp</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:yVal>
-                <c:smooth val="0"/>
-                <c:extLst>
-                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                    <c16:uniqueId val="{00000001-D1EA-4A58-A582-9D1E456A899B}"/>
-                  </c:ext>
-                </c:extLst>
-              </c15:ser>
-            </c15:filteredScatterSeries>
-            <c15:filteredScatterSeries>
-              <c15:ser>
-                <c:idx val="0"/>
-                <c:order val="3"/>
-                <c:tx>
-                  <c:v>Voltage [V]</c:v>
-                </c:tx>
-                <c:spPr>
-                  <a:ln w="15875" cap="rnd">
-                    <a:solidFill>
-                      <a:schemeClr val="accent1"/>
-                    </a:solidFill>
-                    <a:round/>
-                  </a:ln>
-                  <a:effectLst/>
-                </c:spPr>
-                <c:marker>
-                  <c:symbol val="none"/>
-                </c:marker>
-                <c:xVal>
-                  <c:numRef>
-                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>Data!$A$2:$A$500</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="499"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:xVal>
-                <c:yVal>
-                  <c:numRef>
-                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>Data!$C$2:$C$500</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="499"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:yVal>
-                <c:smooth val="0"/>
-                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                    <c16:uniqueId val="{00000003-D1EA-4A58-A582-9D1E456A899B}"/>
-                  </c:ext>
-                </c:extLst>
-              </c15:ser>
-            </c15:filteredScatterSeries>
-            <c15:filteredScatterSeries>
-              <c15:ser>
-                <c:idx val="2"/>
-                <c:order val="4"/>
-                <c:tx>
-                  <c:v>Temprture </c:v>
-                </c:tx>
-                <c:spPr>
-                  <a:ln w="15875" cap="rnd">
-                    <a:solidFill>
-                      <a:schemeClr val="accent3"/>
-                    </a:solidFill>
-                    <a:round/>
-                  </a:ln>
-                  <a:effectLst/>
-                </c:spPr>
-                <c:marker>
-                  <c:symbol val="none"/>
-                </c:marker>
-                <c:xVal>
-                  <c:numRef>
-                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Time</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:xVal>
-                <c:yVal>
-                  <c:numRef>
-                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Temp</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:yVal>
-                <c:smooth val="0"/>
-                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                    <c16:uniqueId val="{00000004-D1EA-4A58-A582-9D1E456A899B}"/>
-                  </c:ext>
-                </c:extLst>
-              </c15:ser>
-            </c15:filteredScatterSeries>
-          </c:ext>
-        </c:extLst>
-      </c:scatterChart>
-      <c:scatterChart>
-        <c:scatterStyle val="lineMarker"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="5"/>
-          <c:order val="2"/>
-          <c:tx>
-            <c:v>Current</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="12700" cap="rnd">
-              <a:solidFill>
-                <a:srgbClr val="0070C0"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>Data!$A$2:$A$50000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="49999"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>Data!$D$2:$D$50000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="49999"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-D1EA-4A58-A582-9D1E456A899B}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:axId val="418454367"/>
-        <c:axId val="418453407"/>
-      </c:scatterChart>
-      <c:valAx>
-        <c:axId val="538752176"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="1"/>
-        <c:axPos val="b"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:noFill/>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="538753616"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:valAx>
-        <c:axId val="538753616"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-          <c:min val="0"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:title>
-          <c:tx>
-            <c:rich>
-              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="all" baseline="0">
-                    <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="50000"/>
-                        <a:lumOff val="50000"/>
-                      </a:schemeClr>
-                    </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
-                    <a:ea typeface="+mn-ea"/>
-                    <a:cs typeface="+mn-cs"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:rPr lang="en-US" sz="700" cap="none" baseline="0"/>
-                  <a:t>Voltage [V]</a:t>
-                </a:r>
-              </a:p>
-            </c:rich>
-          </c:tx>
-          <c:layout>
-            <c:manualLayout>
-              <c:xMode val="edge"/>
-              <c:yMode val="edge"/>
-              <c:x val="9.8896311274100234E-4"/>
-              <c:y val="0.4547112764602021"/>
-            </c:manualLayout>
-          </c:layout>
-          <c:overlay val="0"/>
-          <c:spPr>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="all" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="50000"/>
-                      <a:lumOff val="50000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="en-IL"/>
-            </a:p>
-          </c:txPr>
-        </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="low"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="700" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="50000"/>
-                    <a:lumOff val="50000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-IL"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="538752176"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:valAx>
-        <c:axId val="418453407"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="r"/>
-        <c:title>
-          <c:tx>
-            <c:rich>
-              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="all" baseline="0">
-                    <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="50000"/>
-                        <a:lumOff val="50000"/>
-                      </a:schemeClr>
-                    </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
-                    <a:ea typeface="+mn-ea"/>
-                    <a:cs typeface="+mn-cs"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:rPr lang="en-US" sz="700" cap="none" baseline="0">
-                    <a:solidFill>
-                      <a:srgbClr val="0070C0"/>
-                    </a:solidFill>
-                  </a:rPr>
-                  <a:t>Current {mA]</a:t>
-                </a:r>
-                <a:endParaRPr lang="en-US" sz="700">
-                  <a:solidFill>
-                    <a:srgbClr val="0070C0"/>
-                  </a:solidFill>
-                </a:endParaRPr>
-              </a:p>
-            </c:rich>
-          </c:tx>
-          <c:layout>
-            <c:manualLayout>
-              <c:xMode val="edge"/>
-              <c:yMode val="edge"/>
-              <c:x val="0.94388117068734356"/>
-              <c:y val="0.43909909518572027"/>
-            </c:manualLayout>
-          </c:layout>
-          <c:overlay val="0"/>
-          <c:spPr>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="all" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="50000"/>
-                      <a:lumOff val="50000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="en-US"/>
-            </a:p>
-          </c:txPr>
-        </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="700" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:srgbClr val="0070C0"/>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-IL"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="418454367"/>
-        <c:crosses val="max"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:valAx>
-        <c:axId val="418454367"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="1"/>
-        <c:axPos val="b"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="418453407"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-    </c:plotArea>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
-    <c:extLst/>
-  </c:chart>
-  <c:spPr>
-    <a:noFill/>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:noFill/>
-      <a:round/>
-    </a:ln>
-    <a:effectLst/>
-  </c:spPr>
-  <c:txPr>
-    <a:bodyPr/>
-    <a:lstStyle/>
-    <a:p>
-      <a:pPr>
-        <a:defRPr/>
-      </a:pPr>
-      <a:endParaRPr lang="en-IL"/>
-    </a:p>
-  </c:txPr>
-  <c:printSettings>
-    <c:headerFooter/>
-    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
-    <c:pageSetup/>
-  </c:printSettings>
-</c:chartSpace>
-</file>
-
-<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
-  <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="2"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
-  <c:chart>
-    <c:autoTitleDeleted val="1"/>
-    <c:plotArea>
-      <c:layout>
-        <c:manualLayout>
-          <c:layoutTarget val="inner"/>
-          <c:xMode val="edge"/>
-          <c:yMode val="edge"/>
-          <c:x val="2.6610700965402783E-2"/>
-          <c:y val="8.6154903214406831E-2"/>
-          <c:w val="0.91542975941125893"/>
-          <c:h val="0.88589247051446551"/>
-        </c:manualLayout>
-      </c:layout>
-      <c:scatterChart>
-        <c:scatterStyle val="lineMarker"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="2"/>
-          <c:order val="2"/>
-          <c:tx>
-            <c:v>Temprture [°C]</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="12700" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="bg1"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>Data!$A$2:$A$50000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="49999"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>Data!$E$2:$E$50000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="49999"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-A053-4995-9DEF-DDF35208D668}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:axId val="538752176"/>
-        <c:axId val="538753616"/>
-        <c:extLst>
-          <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-            <c15:filteredScatterSeries>
-              <c15:ser>
-                <c:idx val="0"/>
-                <c:order val="0"/>
-                <c:tx>
-                  <c:v>Voltage [V]</c:v>
-                </c:tx>
-                <c:spPr>
-                  <a:ln w="28575" cap="rnd">
-                    <a:solidFill>
-                      <a:schemeClr val="accent6"/>
-                    </a:solidFill>
-                    <a:round/>
-                  </a:ln>
-                  <a:effectLst/>
-                </c:spPr>
-                <c:marker>
-                  <c:symbol val="none"/>
-                </c:marker>
-                <c:xVal>
-                  <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Time</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:xVal>
-                <c:yVal>
-                  <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Voltage</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:yVal>
-                <c:smooth val="0"/>
-                <c:extLst>
-                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                    <c16:uniqueId val="{00000001-A053-4995-9DEF-DDF35208D668}"/>
-                  </c:ext>
-                </c:extLst>
-              </c15:ser>
-            </c15:filteredScatterSeries>
-          </c:ext>
-        </c:extLst>
-      </c:scatterChart>
-      <c:scatterChart>
-        <c:scatterStyle val="lineMarker"/>
-        <c:varyColors val="0"/>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:axId val="548909984"/>
-        <c:axId val="572448592"/>
-        <c:extLst>
-          <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-            <c15:filteredScatterSeries>
-              <c15:ser>
-                <c:idx val="1"/>
-                <c:order val="1"/>
-                <c:tx>
-                  <c:v>Current [mA]</c:v>
-                </c:tx>
-                <c:spPr>
-                  <a:ln w="28575" cap="rnd">
-                    <a:solidFill>
-                      <a:schemeClr val="accent5"/>
-                    </a:solidFill>
-                    <a:round/>
-                  </a:ln>
-                  <a:effectLst/>
-                </c:spPr>
-                <c:marker>
-                  <c:symbol val="none"/>
-                </c:marker>
-                <c:xVal>
-                  <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Time</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:xVal>
-                <c:yVal>
-                  <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Cur</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:yVal>
-                <c:smooth val="0"/>
-                <c:extLst>
-                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                    <c16:uniqueId val="{00000002-A053-4995-9DEF-DDF35208D668}"/>
-                  </c:ext>
-                </c:extLst>
-              </c15:ser>
-            </c15:filteredScatterSeries>
-          </c:ext>
-        </c:extLst>
-      </c:scatterChart>
-      <c:valAx>
-        <c:axId val="538752176"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="1"/>
-        <c:axPos val="b"/>
-        <c:title>
-          <c:tx>
-            <c:rich>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                    <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="65000"/>
-                        <a:lumOff val="35000"/>
-                      </a:schemeClr>
-                    </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
-                    <a:ea typeface="+mn-ea"/>
-                    <a:cs typeface="+mn-cs"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:rPr lang="en-US">
-                    <a:solidFill>
-                      <a:schemeClr val="bg1"/>
-                    </a:solidFill>
-                  </a:rPr>
-                  <a:t>Axis Title</a:t>
-                </a:r>
-              </a:p>
-            </c:rich>
-          </c:tx>
-          <c:layout>
-            <c:manualLayout>
-              <c:xMode val="edge"/>
-              <c:yMode val="edge"/>
-              <c:x val="0.85113210865135691"/>
-              <c:y val="0.91862299015098592"/>
-            </c:manualLayout>
-          </c:layout>
-          <c:overlay val="0"/>
-          <c:spPr>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="65000"/>
-                      <a:lumOff val="35000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="en-IL"/>
-            </a:p>
-          </c:txPr>
-        </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="out"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="538753616"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:valAx>
-        <c:axId val="538753616"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-          <c:max val="40"/>
-          <c:min val="10"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:title>
-          <c:tx>
-            <c:rich>
-              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                    <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="65000"/>
-                        <a:lumOff val="35000"/>
-                      </a:schemeClr>
-                    </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
-                    <a:ea typeface="+mn-ea"/>
-                    <a:cs typeface="+mn-cs"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:rPr lang="en-US" sz="700" b="0">
-                    <a:solidFill>
-                      <a:srgbClr val="CC0000"/>
-                    </a:solidFill>
-                  </a:rPr>
-                  <a:t>Temperature [°C]</a:t>
-                </a:r>
-              </a:p>
-            </c:rich>
-          </c:tx>
-          <c:layout>
-            <c:manualLayout>
-              <c:xMode val="edge"/>
-              <c:yMode val="edge"/>
-              <c:x val="0.93360835377386531"/>
-              <c:y val="0.43870758937793874"/>
-            </c:manualLayout>
-          </c:layout>
-          <c:overlay val="0"/>
-          <c:spPr>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="65000"/>
-                      <a:lumOff val="35000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="en-IL"/>
-            </a:p>
-          </c:txPr>
-        </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="out"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="high"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="700" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:srgbClr val="CC0000"/>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-IL"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="538752176"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-        <c:majorUnit val="3"/>
-      </c:valAx>
-      <c:valAx>
-        <c:axId val="572448592"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-          <c:max val="40"/>
-          <c:min val="10"/>
-        </c:scaling>
-        <c:delete val="1"/>
-        <c:axPos val="r"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="out"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="548909984"/>
-        <c:crosses val="max"/>
-        <c:crossBetween val="midCat"/>
-        <c:majorUnit val="3"/>
-      </c:valAx>
-      <c:valAx>
-        <c:axId val="548909984"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-          <c:max val="1"/>
-        </c:scaling>
-        <c:delete val="1"/>
-        <c:axPos val="t"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="out"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="572448592"/>
-        <c:crosses val="max"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-    </c:plotArea>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
-    <c:extLst>
-      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
-        <c16r3:dataDisplayOptions16>
-          <c16r3:dispNaAsBlank val="1"/>
-        </c16r3:dataDisplayOptions16>
-      </c:ext>
-    </c:extLst>
-  </c:chart>
-  <c:spPr>
-    <a:noFill/>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:noFill/>
-      <a:round/>
-    </a:ln>
-    <a:effectLst/>
-  </c:spPr>
-  <c:txPr>
-    <a:bodyPr/>
-    <a:lstStyle/>
-    <a:p>
-      <a:pPr>
-        <a:defRPr/>
-      </a:pPr>
-      <a:endParaRPr lang="en-IL"/>
-    </a:p>
-  </c:txPr>
-  <c:printSettings>
-    <c:headerFooter/>
-    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
-    <c:pageSetup/>
-  </c:printSettings>
-</c:chartSpace>
-</file>
-
-<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -3521,6 +2362,1181 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="2.3778746188860379E-2"/>
+          <c:y val="8.6154897307319941E-2"/>
+          <c:w val="0.91542975941125893"/>
+          <c:h val="0.88589247051446551"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:v>Temprture [°C]</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="12700" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Data!$A$2:$A$50000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="49999"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Data!$E$2:$E$50000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="49999"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-A053-4995-9DEF-DDF35208D668}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="538752176"/>
+        <c:axId val="538753616"/>
+        <c:extLst>
+          <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+            <c15:filteredScatterSeries>
+              <c15:ser>
+                <c:idx val="0"/>
+                <c:order val="0"/>
+                <c:tx>
+                  <c:v>Voltage [V]</c:v>
+                </c:tx>
+                <c:spPr>
+                  <a:ln w="28575" cap="rnd">
+                    <a:solidFill>
+                      <a:schemeClr val="accent6"/>
+                    </a:solidFill>
+                    <a:round/>
+                  </a:ln>
+                  <a:effectLst/>
+                </c:spPr>
+                <c:marker>
+                  <c:symbol val="none"/>
+                </c:marker>
+                <c:xVal>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Time</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:xVal>
+                <c:yVal>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Voltage</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:yVal>
+                <c:smooth val="0"/>
+                <c:extLst>
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000001-A053-4995-9DEF-DDF35208D668}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredScatterSeries>
+          </c:ext>
+        </c:extLst>
+      </c:scatterChart>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="548909984"/>
+        <c:axId val="572448592"/>
+        <c:extLst>
+          <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+            <c15:filteredScatterSeries>
+              <c15:ser>
+                <c:idx val="1"/>
+                <c:order val="1"/>
+                <c:tx>
+                  <c:v>Current [mA]</c:v>
+                </c:tx>
+                <c:spPr>
+                  <a:ln w="28575" cap="rnd">
+                    <a:solidFill>
+                      <a:schemeClr val="accent5"/>
+                    </a:solidFill>
+                    <a:round/>
+                  </a:ln>
+                  <a:effectLst/>
+                </c:spPr>
+                <c:marker>
+                  <c:symbol val="none"/>
+                </c:marker>
+                <c:xVal>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Time</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:xVal>
+                <c:yVal>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Cur</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:yVal>
+                <c:smooth val="0"/>
+                <c:extLst>
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000002-A053-4995-9DEF-DDF35208D668}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredScatterSeries>
+          </c:ext>
+        </c:extLst>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="538752176"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US">
+                    <a:solidFill>
+                      <a:schemeClr val="bg1"/>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t>Axis Title</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout>
+            <c:manualLayout>
+              <c:xMode val="edge"/>
+              <c:yMode val="edge"/>
+              <c:x val="0.85113210865135691"/>
+              <c:y val="0.91862299015098592"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-IL"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="538753616"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="538753616"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="40"/>
+          <c:min val="10"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="700" b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="CC0000"/>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t>Temperature [°C]</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout>
+            <c:manualLayout>
+              <c:xMode val="edge"/>
+              <c:yMode val="edge"/>
+              <c:x val="0.93077532245615446"/>
+              <c:y val="0.43870752839497884"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-IL"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="high"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="700" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:srgbClr val="CC0000"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-IL"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="538752176"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+        <c:majorUnit val="3"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="572448592"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="40"/>
+          <c:min val="10"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="r"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="548909984"/>
+        <c:crosses val="max"/>
+        <c:crossBetween val="midCat"/>
+        <c:majorUnit val="3"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="548909984"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="1"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="t"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="572448592"/>
+        <c:crosses val="max"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:solidFill>
+          <a:srgbClr val="000000">
+            <a:alpha val="0"/>
+          </a:srgbClr>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:noFill/>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:noFill/>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-IL"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="3.5666229321094027E-2"/>
+          <c:y val="6.6181460143433082E-2"/>
+          <c:w val="0.92413817547012744"/>
+          <c:h val="0.89478135095678857"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Voltage [V]</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="12700" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Data!$A$2:$A$50000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="49999"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Data!$C$2:$C$50000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="49999"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-D1EA-4A58-A582-9D1E456A899B}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="538752176"/>
+        <c:axId val="538753616"/>
+        <c:extLst>
+          <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+            <c15:filteredScatterSeries>
+              <c15:ser>
+                <c:idx val="4"/>
+                <c:order val="1"/>
+                <c:tx>
+                  <c:v>Temprture </c:v>
+                </c:tx>
+                <c:spPr>
+                  <a:ln w="15875" cap="rnd">
+                    <a:solidFill>
+                      <a:schemeClr val="accent5"/>
+                    </a:solidFill>
+                    <a:round/>
+                  </a:ln>
+                  <a:effectLst/>
+                </c:spPr>
+                <c:marker>
+                  <c:symbol val="none"/>
+                </c:marker>
+                <c:xVal>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Time</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:xVal>
+                <c:yVal>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Temp</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:yVal>
+                <c:smooth val="0"/>
+                <c:extLst>
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000001-D1EA-4A58-A582-9D1E456A899B}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredScatterSeries>
+            <c15:filteredScatterSeries>
+              <c15:ser>
+                <c:idx val="0"/>
+                <c:order val="3"/>
+                <c:tx>
+                  <c:v>Voltage [V]</c:v>
+                </c:tx>
+                <c:spPr>
+                  <a:ln w="15875" cap="rnd">
+                    <a:solidFill>
+                      <a:schemeClr val="accent1"/>
+                    </a:solidFill>
+                    <a:round/>
+                  </a:ln>
+                  <a:effectLst/>
+                </c:spPr>
+                <c:marker>
+                  <c:symbol val="none"/>
+                </c:marker>
+                <c:xVal>
+                  <c:numRef>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>Data!$A$2:$A$500</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="499"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:xVal>
+                <c:yVal>
+                  <c:numRef>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>Data!$C$2:$C$500</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="499"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:yVal>
+                <c:smooth val="0"/>
+                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000003-D1EA-4A58-A582-9D1E456A899B}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredScatterSeries>
+            <c15:filteredScatterSeries>
+              <c15:ser>
+                <c:idx val="2"/>
+                <c:order val="4"/>
+                <c:tx>
+                  <c:v>Temprture </c:v>
+                </c:tx>
+                <c:spPr>
+                  <a:ln w="15875" cap="rnd">
+                    <a:solidFill>
+                      <a:schemeClr val="accent3"/>
+                    </a:solidFill>
+                    <a:round/>
+                  </a:ln>
+                  <a:effectLst/>
+                </c:spPr>
+                <c:marker>
+                  <c:symbol val="none"/>
+                </c:marker>
+                <c:xVal>
+                  <c:numRef>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Time</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:xVal>
+                <c:yVal>
+                  <c:numRef>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Temp</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:yVal>
+                <c:smooth val="0"/>
+                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000004-D1EA-4A58-A582-9D1E456A899B}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredScatterSeries>
+          </c:ext>
+        </c:extLst>
+      </c:scatterChart>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="5"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:v>Current</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="12700" cap="rnd">
+              <a:solidFill>
+                <a:srgbClr val="0070C0"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Data!$A$2:$A$50000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="49999"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Data!$D$2:$D$50000</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="49999"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-D1EA-4A58-A582-9D1E456A899B}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="418454367"/>
+        <c:axId val="418453407"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="538752176"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="538753616"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="538753616"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:min val="0"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="all" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="50000"/>
+                        <a:lumOff val="50000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="700" cap="none" baseline="0"/>
+                  <a:t>Voltage [V]</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout>
+            <c:manualLayout>
+              <c:xMode val="edge"/>
+              <c:yMode val="edge"/>
+              <c:x val="3.3984537135047559E-2"/>
+              <c:y val="0.45695874527714891"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="all" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="50000"/>
+                      <a:lumOff val="50000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-IL"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="low"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="700" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="50000"/>
+                    <a:lumOff val="50000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-IL"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="538752176"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="418453407"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="r"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="all" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="50000"/>
+                        <a:lumOff val="50000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="700" cap="none" baseline="0">
+                    <a:solidFill>
+                      <a:srgbClr val="0070C0"/>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t>Current {mA]</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-US" sz="700">
+                  <a:solidFill>
+                    <a:srgbClr val="0070C0"/>
+                  </a:solidFill>
+                </a:endParaRPr>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout>
+            <c:manualLayout>
+              <c:xMode val="edge"/>
+              <c:yMode val="edge"/>
+              <c:x val="0.94387922706242067"/>
+              <c:y val="0.43601249490300448"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="all" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="50000"/>
+                      <a:lumOff val="50000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="700" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:srgbClr val="0070C0"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-IL"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="418454367"/>
+        <c:crosses val="max"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="418454367"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="418453407"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:solidFill>
+          <a:srgbClr val="000000">
+            <a:alpha val="0"/>
+          </a:srgbClr>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="000000">
+        <a:alpha val="0"/>
+      </a:srgbClr>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:noFill/>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-IL"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -3639,13 +3655,10 @@
 </file>
 
 <file path=xl/charts/colors4.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
-  <a:schemeClr val="accent1"/>
-  <a:schemeClr val="accent2"/>
-  <a:schemeClr val="accent3"/>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="13">
+  <a:schemeClr val="accent6"/>
+  <a:schemeClr val="accent5"/>
   <a:schemeClr val="accent4"/>
-  <a:schemeClr val="accent5"/>
-  <a:schemeClr val="accent6"/>
   <cs:variation/>
   <cs:variation>
     <a:lumMod val="60000"/>
@@ -3716,10 +3729,13 @@
 </file>
 
 <file path=xl/charts/colors6.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="13">
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
   <a:schemeClr val="accent6"/>
-  <a:schemeClr val="accent5"/>
-  <a:schemeClr val="accent4"/>
   <cs:variation/>
   <cs:variation>
     <a:lumMod val="60000"/>
@@ -5277,6 +5293,1046 @@
 </file>
 
 <file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="323">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" b="1" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:effectRef>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:pattFill prst="narHorz">
+        <a:fgClr>
+          <a:schemeClr val="phClr"/>
+        </a:fgClr>
+        <a:bgClr>
+          <a:schemeClr val="phClr">
+            <a:lumMod val="20000"/>
+            <a:lumOff val="80000"/>
+          </a:schemeClr>
+        </a:bgClr>
+      </a:pattFill>
+      <a:effectLst>
+        <a:innerShdw blurRad="114300">
+          <a:schemeClr val="phClr"/>
+        </a:innerShdw>
+      </a:effectLst>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:pattFill prst="narHorz">
+        <a:fgClr>
+          <a:schemeClr val="phClr"/>
+        </a:fgClr>
+        <a:bgClr>
+          <a:schemeClr val="phClr">
+            <a:lumMod val="20000"/>
+            <a:lumOff val="80000"/>
+          </a:schemeClr>
+        </a:bgClr>
+      </a:pattFill>
+      <a:effectLst>
+        <a:innerShdw blurRad="114300">
+          <a:schemeClr val="phClr"/>
+        </a:innerShdw>
+      </a:effectLst>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="6"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="15875" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="50000"/>
+        <a:lumOff val="50000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1800" b="1" kern="1200" cap="all" spc="150" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style5.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="323">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" b="1" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:effectRef>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:pattFill prst="narHorz">
+        <a:fgClr>
+          <a:schemeClr val="phClr"/>
+        </a:fgClr>
+        <a:bgClr>
+          <a:schemeClr val="phClr">
+            <a:lumMod val="20000"/>
+            <a:lumOff val="80000"/>
+          </a:schemeClr>
+        </a:bgClr>
+      </a:pattFill>
+      <a:effectLst>
+        <a:innerShdw blurRad="114300">
+          <a:schemeClr val="phClr"/>
+        </a:innerShdw>
+      </a:effectLst>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:pattFill prst="narHorz">
+        <a:fgClr>
+          <a:schemeClr val="phClr"/>
+        </a:fgClr>
+        <a:bgClr>
+          <a:schemeClr val="phClr">
+            <a:lumMod val="20000"/>
+            <a:lumOff val="80000"/>
+          </a:schemeClr>
+        </a:bgClr>
+      </a:pattFill>
+      <a:effectLst>
+        <a:innerShdw blurRad="114300">
+          <a:schemeClr val="phClr"/>
+        </a:innerShdw>
+      </a:effectLst>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="6"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="15875" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="50000"/>
+        <a:lumOff val="50000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1800" b="1" kern="1200" cap="all" spc="150" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style6.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="325">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -5799,1216 +6855,120 @@
 </cs:chartStyle>
 </file>
 
-<file path=xl/charts/style5.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="323">
-  <cs:axisTitle>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" b="1" kern="1200"/>
-  </cs:axisTitle>
-  <cs:categoryAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:categoryAxis>
-  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="bg1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:chartArea>
-  <cs:dataLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataLabel>
-  <cs:dataLabelCallout>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
-      <a:spAutoFit/>
-    </cs:bodyPr>
-  </cs:dataLabelCallout>
-  <cs:dataPoint>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:effectRef>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:pattFill prst="narHorz">
-        <a:fgClr>
-          <a:schemeClr val="phClr"/>
-        </a:fgClr>
-        <a:bgClr>
-          <a:schemeClr val="phClr">
-            <a:lumMod val="20000"/>
-            <a:lumOff val="80000"/>
-          </a:schemeClr>
-        </a:bgClr>
-      </a:pattFill>
-      <a:effectLst>
-        <a:innerShdw blurRad="114300">
-          <a:schemeClr val="phClr"/>
-        </a:innerShdw>
-      </a:effectLst>
-    </cs:spPr>
-  </cs:dataPoint>
-  <cs:dataPoint3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:pattFill prst="narHorz">
-        <a:fgClr>
-          <a:schemeClr val="phClr"/>
-        </a:fgClr>
-        <a:bgClr>
-          <a:schemeClr val="phClr">
-            <a:lumMod val="20000"/>
-            <a:lumOff val="80000"/>
-          </a:schemeClr>
-        </a:bgClr>
-      </a:pattFill>
-      <a:effectLst>
-        <a:innerShdw blurRad="114300">
-          <a:schemeClr val="phClr"/>
-        </a:innerShdw>
-      </a:effectLst>
-    </cs:spPr>
-  </cs:dataPoint3D>
-  <cs:dataPointLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="28575" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointLine>
-  <cs:dataPointMarker>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="phClr"/>
-      </a:solidFill>
-    </cs:spPr>
-  </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="6"/>
-  <cs:dataPointWireframe>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointWireframe>
-  <cs:dataTable>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataTable>
-  <cs:downBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="65000"/>
-          <a:lumOff val="35000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:downBar>
-  <cs:dropLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dropLine>
-  <cs:errorBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:errorBar>
-  <cs:floor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-  </cs:floor>
-  <cs:gridlineMajor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMajor>
-  <cs:gridlineMinor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="5000"/>
-            <a:lumOff val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="15875" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:legend>
-  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-  </cs:plotArea>
-  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:seriesLine>
-  <cs:title>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="50000"/>
-        <a:lumOff val="50000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1800" b="1" kern="1200" cap="all" spc="150" baseline="0"/>
-  </cs:title>
-  <cs:trendline>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:trendline>
-  <cs:trendlineLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:trendlineLabel>
-  <cs:upBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:upBar>
-  <cs:valueAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:valueAxis>
-  <cs:wall>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-  </cs:wall>
-</cs:chartStyle>
-</file>
-
-<file path=xl/charts/style6.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="323">
-  <cs:axisTitle>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" b="1" kern="1200"/>
-  </cs:axisTitle>
-  <cs:categoryAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:categoryAxis>
-  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="bg1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:chartArea>
-  <cs:dataLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataLabel>
-  <cs:dataLabelCallout>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
-      <a:spAutoFit/>
-    </cs:bodyPr>
-  </cs:dataLabelCallout>
-  <cs:dataPoint>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:effectRef>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:pattFill prst="narHorz">
-        <a:fgClr>
-          <a:schemeClr val="phClr"/>
-        </a:fgClr>
-        <a:bgClr>
-          <a:schemeClr val="phClr">
-            <a:lumMod val="20000"/>
-            <a:lumOff val="80000"/>
-          </a:schemeClr>
-        </a:bgClr>
-      </a:pattFill>
-      <a:effectLst>
-        <a:innerShdw blurRad="114300">
-          <a:schemeClr val="phClr"/>
-        </a:innerShdw>
-      </a:effectLst>
-    </cs:spPr>
-  </cs:dataPoint>
-  <cs:dataPoint3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:pattFill prst="narHorz">
-        <a:fgClr>
-          <a:schemeClr val="phClr"/>
-        </a:fgClr>
-        <a:bgClr>
-          <a:schemeClr val="phClr">
-            <a:lumMod val="20000"/>
-            <a:lumOff val="80000"/>
-          </a:schemeClr>
-        </a:bgClr>
-      </a:pattFill>
-      <a:effectLst>
-        <a:innerShdw blurRad="114300">
-          <a:schemeClr val="phClr"/>
-        </a:innerShdw>
-      </a:effectLst>
-    </cs:spPr>
-  </cs:dataPoint3D>
-  <cs:dataPointLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="28575" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointLine>
-  <cs:dataPointMarker>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="phClr"/>
-      </a:solidFill>
-    </cs:spPr>
-  </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="6"/>
-  <cs:dataPointWireframe>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointWireframe>
-  <cs:dataTable>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataTable>
-  <cs:downBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="65000"/>
-          <a:lumOff val="35000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:downBar>
-  <cs:dropLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dropLine>
-  <cs:errorBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:errorBar>
-  <cs:floor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-  </cs:floor>
-  <cs:gridlineMajor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMajor>
-  <cs:gridlineMinor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="5000"/>
-            <a:lumOff val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="15875" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:legend>
-  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-  </cs:plotArea>
-  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:seriesLine>
-  <cs:title>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="50000"/>
-        <a:lumOff val="50000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1800" b="1" kern="1200" cap="all" spc="150" baseline="0"/>
-  </cs:title>
-  <cs:trendline>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:trendline>
-  <cs:trendlineLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:trendlineLabel>
-  <cs:upBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:upBar>
-  <cs:valueAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:valueAxis>
-  <cs:wall>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-  </cs:wall>
-</cs:chartStyle>
-</file>
-
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>101732</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>110838</xdr:rowOff>
+      <xdr:colOff>97922</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>19107</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>95860</xdr:colOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>130978</xdr:colOff>
       <xdr:row>26</xdr:row>
-      <xdr:rowOff>171782</xdr:rowOff>
+      <xdr:rowOff>167972</xdr:rowOff>
     </xdr:to>
-    <xdr:grpSp>
-      <xdr:nvGrpSpPr>
-        <xdr:cNvPr id="5" name="Group 4">
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="15" name="Chart 14">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1DBA8E76-0713-B2F3-7726-BFF4C193E576}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B6E890E5-E3CB-AD00-9116-EFF2D7DF2232}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvGrpSpPr/>
-      </xdr:nvGrpSpPr>
-      <xdr:grpSpPr>
-        <a:xfrm>
-          <a:off x="608808" y="396588"/>
-          <a:ext cx="9328628" cy="4300089"/>
-          <a:chOff x="614350" y="401783"/>
-          <a:chExt cx="9325165" cy="4265799"/>
-        </a:xfrm>
-      </xdr:grpSpPr>
-      <xdr:grpSp>
-        <xdr:nvGrpSpPr>
-          <xdr:cNvPr id="17" name="Group 16">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B9E8D104-9296-1DD8-DFB1-FA84E760CEEB}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvGrpSpPr/>
-        </xdr:nvGrpSpPr>
-        <xdr:grpSpPr>
-          <a:xfrm>
-            <a:off x="614350" y="423457"/>
-            <a:ext cx="9086052" cy="4244125"/>
-            <a:chOff x="523959" y="465533"/>
-            <a:chExt cx="9086868" cy="4291907"/>
-          </a:xfrm>
-        </xdr:grpSpPr>
-        <xdr:graphicFrame macro="">
-          <xdr:nvGraphicFramePr>
-            <xdr:cNvPr id="15" name="Chart 14">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B6E890E5-E3CB-AD00-9116-EFF2D7DF2232}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvGraphicFramePr>
-              <a:graphicFrameLocks/>
-            </xdr:cNvGraphicFramePr>
-          </xdr:nvGraphicFramePr>
-          <xdr:xfrm>
-            <a:off x="523959" y="534013"/>
-            <a:ext cx="9086868" cy="4223427"/>
-          </xdr:xfrm>
-          <a:graphic>
-            <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-              <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-            </a:graphicData>
-          </a:graphic>
-        </xdr:graphicFrame>
-        <xdr:graphicFrame macro="">
-          <xdr:nvGraphicFramePr>
-            <xdr:cNvPr id="2" name="Chart 1">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{96115982-2F8A-41D8-8A33-376961F2A802}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvGraphicFramePr>
-              <a:graphicFrameLocks/>
-            </xdr:cNvGraphicFramePr>
-          </xdr:nvGraphicFramePr>
-          <xdr:xfrm>
-            <a:off x="583897" y="612983"/>
-            <a:ext cx="8878322" cy="4123478"/>
-          </xdr:xfrm>
-          <a:graphic>
-            <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-              <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
-            </a:graphicData>
-          </a:graphic>
-        </xdr:graphicFrame>
-        <xdr:graphicFrame macro="">
-          <xdr:nvGraphicFramePr>
-            <xdr:cNvPr id="7" name="Chart 6">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{80F85B0E-700A-4724-8B40-68BD122674AB}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvGraphicFramePr>
-              <a:graphicFrameLocks/>
-            </xdr:cNvGraphicFramePr>
-          </xdr:nvGraphicFramePr>
-          <xdr:xfrm>
-            <a:off x="615858" y="465533"/>
-            <a:ext cx="8970502" cy="4144265"/>
-          </xdr:xfrm>
-          <a:graphic>
-            <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-              <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
-            </a:graphicData>
-          </a:graphic>
-        </xdr:graphicFrame>
-        <xdr:graphicFrame macro="">
-          <xdr:nvGraphicFramePr>
-            <xdr:cNvPr id="13" name="Chart 12">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B3EEA2AE-0355-4D4A-8D03-1328397FD53E}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvGraphicFramePr>
-              <a:graphicFrameLocks/>
-            </xdr:cNvGraphicFramePr>
-          </xdr:nvGraphicFramePr>
-          <xdr:xfrm>
-            <a:off x="551287" y="529385"/>
-            <a:ext cx="8861821" cy="4112035"/>
-          </xdr:xfrm>
-          <a:graphic>
-            <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-              <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
-            </a:graphicData>
-          </a:graphic>
-        </xdr:graphicFrame>
-      </xdr:grpSp>
-      <xdr:graphicFrame macro="">
-        <xdr:nvGraphicFramePr>
-          <xdr:cNvPr id="3" name="Chart 2">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A3E3B333-B126-4F82-8581-DE8E788E7472}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvGraphicFramePr>
-            <a:graphicFrameLocks/>
-          </xdr:cNvGraphicFramePr>
-        </xdr:nvGraphicFramePr>
-        <xdr:xfrm>
-          <a:off x="969819" y="401783"/>
-          <a:ext cx="8969696" cy="4098127"/>
-        </xdr:xfrm>
-        <a:graphic>
-          <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-            <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
-          </a:graphicData>
-        </a:graphic>
-      </xdr:graphicFrame>
-    </xdr:grpSp>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>6862</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>41021</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>635569</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>150869</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{96115982-2F8A-41D8-8A33-376961F2A802}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>38832</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>136496</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>110314</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>24610</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="7" name="Chart 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{80F85B0E-700A-4724-8B40-68BD122674AB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
@@ -7043,10 +7003,91 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>110620</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>97678</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>92735</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>82976</xdr:rowOff>
+    </xdr:to>
+    <xdr:grpSp>
+      <xdr:nvGrpSpPr>
+        <xdr:cNvPr id="12" name="Group 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{29F04B0A-2423-E605-13B6-7CD62A63336C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGrpSpPr/>
+      </xdr:nvGrpSpPr>
+      <xdr:grpSpPr>
+        <a:xfrm>
+          <a:off x="620888" y="374515"/>
+          <a:ext cx="9323827" cy="4158201"/>
+          <a:chOff x="621310" y="383428"/>
+          <a:chExt cx="9321752" cy="4231579"/>
+        </a:xfrm>
+      </xdr:grpSpPr>
+      <xdr:graphicFrame macro="">
+        <xdr:nvGraphicFramePr>
+          <xdr:cNvPr id="3" name="Chart 2">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A3E3B333-B126-4F82-8581-DE8E788E7472}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvGraphicFramePr>
+            <a:graphicFrameLocks/>
+          </xdr:cNvGraphicFramePr>
+        </xdr:nvGraphicFramePr>
+        <xdr:xfrm>
+          <a:off x="977502" y="383428"/>
+          <a:ext cx="8965560" cy="4136911"/>
+        </xdr:xfrm>
+        <a:graphic>
+          <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+            <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+          </a:graphicData>
+        </a:graphic>
+      </xdr:graphicFrame>
+      <xdr:graphicFrame macro="">
+        <xdr:nvGraphicFramePr>
+          <xdr:cNvPr id="13" name="Chart 12">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B3EEA2AE-0355-4D4A-8D03-1328397FD53E}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvGraphicFramePr>
+            <a:graphicFrameLocks/>
+          </xdr:cNvGraphicFramePr>
+        </xdr:nvGraphicFramePr>
+        <xdr:xfrm>
+          <a:off x="621310" y="496575"/>
+          <a:ext cx="8854916" cy="4118432"/>
+        </xdr:xfrm>
+        <a:graphic>
+          <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+            <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
+          </a:graphicData>
+        </a:graphic>
+      </xdr:graphicFrame>
+    </xdr:grpSp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>

</xml_diff>

<commit_message>
discharge voltage - safety, pdf graph
</commit_message>
<xml_diff>
--- a/web-console/server/assets/excel_template.xlsx
+++ b/web-console/server/assets/excel_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\DEV\UBA6\web-console\server\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4E43470-6457-4EF9-947D-2A3CF876B303}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23D716DC-4133-4304-A888-8D23E37D970E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3E3B58E4-0181-4207-8002-E1D914CEBC2E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{3E3B58E4-0181-4207-8002-E1D914CEBC2E}"/>
   </bookViews>
   <sheets>
     <sheet name="Report" sheetId="1" r:id="rId1"/>
@@ -236,7 +236,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -246,28 +246,6 @@
     </border>
     <border>
       <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
       <right/>
       <top/>
       <bottom style="medium">
@@ -359,39 +337,37 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
@@ -399,7 +375,6 @@
     </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="3" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1918,471 +1893,6 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="2.6610700965402783E-2"/>
-          <c:y val="8.6154903214406831E-2"/>
-          <c:w val="0.91542975941125893"/>
-          <c:h val="0.88589247051446551"/>
-        </c:manualLayout>
-      </c:layout>
-      <c:scatterChart>
-        <c:scatterStyle val="lineMarker"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="2"/>
-          <c:order val="2"/>
-          <c:tx>
-            <c:v>Temprture [°C]</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="12700" cap="rnd">
-              <a:solidFill>
-                <a:srgbClr val="C00000"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>Data!$A$2:$A$50000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="49999"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>Data!$E$2:$E$50000</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="49999"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-D0FD-465E-A621-0CF646350F47}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:axId val="538752176"/>
-        <c:axId val="538753616"/>
-        <c:extLst>
-          <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-            <c15:filteredScatterSeries>
-              <c15:ser>
-                <c:idx val="0"/>
-                <c:order val="0"/>
-                <c:tx>
-                  <c:v>Voltage [V]</c:v>
-                </c:tx>
-                <c:spPr>
-                  <a:ln w="28575" cap="rnd">
-                    <a:solidFill>
-                      <a:schemeClr val="accent6"/>
-                    </a:solidFill>
-                    <a:round/>
-                  </a:ln>
-                  <a:effectLst/>
-                </c:spPr>
-                <c:marker>
-                  <c:symbol val="none"/>
-                </c:marker>
-                <c:xVal>
-                  <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Time</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:xVal>
-                <c:yVal>
-                  <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Voltage</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:yVal>
-                <c:smooth val="0"/>
-                <c:extLst>
-                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                    <c16:uniqueId val="{00000001-D0FD-465E-A621-0CF646350F47}"/>
-                  </c:ext>
-                </c:extLst>
-              </c15:ser>
-            </c15:filteredScatterSeries>
-          </c:ext>
-        </c:extLst>
-      </c:scatterChart>
-      <c:scatterChart>
-        <c:scatterStyle val="lineMarker"/>
-        <c:varyColors val="0"/>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:axId val="548909984"/>
-        <c:axId val="572448592"/>
-        <c:extLst>
-          <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-            <c15:filteredScatterSeries>
-              <c15:ser>
-                <c:idx val="1"/>
-                <c:order val="1"/>
-                <c:tx>
-                  <c:v>Current [mA]</c:v>
-                </c:tx>
-                <c:spPr>
-                  <a:ln w="28575" cap="rnd">
-                    <a:solidFill>
-                      <a:schemeClr val="accent5"/>
-                    </a:solidFill>
-                    <a:round/>
-                  </a:ln>
-                  <a:effectLst/>
-                </c:spPr>
-                <c:marker>
-                  <c:symbol val="none"/>
-                </c:marker>
-                <c:xVal>
-                  <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Time</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:xVal>
-                <c:yVal>
-                  <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Cur</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:yVal>
-                <c:smooth val="0"/>
-                <c:extLst>
-                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                    <c16:uniqueId val="{00000002-D0FD-465E-A621-0CF646350F47}"/>
-                  </c:ext>
-                </c:extLst>
-              </c15:ser>
-            </c15:filteredScatterSeries>
-          </c:ext>
-        </c:extLst>
-      </c:scatterChart>
-      <c:valAx>
-        <c:axId val="538752176"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="1"/>
-        <c:axPos val="b"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="538753616"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:valAx>
-        <c:axId val="538753616"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-          <c:max val="40"/>
-          <c:min val="10"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="high"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="bg1"/>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-IL"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="538752176"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-        <c:majorUnit val="3"/>
-      </c:valAx>
-      <c:valAx>
-        <c:axId val="572448592"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-          <c:max val="40"/>
-          <c:min val="10"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="r"/>
-        <c:title>
-          <c:tx>
-            <c:rich>
-              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                    <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="65000"/>
-                        <a:lumOff val="35000"/>
-                      </a:schemeClr>
-                    </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
-                    <a:ea typeface="+mn-ea"/>
-                    <a:cs typeface="+mn-cs"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:rPr lang="en-US" sz="700" b="0">
-                    <a:solidFill>
-                      <a:srgbClr val="CC0000"/>
-                    </a:solidFill>
-                  </a:rPr>
-                  <a:t>Temperature [°C]</a:t>
-                </a:r>
-              </a:p>
-            </c:rich>
-          </c:tx>
-          <c:layout>
-            <c:manualLayout>
-              <c:xMode val="edge"/>
-              <c:yMode val="edge"/>
-              <c:x val="0.9635665803108231"/>
-              <c:y val="0.4374240861470281"/>
-            </c:manualLayout>
-          </c:layout>
-          <c:overlay val="0"/>
-          <c:spPr>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="65000"/>
-                      <a:lumOff val="35000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="en-IL"/>
-            </a:p>
-          </c:txPr>
-        </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="700" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:srgbClr val="C00000"/>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-IL"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="548909984"/>
-        <c:crosses val="max"/>
-        <c:crossBetween val="midCat"/>
-        <c:majorUnit val="3"/>
-      </c:valAx>
-      <c:valAx>
-        <c:axId val="548909984"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-          <c:max val="1"/>
-        </c:scaling>
-        <c:delete val="1"/>
-        <c:axPos val="t"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="572448592"/>
-        <c:crosses val="max"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-    </c:plotArea>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
-    <c:extLst>
-      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
-        <c16r3:dataDisplayOptions16>
-          <c16r3:dispNaAsBlank val="1"/>
-        </c16r3:dataDisplayOptions16>
-      </c:ext>
-    </c:extLst>
-  </c:chart>
-  <c:spPr>
-    <a:noFill/>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:noFill/>
-      <a:round/>
-    </a:ln>
-    <a:effectLst/>
-  </c:spPr>
-  <c:txPr>
-    <a:bodyPr/>
-    <a:lstStyle/>
-    <a:p>
-      <a:pPr>
-        <a:defRPr/>
-      </a:pPr>
-      <a:endParaRPr lang="en-IL"/>
-    </a:p>
-  </c:txPr>
-  <c:printSettings>
-    <c:headerFooter/>
-    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
-    <c:pageSetup/>
-  </c:printSettings>
-</c:chartSpace>
-</file>
-
-<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
-  <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="2"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
-  <c:chart>
-    <c:autoTitleDeleted val="1"/>
-    <c:plotArea>
-      <c:layout>
-        <c:manualLayout>
-          <c:layoutTarget val="inner"/>
-          <c:xMode val="edge"/>
-          <c:yMode val="edge"/>
           <c:x val="2.3778746188860379E-2"/>
           <c:y val="8.6154897307319941E-2"/>
           <c:w val="0.91542975941125893"/>
@@ -2874,7 +2384,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -3692,43 +3202,6 @@
 </file>
 
 <file path=xl/charts/colors5.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="13">
-  <a:schemeClr val="accent6"/>
-  <a:schemeClr val="accent5"/>
-  <a:schemeClr val="accent4"/>
-  <cs:variation/>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-    <a:lumOff val="20000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-    <a:lumOff val="40000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-    <a:lumOff val="30000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-    <a:lumOff val="50000"/>
-  </cs:variation>
-</cs:colorStyle>
-</file>
-
-<file path=xl/charts/colors6.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -5813,526 +5286,6 @@
 </file>
 
 <file path=xl/charts/style5.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="323">
-  <cs:axisTitle>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" b="1" kern="1200"/>
-  </cs:axisTitle>
-  <cs:categoryAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:categoryAxis>
-  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="bg1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:chartArea>
-  <cs:dataLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataLabel>
-  <cs:dataLabelCallout>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
-      <a:spAutoFit/>
-    </cs:bodyPr>
-  </cs:dataLabelCallout>
-  <cs:dataPoint>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:effectRef>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:pattFill prst="narHorz">
-        <a:fgClr>
-          <a:schemeClr val="phClr"/>
-        </a:fgClr>
-        <a:bgClr>
-          <a:schemeClr val="phClr">
-            <a:lumMod val="20000"/>
-            <a:lumOff val="80000"/>
-          </a:schemeClr>
-        </a:bgClr>
-      </a:pattFill>
-      <a:effectLst>
-        <a:innerShdw blurRad="114300">
-          <a:schemeClr val="phClr"/>
-        </a:innerShdw>
-      </a:effectLst>
-    </cs:spPr>
-  </cs:dataPoint>
-  <cs:dataPoint3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:pattFill prst="narHorz">
-        <a:fgClr>
-          <a:schemeClr val="phClr"/>
-        </a:fgClr>
-        <a:bgClr>
-          <a:schemeClr val="phClr">
-            <a:lumMod val="20000"/>
-            <a:lumOff val="80000"/>
-          </a:schemeClr>
-        </a:bgClr>
-      </a:pattFill>
-      <a:effectLst>
-        <a:innerShdw blurRad="114300">
-          <a:schemeClr val="phClr"/>
-        </a:innerShdw>
-      </a:effectLst>
-    </cs:spPr>
-  </cs:dataPoint3D>
-  <cs:dataPointLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="28575" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointLine>
-  <cs:dataPointMarker>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="phClr"/>
-      </a:solidFill>
-    </cs:spPr>
-  </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="6"/>
-  <cs:dataPointWireframe>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointWireframe>
-  <cs:dataTable>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataTable>
-  <cs:downBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="65000"/>
-          <a:lumOff val="35000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:downBar>
-  <cs:dropLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dropLine>
-  <cs:errorBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:errorBar>
-  <cs:floor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-  </cs:floor>
-  <cs:gridlineMajor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMajor>
-  <cs:gridlineMinor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="5000"/>
-            <a:lumOff val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="15875" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:legend>
-  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-  </cs:plotArea>
-  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:seriesLine>
-  <cs:title>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="50000"/>
-        <a:lumOff val="50000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1800" b="1" kern="1200" cap="all" spc="150" baseline="0"/>
-  </cs:title>
-  <cs:trendline>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:trendline>
-  <cs:trendlineLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:trendlineLabel>
-  <cs:upBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:upBar>
-  <cs:valueAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:valueAxis>
-  <cs:wall>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-  </cs:wall>
-</cs:chartStyle>
-</file>
-
-<file path=xl/charts/style6.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="325">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -6974,44 +5927,6 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>80</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>573841</xdr:colOff>
-      <xdr:row>102</xdr:row>
-      <xdr:rowOff>135727</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="4" name="Chart 3">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B05BCB74-3B44-4AC2-98BA-5C254D133077}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr>
-          <a:graphicFrameLocks/>
-        </xdr:cNvGraphicFramePr>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>1</xdr:col>
       <xdr:colOff>110620</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>97678</xdr:rowOff>
@@ -7035,8 +5950,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="620888" y="374515"/>
-          <a:ext cx="9323827" cy="4158201"/>
+          <a:off x="620888" y="390232"/>
+          <a:ext cx="9275793" cy="4271548"/>
           <a:chOff x="621310" y="383428"/>
           <a:chExt cx="9321752" cy="4231579"/>
         </a:xfrm>
@@ -7060,7 +5975,7 @@
         </xdr:xfrm>
         <a:graphic>
           <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-            <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+            <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
           </a:graphicData>
         </a:graphic>
       </xdr:graphicFrame>
@@ -7083,7 +5998,7 @@
         </xdr:xfrm>
         <a:graphic>
           <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-            <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
+            <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
           </a:graphicData>
         </a:graphic>
       </xdr:graphicFrame>
@@ -7409,7 +6324,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:O78"/>
+  <dimension ref="B1:O123"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.44140625" style="2" customWidth="1"/>
@@ -7426,7 +6341,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="J1" s="20"/>
+      <c r="J1" s="19"/>
     </row>
     <row r="2" spans="2:14" ht="8.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="3"/>
@@ -7473,266 +6388,266 @@
     </row>
     <row r="5" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B5" s="12"/>
-      <c r="C5" s="24"/>
-      <c r="D5" s="24"/>
-      <c r="E5" s="24"/>
-      <c r="F5" s="24"/>
-      <c r="G5" s="24"/>
-      <c r="H5" s="24"/>
-      <c r="I5" s="24"/>
-      <c r="J5" s="24"/>
+      <c r="C5" s="22"/>
+      <c r="D5" s="22"/>
+      <c r="E5" s="22"/>
+      <c r="F5" s="22"/>
+      <c r="G5" s="22"/>
+      <c r="H5" s="22"/>
+      <c r="I5" s="22"/>
+      <c r="J5" s="22"/>
       <c r="K5" s="13"/>
     </row>
     <row r="6" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B6" s="12"/>
-      <c r="C6" s="24"/>
-      <c r="D6" s="24"/>
-      <c r="E6" s="24"/>
-      <c r="F6" s="24"/>
-      <c r="G6" s="24"/>
-      <c r="H6" s="24"/>
-      <c r="I6" s="24"/>
-      <c r="J6" s="24"/>
+      <c r="C6" s="22"/>
+      <c r="D6" s="22"/>
+      <c r="E6" s="22"/>
+      <c r="F6" s="22"/>
+      <c r="G6" s="22"/>
+      <c r="H6" s="22"/>
+      <c r="I6" s="22"/>
+      <c r="J6" s="22"/>
       <c r="K6" s="13"/>
     </row>
     <row r="7" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B7" s="12"/>
-      <c r="C7" s="24"/>
-      <c r="D7" s="24"/>
-      <c r="E7" s="24"/>
-      <c r="F7" s="24"/>
-      <c r="G7" s="24"/>
-      <c r="H7" s="24"/>
-      <c r="I7" s="24"/>
-      <c r="J7" s="24"/>
+      <c r="C7" s="22"/>
+      <c r="D7" s="22"/>
+      <c r="E7" s="22"/>
+      <c r="F7" s="22"/>
+      <c r="G7" s="22"/>
+      <c r="H7" s="22"/>
+      <c r="I7" s="22"/>
+      <c r="J7" s="22"/>
       <c r="K7" s="13"/>
     </row>
     <row r="8" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B8" s="12"/>
-      <c r="C8" s="24"/>
-      <c r="D8" s="24"/>
-      <c r="E8" s="24"/>
-      <c r="F8" s="24"/>
-      <c r="G8" s="24"/>
-      <c r="H8" s="24"/>
-      <c r="I8" s="24"/>
-      <c r="J8" s="24"/>
+      <c r="C8" s="22"/>
+      <c r="D8" s="22"/>
+      <c r="E8" s="22"/>
+      <c r="F8" s="22"/>
+      <c r="G8" s="22"/>
+      <c r="H8" s="22"/>
+      <c r="I8" s="22"/>
+      <c r="J8" s="22"/>
       <c r="K8" s="13"/>
     </row>
     <row r="9" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B9" s="12"/>
-      <c r="C9" s="24"/>
-      <c r="D9" s="24"/>
-      <c r="E9" s="24"/>
-      <c r="F9" s="24"/>
-      <c r="G9" s="24"/>
-      <c r="H9" s="24"/>
-      <c r="I9" s="24"/>
-      <c r="J9" s="24"/>
+      <c r="C9" s="22"/>
+      <c r="D9" s="22"/>
+      <c r="E9" s="22"/>
+      <c r="F9" s="22"/>
+      <c r="G9" s="22"/>
+      <c r="H9" s="22"/>
+      <c r="I9" s="22"/>
+      <c r="J9" s="22"/>
       <c r="K9" s="13"/>
     </row>
     <row r="10" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B10" s="12"/>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="24"/>
-      <c r="G10" s="24"/>
-      <c r="H10" s="24"/>
-      <c r="I10" s="24"/>
-      <c r="J10" s="24"/>
+      <c r="C10" s="22"/>
+      <c r="D10" s="22"/>
+      <c r="E10" s="22"/>
+      <c r="F10" s="22"/>
+      <c r="G10" s="22"/>
+      <c r="H10" s="22"/>
+      <c r="I10" s="22"/>
+      <c r="J10" s="22"/>
       <c r="K10" s="13"/>
     </row>
     <row r="11" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B11" s="12"/>
-      <c r="C11" s="24"/>
-      <c r="D11" s="24"/>
-      <c r="E11" s="24"/>
-      <c r="F11" s="24"/>
-      <c r="G11" s="24"/>
-      <c r="H11" s="24"/>
-      <c r="I11" s="24"/>
-      <c r="J11" s="24"/>
+      <c r="C11" s="22"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="22"/>
+      <c r="F11" s="22"/>
+      <c r="G11" s="22"/>
+      <c r="H11" s="22"/>
+      <c r="I11" s="22"/>
+      <c r="J11" s="22"/>
       <c r="K11" s="13"/>
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B12" s="12"/>
-      <c r="C12" s="24"/>
-      <c r="D12" s="24"/>
-      <c r="E12" s="24"/>
-      <c r="F12" s="24"/>
-      <c r="G12" s="24"/>
-      <c r="H12" s="24"/>
-      <c r="I12" s="24"/>
-      <c r="J12" s="24"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="22"/>
+      <c r="G12" s="22"/>
+      <c r="H12" s="22"/>
+      <c r="I12" s="22"/>
+      <c r="J12" s="22"/>
       <c r="K12" s="13"/>
     </row>
     <row r="13" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B13" s="12"/>
-      <c r="C13" s="24"/>
-      <c r="D13" s="24"/>
-      <c r="E13" s="24"/>
-      <c r="F13" s="24"/>
-      <c r="G13" s="24"/>
-      <c r="H13" s="24"/>
-      <c r="I13" s="24"/>
-      <c r="J13" s="24"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="22"/>
+      <c r="F13" s="22"/>
+      <c r="G13" s="22"/>
+      <c r="H13" s="22"/>
+      <c r="I13" s="22"/>
+      <c r="J13" s="22"/>
       <c r="K13" s="13"/>
     </row>
     <row r="14" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B14" s="12"/>
-      <c r="C14" s="24"/>
-      <c r="D14" s="24"/>
-      <c r="E14" s="24"/>
-      <c r="F14" s="24"/>
-      <c r="G14" s="24"/>
-      <c r="H14" s="24"/>
-      <c r="I14" s="24"/>
-      <c r="J14" s="24"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="22"/>
+      <c r="F14" s="22"/>
+      <c r="G14" s="22"/>
+      <c r="H14" s="22"/>
+      <c r="I14" s="22"/>
+      <c r="J14" s="22"/>
       <c r="K14" s="13"/>
     </row>
     <row r="15" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B15" s="12"/>
-      <c r="C15" s="24"/>
-      <c r="D15" s="24"/>
-      <c r="E15" s="24"/>
-      <c r="F15" s="24"/>
-      <c r="G15" s="24"/>
-      <c r="H15" s="24"/>
-      <c r="I15" s="24"/>
-      <c r="J15" s="24"/>
+      <c r="C15" s="22"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="22"/>
+      <c r="F15" s="22"/>
+      <c r="G15" s="22"/>
+      <c r="H15" s="22"/>
+      <c r="I15" s="22"/>
+      <c r="J15" s="22"/>
       <c r="K15" s="13"/>
     </row>
     <row r="16" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B16" s="12"/>
-      <c r="C16" s="24"/>
-      <c r="D16" s="24"/>
-      <c r="E16" s="24"/>
-      <c r="F16" s="24"/>
-      <c r="G16" s="24"/>
-      <c r="H16" s="24"/>
-      <c r="I16" s="24"/>
-      <c r="J16" s="24"/>
+      <c r="C16" s="22"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="22"/>
+      <c r="F16" s="22"/>
+      <c r="G16" s="22"/>
+      <c r="H16" s="22"/>
+      <c r="I16" s="22"/>
+      <c r="J16" s="22"/>
       <c r="K16" s="13"/>
     </row>
     <row r="17" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B17" s="12"/>
-      <c r="C17" s="24"/>
-      <c r="D17" s="24"/>
-      <c r="E17" s="24"/>
-      <c r="F17" s="24"/>
-      <c r="G17" s="24"/>
-      <c r="H17" s="24"/>
-      <c r="I17" s="24"/>
-      <c r="J17" s="24"/>
+      <c r="C17" s="22"/>
+      <c r="D17" s="22"/>
+      <c r="E17" s="22"/>
+      <c r="F17" s="22"/>
+      <c r="G17" s="22"/>
+      <c r="H17" s="22"/>
+      <c r="I17" s="22"/>
+      <c r="J17" s="22"/>
       <c r="K17" s="13"/>
     </row>
     <row r="18" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B18" s="12"/>
-      <c r="C18" s="24"/>
-      <c r="D18" s="24"/>
-      <c r="E18" s="24"/>
-      <c r="F18" s="24"/>
-      <c r="G18" s="24"/>
-      <c r="H18" s="24"/>
-      <c r="I18" s="24"/>
-      <c r="J18" s="24"/>
+      <c r="C18" s="22"/>
+      <c r="D18" s="22"/>
+      <c r="E18" s="22"/>
+      <c r="F18" s="22"/>
+      <c r="G18" s="22"/>
+      <c r="H18" s="22"/>
+      <c r="I18" s="22"/>
+      <c r="J18" s="22"/>
       <c r="K18" s="13"/>
     </row>
     <row r="19" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B19" s="12"/>
-      <c r="C19" s="24"/>
-      <c r="D19" s="24"/>
-      <c r="E19" s="24"/>
-      <c r="F19" s="24"/>
-      <c r="G19" s="24"/>
-      <c r="H19" s="24"/>
-      <c r="I19" s="24"/>
-      <c r="J19" s="24"/>
+      <c r="C19" s="22"/>
+      <c r="D19" s="22"/>
+      <c r="E19" s="22"/>
+      <c r="F19" s="22"/>
+      <c r="G19" s="22"/>
+      <c r="H19" s="22"/>
+      <c r="I19" s="22"/>
+      <c r="J19" s="22"/>
       <c r="K19" s="13"/>
     </row>
     <row r="20" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B20" s="12"/>
-      <c r="C20" s="24"/>
-      <c r="D20" s="24"/>
-      <c r="E20" s="24"/>
-      <c r="F20" s="24"/>
-      <c r="G20" s="24"/>
-      <c r="H20" s="24"/>
-      <c r="I20" s="24"/>
-      <c r="J20" s="24"/>
+      <c r="C20" s="22"/>
+      <c r="D20" s="22"/>
+      <c r="E20" s="22"/>
+      <c r="F20" s="22"/>
+      <c r="G20" s="22"/>
+      <c r="H20" s="22"/>
+      <c r="I20" s="22"/>
+      <c r="J20" s="22"/>
       <c r="K20" s="13"/>
     </row>
     <row r="21" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B21" s="12"/>
-      <c r="C21" s="24"/>
-      <c r="D21" s="24"/>
-      <c r="E21" s="24"/>
-      <c r="F21" s="24"/>
-      <c r="G21" s="24"/>
-      <c r="H21" s="24"/>
-      <c r="I21" s="24"/>
-      <c r="J21" s="24"/>
+      <c r="C21" s="22"/>
+      <c r="D21" s="22"/>
+      <c r="E21" s="22"/>
+      <c r="F21" s="22"/>
+      <c r="G21" s="22"/>
+      <c r="H21" s="22"/>
+      <c r="I21" s="22"/>
+      <c r="J21" s="22"/>
       <c r="K21" s="13"/>
     </row>
     <row r="22" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B22" s="12"/>
-      <c r="C22" s="24"/>
-      <c r="D22" s="24"/>
-      <c r="E22" s="24"/>
-      <c r="F22" s="24"/>
-      <c r="G22" s="24"/>
-      <c r="H22" s="24"/>
-      <c r="I22" s="24"/>
-      <c r="J22" s="24"/>
+      <c r="C22" s="22"/>
+      <c r="D22" s="22"/>
+      <c r="E22" s="22"/>
+      <c r="F22" s="22"/>
+      <c r="G22" s="22"/>
+      <c r="H22" s="22"/>
+      <c r="I22" s="22"/>
+      <c r="J22" s="22"/>
       <c r="K22" s="13"/>
     </row>
     <row r="23" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B23" s="12"/>
-      <c r="C23" s="24"/>
-      <c r="D23" s="24"/>
-      <c r="E23" s="24"/>
-      <c r="F23" s="24"/>
-      <c r="G23" s="24"/>
-      <c r="H23" s="24"/>
-      <c r="I23" s="24"/>
-      <c r="J23" s="24"/>
+      <c r="C23" s="22"/>
+      <c r="D23" s="22"/>
+      <c r="E23" s="22"/>
+      <c r="F23" s="22"/>
+      <c r="G23" s="22"/>
+      <c r="H23" s="22"/>
+      <c r="I23" s="22"/>
+      <c r="J23" s="22"/>
       <c r="K23" s="13"/>
     </row>
     <row r="24" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B24" s="12"/>
-      <c r="C24" s="24"/>
-      <c r="D24" s="24"/>
-      <c r="E24" s="24"/>
-      <c r="F24" s="24"/>
-      <c r="G24" s="24"/>
-      <c r="H24" s="24"/>
-      <c r="I24" s="24"/>
-      <c r="J24" s="24"/>
+      <c r="C24" s="22"/>
+      <c r="D24" s="22"/>
+      <c r="E24" s="22"/>
+      <c r="F24" s="22"/>
+      <c r="G24" s="22"/>
+      <c r="H24" s="22"/>
+      <c r="I24" s="22"/>
+      <c r="J24" s="22"/>
       <c r="K24" s="13"/>
     </row>
     <row r="25" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B25" s="12"/>
-      <c r="C25" s="24"/>
-      <c r="D25" s="24"/>
-      <c r="E25" s="24"/>
-      <c r="F25" s="24"/>
-      <c r="G25" s="24"/>
-      <c r="H25" s="24"/>
-      <c r="I25" s="24"/>
-      <c r="J25" s="24"/>
+      <c r="C25" s="22"/>
+      <c r="D25" s="22"/>
+      <c r="E25" s="22"/>
+      <c r="F25" s="22"/>
+      <c r="G25" s="22"/>
+      <c r="H25" s="22"/>
+      <c r="I25" s="22"/>
+      <c r="J25" s="22"/>
       <c r="K25" s="13"/>
     </row>
     <row r="26" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B26" s="12"/>
-      <c r="C26" s="24"/>
-      <c r="D26" s="24"/>
-      <c r="E26" s="24"/>
-      <c r="F26" s="24"/>
-      <c r="G26" s="24"/>
-      <c r="H26" s="24"/>
-      <c r="I26" s="24"/>
-      <c r="J26" s="24"/>
+      <c r="C26" s="22"/>
+      <c r="D26" s="22"/>
+      <c r="E26" s="22"/>
+      <c r="F26" s="22"/>
+      <c r="G26" s="22"/>
+      <c r="H26" s="22"/>
+      <c r="I26" s="22"/>
+      <c r="J26" s="22"/>
       <c r="K26" s="13"/>
       <c r="M26" s="14"/>
     </row>
@@ -7754,7 +6669,7 @@
       <c r="I28" s="8"/>
       <c r="J28" s="8"/>
       <c r="K28" s="9"/>
-      <c r="L28" s="23"/>
+      <c r="L28" s="21"/>
       <c r="M28" s="15"/>
     </row>
     <row r="29" spans="2:15" x14ac:dyDescent="0.3">
@@ -7765,9 +6680,9 @@
       <c r="H29" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I29" s="25"/>
+      <c r="I29" s="23"/>
       <c r="K29" s="13"/>
-      <c r="L29" s="23"/>
+      <c r="L29" s="21"/>
       <c r="M29" s="16"/>
     </row>
     <row r="30" spans="2:15" x14ac:dyDescent="0.3">
@@ -7775,7 +6690,7 @@
       <c r="H30" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I30" s="25"/>
+      <c r="I30" s="23"/>
       <c r="K30" s="13"/>
       <c r="L30" s="17"/>
       <c r="M30" s="17"/>
@@ -7790,7 +6705,7 @@
       <c r="H31" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="I31" s="25"/>
+      <c r="I31" s="23"/>
       <c r="K31" s="13"/>
       <c r="L31" s="17"/>
       <c r="M31" s="17"/>
@@ -7808,7 +6723,7 @@
       <c r="H32" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="I32" s="25"/>
+      <c r="I32" s="23"/>
       <c r="J32" s="2" t="s">
         <v>30</v>
       </c>
@@ -7823,7 +6738,7 @@
       <c r="H33" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="I33" s="25"/>
+      <c r="I33" s="23"/>
       <c r="J33" s="2" t="s">
         <v>31</v>
       </c>
@@ -7838,7 +6753,7 @@
       <c r="H34" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="I34" s="25"/>
+      <c r="I34" s="23"/>
       <c r="J34" s="2" t="s">
         <v>1</v>
       </c>
@@ -7853,7 +6768,7 @@
       <c r="H35" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I35" s="25"/>
+      <c r="I35" s="23"/>
       <c r="K35" s="13"/>
       <c r="L35" s="17"/>
       <c r="M35" s="17"/>
@@ -7868,7 +6783,7 @@
       <c r="H36" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="I36" s="25"/>
+      <c r="I36" s="23"/>
       <c r="K36" s="13"/>
       <c r="L36" s="17"/>
       <c r="M36" s="17"/>
@@ -7883,7 +6798,7 @@
       <c r="H37" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="I37" s="25"/>
+      <c r="I37" s="23"/>
       <c r="K37" s="13"/>
       <c r="L37" s="17"/>
       <c r="M37" s="17"/>
@@ -7903,15 +6818,15 @@
     </row>
     <row r="39" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B39" s="12"/>
-      <c r="D39" s="28" t="s">
+      <c r="D39" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="E39" s="28"/>
-      <c r="F39" s="28"/>
-      <c r="G39" s="28"/>
-      <c r="H39" s="28"/>
-      <c r="I39" s="28"/>
-      <c r="J39" s="28"/>
+      <c r="E39" s="25"/>
+      <c r="F39" s="25"/>
+      <c r="G39" s="25"/>
+      <c r="H39" s="25"/>
+      <c r="I39" s="25"/>
+      <c r="J39" s="25"/>
       <c r="K39" s="13"/>
       <c r="L39" s="17"/>
       <c r="M39" s="17"/>
@@ -8227,20 +7142,194 @@
     <row r="77" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B77" s="12"/>
       <c r="K77" s="13"/>
-      <c r="L77" s="23"/>
-      <c r="M77" s="22"/>
-    </row>
-    <row r="78" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B78" s="19"/>
-      <c r="C78" s="20"/>
-      <c r="D78" s="20"/>
-      <c r="E78" s="20"/>
-      <c r="F78" s="20"/>
-      <c r="G78" s="20"/>
-      <c r="H78" s="27"/>
-      <c r="I78" s="27"/>
-      <c r="J78" s="27"/>
-      <c r="K78" s="21"/>
+      <c r="M77" s="20"/>
+    </row>
+    <row r="78" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="B78" s="12"/>
+      <c r="H78" s="8"/>
+      <c r="I78" s="8"/>
+      <c r="J78" s="8"/>
+      <c r="K78" s="13"/>
+    </row>
+    <row r="79" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="B79" s="12"/>
+      <c r="K79" s="13"/>
+    </row>
+    <row r="80" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="B80" s="12"/>
+      <c r="K80" s="13"/>
+    </row>
+    <row r="81" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B81" s="12"/>
+      <c r="K81" s="13"/>
+    </row>
+    <row r="82" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B82" s="12"/>
+      <c r="K82" s="13"/>
+    </row>
+    <row r="83" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B83" s="12"/>
+      <c r="K83" s="13"/>
+    </row>
+    <row r="84" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B84" s="12"/>
+      <c r="K84" s="13"/>
+    </row>
+    <row r="85" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B85" s="12"/>
+      <c r="K85" s="13"/>
+    </row>
+    <row r="86" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B86" s="12"/>
+      <c r="K86" s="13"/>
+    </row>
+    <row r="87" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B87" s="12"/>
+      <c r="K87" s="13"/>
+    </row>
+    <row r="88" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B88" s="12"/>
+      <c r="K88" s="13"/>
+    </row>
+    <row r="89" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B89" s="12"/>
+      <c r="K89" s="13"/>
+    </row>
+    <row r="90" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B90" s="12"/>
+      <c r="K90" s="13"/>
+    </row>
+    <row r="91" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B91" s="12"/>
+      <c r="K91" s="13"/>
+    </row>
+    <row r="92" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B92" s="12"/>
+      <c r="K92" s="13"/>
+    </row>
+    <row r="93" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B93" s="12"/>
+      <c r="K93" s="13"/>
+    </row>
+    <row r="94" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B94" s="12"/>
+      <c r="K94" s="13"/>
+    </row>
+    <row r="95" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B95" s="12"/>
+      <c r="K95" s="13"/>
+    </row>
+    <row r="96" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B96" s="12"/>
+      <c r="K96" s="13"/>
+    </row>
+    <row r="97" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B97" s="12"/>
+      <c r="K97" s="13"/>
+    </row>
+    <row r="98" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B98" s="12"/>
+      <c r="K98" s="13"/>
+    </row>
+    <row r="99" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B99" s="12"/>
+      <c r="K99" s="13"/>
+    </row>
+    <row r="100" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B100" s="12"/>
+      <c r="K100" s="13"/>
+    </row>
+    <row r="101" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B101" s="12"/>
+      <c r="K101" s="13"/>
+    </row>
+    <row r="102" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B102" s="12"/>
+      <c r="K102" s="13"/>
+    </row>
+    <row r="103" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B103" s="12"/>
+      <c r="K103" s="13"/>
+    </row>
+    <row r="104" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B104" s="12"/>
+      <c r="K104" s="13"/>
+    </row>
+    <row r="105" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B105" s="12"/>
+      <c r="K105" s="13"/>
+    </row>
+    <row r="106" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B106" s="12"/>
+      <c r="K106" s="13"/>
+    </row>
+    <row r="107" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B107" s="12"/>
+      <c r="K107" s="13"/>
+    </row>
+    <row r="108" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B108" s="12"/>
+      <c r="K108" s="13"/>
+    </row>
+    <row r="109" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B109" s="12"/>
+      <c r="K109" s="13"/>
+    </row>
+    <row r="110" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B110" s="12"/>
+      <c r="K110" s="13"/>
+    </row>
+    <row r="111" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B111" s="12"/>
+      <c r="K111" s="13"/>
+    </row>
+    <row r="112" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B112" s="12"/>
+      <c r="K112" s="13"/>
+    </row>
+    <row r="113" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B113" s="12"/>
+      <c r="K113" s="13"/>
+    </row>
+    <row r="114" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B114" s="12"/>
+      <c r="K114" s="13"/>
+    </row>
+    <row r="115" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B115" s="12"/>
+      <c r="K115" s="13"/>
+    </row>
+    <row r="116" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B116" s="12"/>
+      <c r="K116" s="13"/>
+    </row>
+    <row r="117" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B117" s="12"/>
+      <c r="K117" s="13"/>
+    </row>
+    <row r="118" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B118" s="12"/>
+      <c r="K118" s="13"/>
+    </row>
+    <row r="119" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B119" s="12"/>
+      <c r="K119" s="13"/>
+    </row>
+    <row r="120" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B120" s="12"/>
+      <c r="K120" s="13"/>
+    </row>
+    <row r="121" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B121" s="12"/>
+      <c r="K121" s="13"/>
+    </row>
+    <row r="122" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B122" s="12"/>
+      <c r="K122" s="13"/>
+    </row>
+    <row r="123" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B123" s="12"/>
+      <c r="K123" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -8267,25 +7356,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="24" t="s">
         <v>24</v>
       </c>
       <c r="B1" t="s">
         <v>26</v>
       </c>
-      <c r="C1" s="26" t="s">
+      <c r="C1" s="24" t="s">
         <v>23</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="E1" s="26" t="s">
+      <c r="E1" s="24" t="s">
         <v>25</v>
       </c>
       <c r="F1" t="s">
         <v>27</v>
       </c>
-      <c r="G1" s="26" t="s">
+      <c r="G1" s="24" t="s">
         <v>28</v>
       </c>
     </row>

</xml_diff>

<commit_message>
bug 16: sample rate - download XLSX/PDF files (not yet finished)
</commit_message>
<xml_diff>
--- a/web-console/server/assets/excel_template.xlsx
+++ b/web-console/server/assets/excel_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\DEV\UBA6\web-console\server\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23D716DC-4133-4304-A888-8D23E37D970E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97BA26B2-DCF2-4EC1-B818-EBEA7FF1D235}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{3E3B58E4-0181-4207-8002-E1D914CEBC2E}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{3E3B58E4-0181-4207-8002-E1D914CEBC2E}"/>
   </bookViews>
   <sheets>
     <sheet name="Report" sheetId="1" r:id="rId1"/>
@@ -41,8 +41,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="33">
   <si>
     <t>Wh</t>
   </si>
@@ -162,12 +184,15 @@
   <si>
     <t>Parallel</t>
   </si>
+  <si>
+    <t>Sample Rate</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -221,8 +246,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -235,8 +268,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor theme="4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -331,13 +370,37 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
@@ -378,6 +441,8 @@
     <xf numFmtId="49" fontId="3" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="11" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -508,6 +573,171 @@
             </c:ext>
           </c:extLst>
         </c:ser>
+        <c:ser>
+          <c:idx val="4"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Temprture </c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst>
+              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                <a:srgbClr val="000000">
+                  <a:alpha val="63000"/>
+                </a:srgbClr>
+              </a:outerShdw>
+            </a:effectLst>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>[0]!Time</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>[0]!Temp</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-71AD-41FA-AA0E-8879577C3941}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="5"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:v>Current</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst>
+              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                <a:srgbClr val="000000">
+                  <a:alpha val="63000"/>
+                </a:srgbClr>
+              </a:outerShdw>
+            </a:effectLst>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>[0]!Time</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>[0]!Cur</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-71AD-41FA-AA0E-8879577C3941}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="4"/>
+          <c:tx>
+            <c:v>Temprture </c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst>
+              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                <a:srgbClr val="000000">
+                  <a:alpha val="63000"/>
+                </a:srgbClr>
+              </a:outerShdw>
+            </a:effectLst>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>[0]!Time</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>[0]!Temp</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000004-71AD-41FA-AA0E-8879577C3941}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
         <c:dLbls>
           <c:showLegendKey val="0"/>
           <c:showVal val="0"/>
@@ -520,144 +750,6 @@
         <c:axId val="538753616"/>
         <c:extLst>
           <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-            <c15:filteredScatterSeries>
-              <c15:ser>
-                <c:idx val="4"/>
-                <c:order val="1"/>
-                <c:tx>
-                  <c:v>Temprture </c:v>
-                </c:tx>
-                <c:spPr>
-                  <a:ln w="9525" cap="rnd">
-                    <a:solidFill>
-                      <a:schemeClr val="accent5"/>
-                    </a:solidFill>
-                    <a:round/>
-                  </a:ln>
-                  <a:effectLst>
-                    <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-                      <a:srgbClr val="000000">
-                        <a:alpha val="63000"/>
-                      </a:srgbClr>
-                    </a:outerShdw>
-                  </a:effectLst>
-                </c:spPr>
-                <c:marker>
-                  <c:symbol val="none"/>
-                </c:marker>
-                <c:xVal>
-                  <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Time</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:xVal>
-                <c:yVal>
-                  <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Temp</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:yVal>
-                <c:smooth val="0"/>
-                <c:extLst>
-                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                    <c16:uniqueId val="{00000001-71AD-41FA-AA0E-8879577C3941}"/>
-                  </c:ext>
-                </c:extLst>
-              </c15:ser>
-            </c15:filteredScatterSeries>
-            <c15:filteredScatterSeries>
-              <c15:ser>
-                <c:idx val="5"/>
-                <c:order val="2"/>
-                <c:tx>
-                  <c:v>Current</c:v>
-                </c:tx>
-                <c:spPr>
-                  <a:ln w="9525" cap="rnd">
-                    <a:solidFill>
-                      <a:schemeClr val="accent6"/>
-                    </a:solidFill>
-                    <a:round/>
-                  </a:ln>
-                  <a:effectLst>
-                    <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-                      <a:srgbClr val="000000">
-                        <a:alpha val="63000"/>
-                      </a:srgbClr>
-                    </a:outerShdw>
-                  </a:effectLst>
-                </c:spPr>
-                <c:marker>
-                  <c:symbol val="none"/>
-                </c:marker>
-                <c:xVal>
-                  <c:numRef>
-                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Time</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:xVal>
-                <c:yVal>
-                  <c:numRef>
-                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Cur</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:yVal>
-                <c:smooth val="0"/>
-                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                    <c16:uniqueId val="{00000002-71AD-41FA-AA0E-8879577C3941}"/>
-                  </c:ext>
-                </c:extLst>
-              </c15:ser>
-            </c15:filteredScatterSeries>
             <c15:filteredScatterSeries>
               <c15:ser>
                 <c:idx val="0"/>
@@ -685,8 +777,8 @@
                 </c:marker>
                 <c:xVal>
                   <c:numRef>
-                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:formulaRef>
                           <c15:sqref>Data!$A$2:$A$500</c15:sqref>
                         </c15:formulaRef>
@@ -703,8 +795,8 @@
                 </c:xVal>
                 <c:yVal>
                   <c:numRef>
-                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:formulaRef>
                           <c15:sqref>Data!$C$2:$C$500</c15:sqref>
                         </c15:formulaRef>
@@ -720,78 +812,9 @@
                   </c:numRef>
                 </c:yVal>
                 <c:smooth val="0"/>
-                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                <c:extLst>
                   <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                     <c16:uniqueId val="{00000003-71AD-41FA-AA0E-8879577C3941}"/>
-                  </c:ext>
-                </c:extLst>
-              </c15:ser>
-            </c15:filteredScatterSeries>
-            <c15:filteredScatterSeries>
-              <c15:ser>
-                <c:idx val="2"/>
-                <c:order val="4"/>
-                <c:tx>
-                  <c:v>Temprture </c:v>
-                </c:tx>
-                <c:spPr>
-                  <a:ln w="9525" cap="rnd">
-                    <a:solidFill>
-                      <a:schemeClr val="accent3"/>
-                    </a:solidFill>
-                    <a:round/>
-                  </a:ln>
-                  <a:effectLst>
-                    <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-                      <a:srgbClr val="000000">
-                        <a:alpha val="63000"/>
-                      </a:srgbClr>
-                    </a:outerShdw>
-                  </a:effectLst>
-                </c:spPr>
-                <c:marker>
-                  <c:symbol val="none"/>
-                </c:marker>
-                <c:xVal>
-                  <c:numRef>
-                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Time</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:xVal>
-                <c:yVal>
-                  <c:numRef>
-                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Temp</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:yVal>
-                <c:smooth val="0"/>
-                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                    <c16:uniqueId val="{00000004-71AD-41FA-AA0E-8879577C3941}"/>
                   </c:ext>
                 </c:extLst>
               </c15:ser>
@@ -1016,6 +1039,177 @@
             </c:ext>
           </c:extLst>
         </c:ser>
+        <c:ser>
+          <c:idx val="4"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Temprture </c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="9525" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent5"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst>
+              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                <a:srgbClr val="000000">
+                  <a:alpha val="63000"/>
+                </a:srgbClr>
+              </a:outerShdw>
+            </a:effectLst>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>[0]!Time</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>[0]!Temp</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-E102-49FF-BA83-7CFBA68AD1C9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="5"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:v>Current</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="9525" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent6"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst>
+              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                <a:srgbClr val="000000">
+                  <a:alpha val="63000"/>
+                </a:srgbClr>
+              </a:outerShdw>
+            </a:effectLst>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>[0]!Time</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>[0]!Cur</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-E102-49FF-BA83-7CFBA68AD1C9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="4"/>
+          <c:tx>
+            <c:v>Temprture </c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="9525" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst>
+              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                <a:srgbClr val="000000">
+                  <a:alpha val="63000"/>
+                </a:srgbClr>
+              </a:outerShdw>
+            </a:effectLst>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>[0]!Time</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>[0]!Temp</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000004-E102-49FF-BA83-7CFBA68AD1C9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
         <c:dLbls>
           <c:showLegendKey val="0"/>
           <c:showVal val="0"/>
@@ -1028,144 +1222,6 @@
         <c:axId val="538753616"/>
         <c:extLst>
           <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-            <c15:filteredScatterSeries>
-              <c15:ser>
-                <c:idx val="4"/>
-                <c:order val="1"/>
-                <c:tx>
-                  <c:v>Temprture </c:v>
-                </c:tx>
-                <c:spPr>
-                  <a:ln w="9525" cap="rnd">
-                    <a:solidFill>
-                      <a:schemeClr val="accent5"/>
-                    </a:solidFill>
-                    <a:round/>
-                  </a:ln>
-                  <a:effectLst>
-                    <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-                      <a:srgbClr val="000000">
-                        <a:alpha val="63000"/>
-                      </a:srgbClr>
-                    </a:outerShdw>
-                  </a:effectLst>
-                </c:spPr>
-                <c:marker>
-                  <c:symbol val="none"/>
-                </c:marker>
-                <c:xVal>
-                  <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Time</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:xVal>
-                <c:yVal>
-                  <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Temp</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:yVal>
-                <c:smooth val="0"/>
-                <c:extLst>
-                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                    <c16:uniqueId val="{00000001-E102-49FF-BA83-7CFBA68AD1C9}"/>
-                  </c:ext>
-                </c:extLst>
-              </c15:ser>
-            </c15:filteredScatterSeries>
-            <c15:filteredScatterSeries>
-              <c15:ser>
-                <c:idx val="5"/>
-                <c:order val="2"/>
-                <c:tx>
-                  <c:v>Current</c:v>
-                </c:tx>
-                <c:spPr>
-                  <a:ln w="9525" cap="rnd">
-                    <a:solidFill>
-                      <a:schemeClr val="accent6"/>
-                    </a:solidFill>
-                    <a:round/>
-                  </a:ln>
-                  <a:effectLst>
-                    <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-                      <a:srgbClr val="000000">
-                        <a:alpha val="63000"/>
-                      </a:srgbClr>
-                    </a:outerShdw>
-                  </a:effectLst>
-                </c:spPr>
-                <c:marker>
-                  <c:symbol val="none"/>
-                </c:marker>
-                <c:xVal>
-                  <c:numRef>
-                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Time</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:xVal>
-                <c:yVal>
-                  <c:numRef>
-                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Cur</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:yVal>
-                <c:smooth val="0"/>
-                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                    <c16:uniqueId val="{00000002-E102-49FF-BA83-7CFBA68AD1C9}"/>
-                  </c:ext>
-                </c:extLst>
-              </c15:ser>
-            </c15:filteredScatterSeries>
             <c15:filteredScatterSeries>
               <c15:ser>
                 <c:idx val="0"/>
@@ -1193,8 +1249,8 @@
                 </c:marker>
                 <c:xVal>
                   <c:numRef>
-                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:formulaRef>
                           <c15:sqref>Data!$A$2:$A$500</c15:sqref>
                         </c15:formulaRef>
@@ -1211,8 +1267,8 @@
                 </c:xVal>
                 <c:yVal>
                   <c:numRef>
-                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:formulaRef>
                           <c15:sqref>Data!$C$2:$C$500</c15:sqref>
                         </c15:formulaRef>
@@ -1228,78 +1284,9 @@
                   </c:numRef>
                 </c:yVal>
                 <c:smooth val="0"/>
-                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                <c:extLst>
                   <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                     <c16:uniqueId val="{00000003-E102-49FF-BA83-7CFBA68AD1C9}"/>
-                  </c:ext>
-                </c:extLst>
-              </c15:ser>
-            </c15:filteredScatterSeries>
-            <c15:filteredScatterSeries>
-              <c15:ser>
-                <c:idx val="2"/>
-                <c:order val="4"/>
-                <c:tx>
-                  <c:v>Temprture </c:v>
-                </c:tx>
-                <c:spPr>
-                  <a:ln w="9525" cap="rnd">
-                    <a:solidFill>
-                      <a:schemeClr val="accent3"/>
-                    </a:solidFill>
-                    <a:round/>
-                  </a:ln>
-                  <a:effectLst>
-                    <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-                      <a:srgbClr val="000000">
-                        <a:alpha val="63000"/>
-                      </a:srgbClr>
-                    </a:outerShdw>
-                  </a:effectLst>
-                </c:spPr>
-                <c:marker>
-                  <c:symbol val="none"/>
-                </c:marker>
-                <c:xVal>
-                  <c:numRef>
-                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Time</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:xVal>
-                <c:yVal>
-                  <c:numRef>
-                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Temp</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:yVal>
-                <c:smooth val="0"/>
-                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                    <c16:uniqueId val="{00000004-E102-49FF-BA83-7CFBA68AD1C9}"/>
                   </c:ext>
                 </c:extLst>
               </c15:ser>
@@ -1525,6 +1512,57 @@
         <c:scatterStyle val="lineMarker"/>
         <c:varyColors val="0"/>
         <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Voltage [V]</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent6"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>[0]!Time</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>[0]!Voltage</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-D4ED-46DC-869B-EE0C9C2EF0E9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
           <c:idx val="2"/>
           <c:order val="2"/>
           <c:tx>
@@ -1583,77 +1621,62 @@
         </c:dLbls>
         <c:axId val="538752176"/>
         <c:axId val="538753616"/>
-        <c:extLst>
-          <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-            <c15:filteredScatterSeries>
-              <c15:ser>
-                <c:idx val="0"/>
-                <c:order val="0"/>
-                <c:tx>
-                  <c:v>Voltage [V]</c:v>
-                </c:tx>
-                <c:spPr>
-                  <a:ln w="28575" cap="rnd">
-                    <a:solidFill>
-                      <a:schemeClr val="accent6"/>
-                    </a:solidFill>
-                    <a:round/>
-                  </a:ln>
-                  <a:effectLst/>
-                </c:spPr>
-                <c:marker>
-                  <c:symbol val="none"/>
-                </c:marker>
-                <c:xVal>
-                  <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Time</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:xVal>
-                <c:yVal>
-                  <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Voltage</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:yVal>
-                <c:smooth val="0"/>
-                <c:extLst>
-                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                    <c16:uniqueId val="{00000001-D4ED-46DC-869B-EE0C9C2EF0E9}"/>
-                  </c:ext>
-                </c:extLst>
-              </c15:ser>
-            </c15:filteredScatterSeries>
-          </c:ext>
-        </c:extLst>
+        <c:extLst/>
       </c:scatterChart>
       <c:scatterChart>
         <c:scatterStyle val="lineMarker"/>
         <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Current [mA]</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent5"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>[0]!Time</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>[0]!Cur</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-D4ED-46DC-869B-EE0C9C2EF0E9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
         <c:dLbls>
           <c:showLegendKey val="0"/>
           <c:showVal val="0"/>
@@ -1664,73 +1687,7 @@
         </c:dLbls>
         <c:axId val="548909984"/>
         <c:axId val="572448592"/>
-        <c:extLst>
-          <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-            <c15:filteredScatterSeries>
-              <c15:ser>
-                <c:idx val="1"/>
-                <c:order val="1"/>
-                <c:tx>
-                  <c:v>Current [mA]</c:v>
-                </c:tx>
-                <c:spPr>
-                  <a:ln w="28575" cap="rnd">
-                    <a:solidFill>
-                      <a:schemeClr val="accent5"/>
-                    </a:solidFill>
-                    <a:round/>
-                  </a:ln>
-                  <a:effectLst/>
-                </c:spPr>
-                <c:marker>
-                  <c:symbol val="none"/>
-                </c:marker>
-                <c:xVal>
-                  <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Time</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:xVal>
-                <c:yVal>
-                  <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Cur</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:yVal>
-                <c:smooth val="0"/>
-                <c:extLst>
-                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                    <c16:uniqueId val="{00000002-D4ED-46DC-869B-EE0C9C2EF0E9}"/>
-                  </c:ext>
-                </c:extLst>
-              </c15:ser>
-            </c15:filteredScatterSeries>
-          </c:ext>
-        </c:extLst>
+        <c:extLst/>
       </c:scatterChart>
       <c:valAx>
         <c:axId val="538752176"/>
@@ -1903,6 +1860,57 @@
         <c:scatterStyle val="lineMarker"/>
         <c:varyColors val="0"/>
         <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Voltage [V]</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent6"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>[0]!Time</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>[0]!Voltage</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-A053-4995-9DEF-DDF35208D668}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
           <c:idx val="2"/>
           <c:order val="2"/>
           <c:tx>
@@ -1961,77 +1969,62 @@
         </c:dLbls>
         <c:axId val="538752176"/>
         <c:axId val="538753616"/>
-        <c:extLst>
-          <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-            <c15:filteredScatterSeries>
-              <c15:ser>
-                <c:idx val="0"/>
-                <c:order val="0"/>
-                <c:tx>
-                  <c:v>Voltage [V]</c:v>
-                </c:tx>
-                <c:spPr>
-                  <a:ln w="28575" cap="rnd">
-                    <a:solidFill>
-                      <a:schemeClr val="accent6"/>
-                    </a:solidFill>
-                    <a:round/>
-                  </a:ln>
-                  <a:effectLst/>
-                </c:spPr>
-                <c:marker>
-                  <c:symbol val="none"/>
-                </c:marker>
-                <c:xVal>
-                  <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Time</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:xVal>
-                <c:yVal>
-                  <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Voltage</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:yVal>
-                <c:smooth val="0"/>
-                <c:extLst>
-                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                    <c16:uniqueId val="{00000001-A053-4995-9DEF-DDF35208D668}"/>
-                  </c:ext>
-                </c:extLst>
-              </c15:ser>
-            </c15:filteredScatterSeries>
-          </c:ext>
-        </c:extLst>
+        <c:extLst/>
       </c:scatterChart>
       <c:scatterChart>
         <c:scatterStyle val="lineMarker"/>
         <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Current [mA]</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent5"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>[0]!Time</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>[0]!Cur</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-A053-4995-9DEF-DDF35208D668}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
         <c:dLbls>
           <c:showLegendKey val="0"/>
           <c:showVal val="0"/>
@@ -2042,73 +2035,7 @@
         </c:dLbls>
         <c:axId val="548909984"/>
         <c:axId val="572448592"/>
-        <c:extLst>
-          <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-            <c15:filteredScatterSeries>
-              <c15:ser>
-                <c:idx val="1"/>
-                <c:order val="1"/>
-                <c:tx>
-                  <c:v>Current [mA]</c:v>
-                </c:tx>
-                <c:spPr>
-                  <a:ln w="28575" cap="rnd">
-                    <a:solidFill>
-                      <a:schemeClr val="accent5"/>
-                    </a:solidFill>
-                    <a:round/>
-                  </a:ln>
-                  <a:effectLst/>
-                </c:spPr>
-                <c:marker>
-                  <c:symbol val="none"/>
-                </c:marker>
-                <c:xVal>
-                  <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Time</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:xVal>
-                <c:yVal>
-                  <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Cur</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:yVal>
-                <c:smooth val="0"/>
-                <c:extLst>
-                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                    <c16:uniqueId val="{00000002-A053-4995-9DEF-DDF35208D668}"/>
-                  </c:ext>
-                </c:extLst>
-              </c15:ser>
-            </c15:filteredScatterSeries>
-          </c:ext>
-        </c:extLst>
+        <c:extLst/>
       </c:scatterChart>
       <c:valAx>
         <c:axId val="538752176"/>
@@ -2463,6 +2390,108 @@
             </c:ext>
           </c:extLst>
         </c:ser>
+        <c:ser>
+          <c:idx val="4"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Temprture </c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="15875" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent5"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>[0]!Time</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>[0]!Temp</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-D1EA-4A58-A582-9D1E456A899B}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="4"/>
+          <c:tx>
+            <c:v>Temprture </c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="15875" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>[0]!Time</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>[0]!Temp</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000004-D1EA-4A58-A582-9D1E456A899B}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
         <c:dLbls>
           <c:showLegendKey val="0"/>
           <c:showVal val="0"/>
@@ -2475,69 +2504,6 @@
         <c:axId val="538753616"/>
         <c:extLst>
           <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-            <c15:filteredScatterSeries>
-              <c15:ser>
-                <c:idx val="4"/>
-                <c:order val="1"/>
-                <c:tx>
-                  <c:v>Temprture </c:v>
-                </c:tx>
-                <c:spPr>
-                  <a:ln w="15875" cap="rnd">
-                    <a:solidFill>
-                      <a:schemeClr val="accent5"/>
-                    </a:solidFill>
-                    <a:round/>
-                  </a:ln>
-                  <a:effectLst/>
-                </c:spPr>
-                <c:marker>
-                  <c:symbol val="none"/>
-                </c:marker>
-                <c:xVal>
-                  <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Time</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:xVal>
-                <c:yVal>
-                  <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Temp</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:yVal>
-                <c:smooth val="0"/>
-                <c:extLst>
-                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                    <c16:uniqueId val="{00000001-D1EA-4A58-A582-9D1E456A899B}"/>
-                  </c:ext>
-                </c:extLst>
-              </c15:ser>
-            </c15:filteredScatterSeries>
             <c15:filteredScatterSeries>
               <c15:ser>
                 <c:idx val="0"/>
@@ -2559,8 +2525,8 @@
                 </c:marker>
                 <c:xVal>
                   <c:numRef>
-                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:formulaRef>
                           <c15:sqref>Data!$A$2:$A$500</c15:sqref>
                         </c15:formulaRef>
@@ -2577,8 +2543,8 @@
                 </c:xVal>
                 <c:yVal>
                   <c:numRef>
-                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:formulaRef>
                           <c15:sqref>Data!$C$2:$C$500</c15:sqref>
                         </c15:formulaRef>
@@ -2594,72 +2560,9 @@
                   </c:numRef>
                 </c:yVal>
                 <c:smooth val="0"/>
-                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                <c:extLst>
                   <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                     <c16:uniqueId val="{00000003-D1EA-4A58-A582-9D1E456A899B}"/>
-                  </c:ext>
-                </c:extLst>
-              </c15:ser>
-            </c15:filteredScatterSeries>
-            <c15:filteredScatterSeries>
-              <c15:ser>
-                <c:idx val="2"/>
-                <c:order val="4"/>
-                <c:tx>
-                  <c:v>Temprture </c:v>
-                </c:tx>
-                <c:spPr>
-                  <a:ln w="15875" cap="rnd">
-                    <a:solidFill>
-                      <a:schemeClr val="accent3"/>
-                    </a:solidFill>
-                    <a:round/>
-                  </a:ln>
-                  <a:effectLst/>
-                </c:spPr>
-                <c:marker>
-                  <c:symbol val="none"/>
-                </c:marker>
-                <c:xVal>
-                  <c:numRef>
-                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Time</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:xVal>
-                <c:yVal>
-                  <c:numRef>
-                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>[0]!Temp</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:yVal>
-                <c:smooth val="0"/>
-                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                    <c16:uniqueId val="{00000004-D1EA-4A58-A582-9D1E456A899B}"/>
                   </c:ext>
                 </c:extLst>
               </c15:ser>
@@ -5950,8 +5853,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="620888" y="390232"/>
-          <a:ext cx="9275793" cy="4271548"/>
+          <a:off x="620888" y="374515"/>
+          <a:ext cx="9323827" cy="4158201"/>
           <a:chOff x="621310" y="383428"/>
           <a:chExt cx="9321752" cy="4231579"/>
         </a:xfrm>
@@ -7343,7 +7246,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BE78AA8-3E87-47A3-991D-56AC1DEC39E3}">
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:S19"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.88671875" style="1" customWidth="1"/>
@@ -7352,10 +7255,18 @@
     <col min="5" max="5" width="22.5546875" style="1" customWidth="1"/>
     <col min="6" max="6" width="13.109375" style="1" customWidth="1"/>
     <col min="7" max="7" width="13.33203125" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="9.109375" style="1"/>
+    <col min="8" max="9" width="9.109375" style="1"/>
+    <col min="10" max="10" width="12.88671875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="15.88671875" style="1" customWidth="1"/>
+    <col min="12" max="12" width="13.6640625" style="1" customWidth="1"/>
+    <col min="13" max="13" width="14.6640625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="21" style="1" customWidth="1"/>
+    <col min="15" max="16" width="9.109375" style="1"/>
+    <col min="17" max="17" width="24.44140625" style="1" customWidth="1"/>
+    <col min="18" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A1" s="24" t="s">
         <v>24</v>
       </c>
@@ -7377,8 +7288,23 @@
       <c r="G1" s="24" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="J1" s="24" t="s">
+        <v>32</v>
+      </c>
+      <c r="K1" s="27" t="s">
+        <v>24</v>
+      </c>
+      <c r="L1" s="26" t="s">
+        <v>23</v>
+      </c>
+      <c r="M1" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="N1" s="26" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>0</v>
       </c>
@@ -7400,6 +7326,10 @@
       <c r="G2" s="1">
         <v>0</v>
       </c>
+      <c r="S2" s="1" t="e" cm="1">
+        <f t="array" ref="S2">INDEX(A2:A100000,_xlfn.SEQUENCE(ROUNDUP(COUNTA(A2:A100000)/I1,0),1,1,I1))</f>
+        <v>#DIV/0!</v>
+      </c>
     </row>
     <row r="19" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K19" s="2"/>

</xml_diff>

<commit_message>
bug 16: xlsx chart
</commit_message>
<xml_diff>
--- a/web-console/server/assets/excel_template.xlsx
+++ b/web-console/server/assets/excel_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\DEV\UBA6\web-console\server\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97BA26B2-DCF2-4EC1-B818-EBEA7FF1D235}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93D08DA2-7AC9-470B-A1E0-87F197B9FB35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{3E3B58E4-0181-4207-8002-E1D914CEBC2E}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3E3B58E4-0181-4207-8002-E1D914CEBC2E}"/>
   </bookViews>
   <sheets>
     <sheet name="Report" sheetId="1" r:id="rId1"/>
@@ -41,30 +41,8 @@
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="32">
   <si>
     <t>Wh</t>
   </si>
@@ -184,15 +162,12 @@
   <si>
     <t>Parallel</t>
   </si>
-  <si>
-    <t>Sample Rate</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -246,16 +221,8 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -268,14 +235,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor theme="4"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="12">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -370,37 +331,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
-      </top>
-      <bottom style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
-      </top>
-      <bottom style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
@@ -441,8 +378,6 @@
     <xf numFmtId="49" fontId="3" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="11" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -472,8 +407,8 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFCC0000"/>
       <color rgb="FF000000"/>
-      <color rgb="FFCC0000"/>
       <color rgb="FF009999"/>
       <color rgb="FF0066FF"/>
       <color rgb="FF009900"/>
@@ -573,171 +508,6 @@
             </c:ext>
           </c:extLst>
         </c:ser>
-        <c:ser>
-          <c:idx val="4"/>
-          <c:order val="1"/>
-          <c:tx>
-            <c:v>Temprture </c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="25400" cap="rnd">
-              <a:noFill/>
-              <a:round/>
-            </a:ln>
-            <a:effectLst>
-              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-                <a:srgbClr val="000000">
-                  <a:alpha val="63000"/>
-                </a:srgbClr>
-              </a:outerShdw>
-            </a:effectLst>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>[0]!Time</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>[0]!Temp</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-71AD-41FA-AA0E-8879577C3941}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="5"/>
-          <c:order val="2"/>
-          <c:tx>
-            <c:v>Current</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="25400" cap="rnd">
-              <a:noFill/>
-              <a:round/>
-            </a:ln>
-            <a:effectLst>
-              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-                <a:srgbClr val="000000">
-                  <a:alpha val="63000"/>
-                </a:srgbClr>
-              </a:outerShdw>
-            </a:effectLst>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>[0]!Time</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>[0]!Cur</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-71AD-41FA-AA0E-8879577C3941}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="2"/>
-          <c:order val="4"/>
-          <c:tx>
-            <c:v>Temprture </c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="25400" cap="rnd">
-              <a:noFill/>
-              <a:round/>
-            </a:ln>
-            <a:effectLst>
-              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-                <a:srgbClr val="000000">
-                  <a:alpha val="63000"/>
-                </a:srgbClr>
-              </a:outerShdw>
-            </a:effectLst>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>[0]!Time</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>[0]!Temp</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-71AD-41FA-AA0E-8879577C3941}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
         <c:dLbls>
           <c:showLegendKey val="0"/>
           <c:showVal val="0"/>
@@ -750,6 +520,144 @@
         <c:axId val="538753616"/>
         <c:extLst>
           <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+            <c15:filteredScatterSeries>
+              <c15:ser>
+                <c:idx val="4"/>
+                <c:order val="1"/>
+                <c:tx>
+                  <c:v>Temprture </c:v>
+                </c:tx>
+                <c:spPr>
+                  <a:ln w="9525" cap="rnd">
+                    <a:solidFill>
+                      <a:schemeClr val="accent5"/>
+                    </a:solidFill>
+                    <a:round/>
+                  </a:ln>
+                  <a:effectLst>
+                    <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                      <a:srgbClr val="000000">
+                        <a:alpha val="63000"/>
+                      </a:srgbClr>
+                    </a:outerShdw>
+                  </a:effectLst>
+                </c:spPr>
+                <c:marker>
+                  <c:symbol val="none"/>
+                </c:marker>
+                <c:xVal>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Time</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:xVal>
+                <c:yVal>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Temp</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:yVal>
+                <c:smooth val="0"/>
+                <c:extLst>
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000001-71AD-41FA-AA0E-8879577C3941}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredScatterSeries>
+            <c15:filteredScatterSeries>
+              <c15:ser>
+                <c:idx val="5"/>
+                <c:order val="2"/>
+                <c:tx>
+                  <c:v>Current</c:v>
+                </c:tx>
+                <c:spPr>
+                  <a:ln w="9525" cap="rnd">
+                    <a:solidFill>
+                      <a:schemeClr val="accent6"/>
+                    </a:solidFill>
+                    <a:round/>
+                  </a:ln>
+                  <a:effectLst>
+                    <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                      <a:srgbClr val="000000">
+                        <a:alpha val="63000"/>
+                      </a:srgbClr>
+                    </a:outerShdw>
+                  </a:effectLst>
+                </c:spPr>
+                <c:marker>
+                  <c:symbol val="none"/>
+                </c:marker>
+                <c:xVal>
+                  <c:numRef>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Time</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:xVal>
+                <c:yVal>
+                  <c:numRef>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Cur</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:yVal>
+                <c:smooth val="0"/>
+                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000002-71AD-41FA-AA0E-8879577C3941}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredScatterSeries>
             <c15:filteredScatterSeries>
               <c15:ser>
                 <c:idx val="0"/>
@@ -777,8 +685,8 @@
                 </c:marker>
                 <c:xVal>
                   <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:formulaRef>
                           <c15:sqref>Data!$A$2:$A$500</c15:sqref>
                         </c15:formulaRef>
@@ -795,8 +703,8 @@
                 </c:xVal>
                 <c:yVal>
                   <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:formulaRef>
                           <c15:sqref>Data!$C$2:$C$500</c15:sqref>
                         </c15:formulaRef>
@@ -812,9 +720,78 @@
                   </c:numRef>
                 </c:yVal>
                 <c:smooth val="0"/>
-                <c:extLst>
+                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
                   <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                     <c16:uniqueId val="{00000003-71AD-41FA-AA0E-8879577C3941}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredScatterSeries>
+            <c15:filteredScatterSeries>
+              <c15:ser>
+                <c:idx val="2"/>
+                <c:order val="4"/>
+                <c:tx>
+                  <c:v>Temprture </c:v>
+                </c:tx>
+                <c:spPr>
+                  <a:ln w="9525" cap="rnd">
+                    <a:solidFill>
+                      <a:schemeClr val="accent3"/>
+                    </a:solidFill>
+                    <a:round/>
+                  </a:ln>
+                  <a:effectLst>
+                    <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                      <a:srgbClr val="000000">
+                        <a:alpha val="63000"/>
+                      </a:srgbClr>
+                    </a:outerShdw>
+                  </a:effectLst>
+                </c:spPr>
+                <c:marker>
+                  <c:symbol val="none"/>
+                </c:marker>
+                <c:xVal>
+                  <c:numRef>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Time</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:xVal>
+                <c:yVal>
+                  <c:numRef>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Temp</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:yVal>
+                <c:smooth val="0"/>
+                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000004-71AD-41FA-AA0E-8879577C3941}"/>
                   </c:ext>
                 </c:extLst>
               </c15:ser>
@@ -1039,177 +1016,6 @@
             </c:ext>
           </c:extLst>
         </c:ser>
-        <c:ser>
-          <c:idx val="4"/>
-          <c:order val="1"/>
-          <c:tx>
-            <c:v>Temprture </c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="9525" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent5"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst>
-              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-                <a:srgbClr val="000000">
-                  <a:alpha val="63000"/>
-                </a:srgbClr>
-              </a:outerShdw>
-            </a:effectLst>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>[0]!Time</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>[0]!Temp</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-E102-49FF-BA83-7CFBA68AD1C9}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="5"/>
-          <c:order val="2"/>
-          <c:tx>
-            <c:v>Current</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="9525" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent6"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst>
-              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-                <a:srgbClr val="000000">
-                  <a:alpha val="63000"/>
-                </a:srgbClr>
-              </a:outerShdw>
-            </a:effectLst>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>[0]!Time</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>[0]!Cur</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-E102-49FF-BA83-7CFBA68AD1C9}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="2"/>
-          <c:order val="4"/>
-          <c:tx>
-            <c:v>Temprture </c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="9525" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent3"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst>
-              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-                <a:srgbClr val="000000">
-                  <a:alpha val="63000"/>
-                </a:srgbClr>
-              </a:outerShdw>
-            </a:effectLst>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>[0]!Time</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>[0]!Temp</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-E102-49FF-BA83-7CFBA68AD1C9}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
         <c:dLbls>
           <c:showLegendKey val="0"/>
           <c:showVal val="0"/>
@@ -1222,6 +1028,144 @@
         <c:axId val="538753616"/>
         <c:extLst>
           <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+            <c15:filteredScatterSeries>
+              <c15:ser>
+                <c:idx val="4"/>
+                <c:order val="1"/>
+                <c:tx>
+                  <c:v>Temprture </c:v>
+                </c:tx>
+                <c:spPr>
+                  <a:ln w="9525" cap="rnd">
+                    <a:solidFill>
+                      <a:schemeClr val="accent5"/>
+                    </a:solidFill>
+                    <a:round/>
+                  </a:ln>
+                  <a:effectLst>
+                    <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                      <a:srgbClr val="000000">
+                        <a:alpha val="63000"/>
+                      </a:srgbClr>
+                    </a:outerShdw>
+                  </a:effectLst>
+                </c:spPr>
+                <c:marker>
+                  <c:symbol val="none"/>
+                </c:marker>
+                <c:xVal>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Time</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:xVal>
+                <c:yVal>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Temp</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:yVal>
+                <c:smooth val="0"/>
+                <c:extLst>
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000001-E102-49FF-BA83-7CFBA68AD1C9}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredScatterSeries>
+            <c15:filteredScatterSeries>
+              <c15:ser>
+                <c:idx val="5"/>
+                <c:order val="2"/>
+                <c:tx>
+                  <c:v>Current</c:v>
+                </c:tx>
+                <c:spPr>
+                  <a:ln w="9525" cap="rnd">
+                    <a:solidFill>
+                      <a:schemeClr val="accent6"/>
+                    </a:solidFill>
+                    <a:round/>
+                  </a:ln>
+                  <a:effectLst>
+                    <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                      <a:srgbClr val="000000">
+                        <a:alpha val="63000"/>
+                      </a:srgbClr>
+                    </a:outerShdw>
+                  </a:effectLst>
+                </c:spPr>
+                <c:marker>
+                  <c:symbol val="none"/>
+                </c:marker>
+                <c:xVal>
+                  <c:numRef>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Time</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:xVal>
+                <c:yVal>
+                  <c:numRef>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Cur</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:yVal>
+                <c:smooth val="0"/>
+                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000002-E102-49FF-BA83-7CFBA68AD1C9}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredScatterSeries>
             <c15:filteredScatterSeries>
               <c15:ser>
                 <c:idx val="0"/>
@@ -1249,8 +1193,8 @@
                 </c:marker>
                 <c:xVal>
                   <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:formulaRef>
                           <c15:sqref>Data!$A$2:$A$500</c15:sqref>
                         </c15:formulaRef>
@@ -1267,8 +1211,8 @@
                 </c:xVal>
                 <c:yVal>
                   <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:formulaRef>
                           <c15:sqref>Data!$C$2:$C$500</c15:sqref>
                         </c15:formulaRef>
@@ -1284,9 +1228,78 @@
                   </c:numRef>
                 </c:yVal>
                 <c:smooth val="0"/>
-                <c:extLst>
+                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
                   <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                     <c16:uniqueId val="{00000003-E102-49FF-BA83-7CFBA68AD1C9}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredScatterSeries>
+            <c15:filteredScatterSeries>
+              <c15:ser>
+                <c:idx val="2"/>
+                <c:order val="4"/>
+                <c:tx>
+                  <c:v>Temprture </c:v>
+                </c:tx>
+                <c:spPr>
+                  <a:ln w="9525" cap="rnd">
+                    <a:solidFill>
+                      <a:schemeClr val="accent3"/>
+                    </a:solidFill>
+                    <a:round/>
+                  </a:ln>
+                  <a:effectLst>
+                    <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                      <a:srgbClr val="000000">
+                        <a:alpha val="63000"/>
+                      </a:srgbClr>
+                    </a:outerShdw>
+                  </a:effectLst>
+                </c:spPr>
+                <c:marker>
+                  <c:symbol val="none"/>
+                </c:marker>
+                <c:xVal>
+                  <c:numRef>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Time</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:xVal>
+                <c:yVal>
+                  <c:numRef>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Temp</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:yVal>
+                <c:smooth val="0"/>
+                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000004-E102-49FF-BA83-7CFBA68AD1C9}"/>
                   </c:ext>
                 </c:extLst>
               </c15:ser>
@@ -1512,57 +1525,6 @@
         <c:scatterStyle val="lineMarker"/>
         <c:varyColors val="0"/>
         <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:tx>
-            <c:v>Voltage [V]</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent6"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>[0]!Time</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>[0]!Voltage</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-D4ED-46DC-869B-EE0C9C2EF0E9}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
           <c:idx val="2"/>
           <c:order val="2"/>
           <c:tx>
@@ -1582,25 +1544,19 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Data!$A$2:$A$50000</c:f>
+              <c:f>Data!$K$2:$K$50000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="49999"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Data!$E$2:$E$50000</c:f>
+              <c:f>Data!$N$2:$N$50000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="49999"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -1621,62 +1577,77 @@
         </c:dLbls>
         <c:axId val="538752176"/>
         <c:axId val="538753616"/>
-        <c:extLst/>
+        <c:extLst>
+          <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+            <c15:filteredScatterSeries>
+              <c15:ser>
+                <c:idx val="0"/>
+                <c:order val="0"/>
+                <c:tx>
+                  <c:v>Voltage [V]</c:v>
+                </c:tx>
+                <c:spPr>
+                  <a:ln w="28575" cap="rnd">
+                    <a:solidFill>
+                      <a:schemeClr val="accent6"/>
+                    </a:solidFill>
+                    <a:round/>
+                  </a:ln>
+                  <a:effectLst/>
+                </c:spPr>
+                <c:marker>
+                  <c:symbol val="none"/>
+                </c:marker>
+                <c:xVal>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Time</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:xVal>
+                <c:yVal>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Voltage</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:yVal>
+                <c:smooth val="0"/>
+                <c:extLst>
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000001-D4ED-46DC-869B-EE0C9C2EF0E9}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredScatterSeries>
+          </c:ext>
+        </c:extLst>
       </c:scatterChart>
       <c:scatterChart>
         <c:scatterStyle val="lineMarker"/>
         <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
-          <c:tx>
-            <c:v>Current [mA]</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent5"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>[0]!Time</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>[0]!Cur</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-D4ED-46DC-869B-EE0C9C2EF0E9}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
         <c:dLbls>
           <c:showLegendKey val="0"/>
           <c:showVal val="0"/>
@@ -1687,7 +1658,73 @@
         </c:dLbls>
         <c:axId val="548909984"/>
         <c:axId val="572448592"/>
-        <c:extLst/>
+        <c:extLst>
+          <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+            <c15:filteredScatterSeries>
+              <c15:ser>
+                <c:idx val="1"/>
+                <c:order val="1"/>
+                <c:tx>
+                  <c:v>Current [mA]</c:v>
+                </c:tx>
+                <c:spPr>
+                  <a:ln w="28575" cap="rnd">
+                    <a:solidFill>
+                      <a:schemeClr val="accent5"/>
+                    </a:solidFill>
+                    <a:round/>
+                  </a:ln>
+                  <a:effectLst/>
+                </c:spPr>
+                <c:marker>
+                  <c:symbol val="none"/>
+                </c:marker>
+                <c:xVal>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Time</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:xVal>
+                <c:yVal>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Cur</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:yVal>
+                <c:smooth val="0"/>
+                <c:extLst>
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000002-D4ED-46DC-869B-EE0C9C2EF0E9}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredScatterSeries>
+          </c:ext>
+        </c:extLst>
       </c:scatterChart>
       <c:valAx>
         <c:axId val="538752176"/>
@@ -1860,57 +1897,6 @@
         <c:scatterStyle val="lineMarker"/>
         <c:varyColors val="0"/>
         <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:tx>
-            <c:v>Voltage [V]</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent6"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>[0]!Time</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>[0]!Voltage</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-A053-4995-9DEF-DDF35208D668}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
           <c:idx val="2"/>
           <c:order val="2"/>
           <c:tx>
@@ -1969,62 +1955,77 @@
         </c:dLbls>
         <c:axId val="538752176"/>
         <c:axId val="538753616"/>
-        <c:extLst/>
+        <c:extLst>
+          <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+            <c15:filteredScatterSeries>
+              <c15:ser>
+                <c:idx val="0"/>
+                <c:order val="0"/>
+                <c:tx>
+                  <c:v>Voltage [V]</c:v>
+                </c:tx>
+                <c:spPr>
+                  <a:ln w="28575" cap="rnd">
+                    <a:solidFill>
+                      <a:schemeClr val="accent6"/>
+                    </a:solidFill>
+                    <a:round/>
+                  </a:ln>
+                  <a:effectLst/>
+                </c:spPr>
+                <c:marker>
+                  <c:symbol val="none"/>
+                </c:marker>
+                <c:xVal>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Time</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:xVal>
+                <c:yVal>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Voltage</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:yVal>
+                <c:smooth val="0"/>
+                <c:extLst>
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000001-A053-4995-9DEF-DDF35208D668}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredScatterSeries>
+          </c:ext>
+        </c:extLst>
       </c:scatterChart>
       <c:scatterChart>
         <c:scatterStyle val="lineMarker"/>
         <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
-          <c:tx>
-            <c:v>Current [mA]</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent5"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>[0]!Time</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>[0]!Cur</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-A053-4995-9DEF-DDF35208D668}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
         <c:dLbls>
           <c:showLegendKey val="0"/>
           <c:showVal val="0"/>
@@ -2035,7 +2036,73 @@
         </c:dLbls>
         <c:axId val="548909984"/>
         <c:axId val="572448592"/>
-        <c:extLst/>
+        <c:extLst>
+          <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+            <c15:filteredScatterSeries>
+              <c15:ser>
+                <c:idx val="1"/>
+                <c:order val="1"/>
+                <c:tx>
+                  <c:v>Current [mA]</c:v>
+                </c:tx>
+                <c:spPr>
+                  <a:ln w="28575" cap="rnd">
+                    <a:solidFill>
+                      <a:schemeClr val="accent5"/>
+                    </a:solidFill>
+                    <a:round/>
+                  </a:ln>
+                  <a:effectLst/>
+                </c:spPr>
+                <c:marker>
+                  <c:symbol val="none"/>
+                </c:marker>
+                <c:xVal>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Time</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:xVal>
+                <c:yVal>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Cur</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:yVal>
+                <c:smooth val="0"/>
+                <c:extLst>
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000002-A053-4995-9DEF-DDF35208D668}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredScatterSeries>
+          </c:ext>
+        </c:extLst>
       </c:scatterChart>
       <c:valAx>
         <c:axId val="538752176"/>
@@ -2350,7 +2417,7 @@
           <c:spPr>
             <a:ln w="12700" cap="rnd">
               <a:solidFill>
-                <a:schemeClr val="tx1"/>
+                <a:schemeClr val="accent6"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -2361,25 +2428,19 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Data!$A$2:$A$50000</c:f>
+              <c:f>Data!$K$2:$K$50000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="49999"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Data!$C$2:$C$50000</c:f>
+              <c:f>Data!$L$2:$L$50000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="49999"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -2387,108 +2448,6 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000000-D1EA-4A58-A582-9D1E456A899B}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="4"/>
-          <c:order val="1"/>
-          <c:tx>
-            <c:v>Temprture </c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="15875" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent5"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>[0]!Time</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>[0]!Temp</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-D1EA-4A58-A582-9D1E456A899B}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="2"/>
-          <c:order val="4"/>
-          <c:tx>
-            <c:v>Temprture </c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="15875" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent3"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>[0]!Time</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>[0]!Temp</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-              <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"/>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-D1EA-4A58-A582-9D1E456A899B}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2506,15 +2465,15 @@
           <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
             <c15:filteredScatterSeries>
               <c15:ser>
-                <c:idx val="0"/>
-                <c:order val="3"/>
+                <c:idx val="4"/>
+                <c:order val="1"/>
                 <c:tx>
-                  <c:v>Voltage [V]</c:v>
+                  <c:v>Temprture </c:v>
                 </c:tx>
                 <c:spPr>
                   <a:ln w="15875" cap="rnd">
                     <a:solidFill>
-                      <a:schemeClr val="accent1"/>
+                      <a:schemeClr val="accent5"/>
                     </a:solidFill>
                     <a:round/>
                   </a:ln>
@@ -2527,6 +2486,69 @@
                   <c:numRef>
                     <c:extLst>
                       <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Time</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:xVal>
+                <c:yVal>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Temp</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:yVal>
+                <c:smooth val="0"/>
+                <c:extLst>
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000001-D1EA-4A58-A582-9D1E456A899B}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredScatterSeries>
+            <c15:filteredScatterSeries>
+              <c15:ser>
+                <c:idx val="0"/>
+                <c:order val="3"/>
+                <c:tx>
+                  <c:v>Voltage [V]</c:v>
+                </c:tx>
+                <c:spPr>
+                  <a:ln w="12700" cap="rnd">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1"/>
+                    </a:solidFill>
+                    <a:round/>
+                  </a:ln>
+                  <a:effectLst/>
+                </c:spPr>
+                <c:marker>
+                  <c:symbol val="none"/>
+                </c:marker>
+                <c:xVal>
+                  <c:numRef>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:formulaRef>
                           <c15:sqref>Data!$A$2:$A$500</c15:sqref>
                         </c15:formulaRef>
@@ -2543,8 +2565,8 @@
                 </c:xVal>
                 <c:yVal>
                   <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:formulaRef>
                           <c15:sqref>Data!$C$2:$C$500</c15:sqref>
                         </c15:formulaRef>
@@ -2560,9 +2582,72 @@
                   </c:numRef>
                 </c:yVal>
                 <c:smooth val="0"/>
-                <c:extLst>
+                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
                   <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                     <c16:uniqueId val="{00000003-D1EA-4A58-A582-9D1E456A899B}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredScatterSeries>
+            <c15:filteredScatterSeries>
+              <c15:ser>
+                <c:idx val="2"/>
+                <c:order val="4"/>
+                <c:tx>
+                  <c:v>Temprture </c:v>
+                </c:tx>
+                <c:spPr>
+                  <a:ln w="15875" cap="rnd">
+                    <a:solidFill>
+                      <a:schemeClr val="accent3"/>
+                    </a:solidFill>
+                    <a:round/>
+                  </a:ln>
+                  <a:effectLst/>
+                </c:spPr>
+                <c:marker>
+                  <c:symbol val="none"/>
+                </c:marker>
+                <c:xVal>
+                  <c:numRef>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Time</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:xVal>
+                <c:yVal>
+                  <c:numRef>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                      <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[0]!Temp</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="1"/>
+                      <c:pt idx="0">
+                        <c:v>0</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:yVal>
+                <c:smooth val="0"/>
+                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000004-D1EA-4A58-A582-9D1E456A899B}"/>
                   </c:ext>
                 </c:extLst>
               </c15:ser>
@@ -2593,25 +2678,19 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Data!$A$2:$A$50000</c:f>
+              <c:f>Data!$K$2:$K$50000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="49999"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Data!$D$2:$D$50000</c:f>
+              <c:f>Data!$M$2:$M$50000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="49999"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -2922,9 +3001,11 @@
   </c:chart>
   <c:spPr>
     <a:solidFill>
-      <a:srgbClr val="000000">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="50000"/>
+        <a:lumOff val="50000"/>
         <a:alpha val="0"/>
-      </a:srgbClr>
+      </a:schemeClr>
     </a:solidFill>
     <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:noFill/>
@@ -5832,13 +5913,13 @@
       <xdr:col>1</xdr:col>
       <xdr:colOff>110620</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>97678</xdr:rowOff>
+      <xdr:rowOff>85364</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>92735</xdr:colOff>
+      <xdr:colOff>96545</xdr:colOff>
       <xdr:row>26</xdr:row>
-      <xdr:rowOff>82976</xdr:rowOff>
+      <xdr:rowOff>76377</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
@@ -5853,8 +5934,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="620888" y="374515"/>
-          <a:ext cx="9323827" cy="4158201"/>
+          <a:off x="620888" y="367916"/>
+          <a:ext cx="9320017" cy="4156296"/>
           <a:chOff x="621310" y="383428"/>
           <a:chExt cx="9321752" cy="4231579"/>
         </a:xfrm>
@@ -7246,7 +7327,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BE78AA8-3E87-47A3-991D-56AC1DEC39E3}">
-  <dimension ref="A1:S19"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.88671875" style="1" customWidth="1"/>
@@ -7255,18 +7336,10 @@
     <col min="5" max="5" width="22.5546875" style="1" customWidth="1"/>
     <col min="6" max="6" width="13.109375" style="1" customWidth="1"/>
     <col min="7" max="7" width="13.33203125" style="1" customWidth="1"/>
-    <col min="8" max="9" width="9.109375" style="1"/>
-    <col min="10" max="10" width="12.88671875" style="1" customWidth="1"/>
-    <col min="11" max="11" width="15.88671875" style="1" customWidth="1"/>
-    <col min="12" max="12" width="13.6640625" style="1" customWidth="1"/>
-    <col min="13" max="13" width="14.6640625" style="1" customWidth="1"/>
-    <col min="14" max="14" width="21" style="1" customWidth="1"/>
-    <col min="15" max="16" width="9.109375" style="1"/>
-    <col min="17" max="17" width="24.44140625" style="1" customWidth="1"/>
-    <col min="18" max="16384" width="9.109375" style="1"/>
+    <col min="8" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="24" t="s">
         <v>24</v>
       </c>
@@ -7288,23 +7361,8 @@
       <c r="G1" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="J1" s="24" t="s">
-        <v>32</v>
-      </c>
-      <c r="K1" s="27" t="s">
-        <v>24</v>
-      </c>
-      <c r="L1" s="26" t="s">
-        <v>23</v>
-      </c>
-      <c r="M1" s="26" t="s">
-        <v>18</v>
-      </c>
-      <c r="N1" s="26" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>0</v>
       </c>
@@ -7326,10 +7384,6 @@
       <c r="G2" s="1">
         <v>0</v>
       </c>
-      <c r="S2" s="1" t="e" cm="1">
-        <f t="array" ref="S2">INDEX(A2:A100000,_xlfn.SEQUENCE(ROUNDUP(COUNTA(A2:A100000)/I1,0),1,1,I1))</f>
-        <v>#DIV/0!</v>
-      </c>
     </row>
     <row r="19" spans="11:11" x14ac:dyDescent="0.3">
       <c r="K19" s="2"/>

</xml_diff>